<commit_message>
Codex v1.4: sync from Anima; requirements v1.5 and backlog synced from Drive
Luna Physics (PHY-01..PHY-06, ARC-10, ADR-017): six layers, deterministic
fixed-point 3D physics, new milestone M1b (US-025..US-029) right after M1.
</commit_message>
<xml_diff>
--- a/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
+++ b/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
@@ -603,6 +603,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -645,6 +646,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
@@ -739,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -763,6 +765,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -777,6 +780,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
@@ -1121,12 +1125,12 @@
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Assumption: pausable real time with speed control (pause, 1x, 2x, 4x). Needs owner confirmation (OPEN-04).</t>
+          <t>Pausable real time with speed control (pause, 1x, 2x, 4x). Decided by the owner (D-01, 2026-09-30).</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
@@ -1135,71 +1139,77 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>MVP-13</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Luna Physics core: deterministic 3D fixed-point math, hit detection, ballistics, basic rigid bodies and material properties, proven by a spear throw in the demo (M1b). Advanced physics and chemistry return with later Ages.</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>PHY-01..PHY-06, ARC-10, ADR-017</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Success and kill criteria (decided before building)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="C24" s="6" t="inlineStr">
         <is>
           <t>How measured</t>
         </is>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D24" s="6" t="inlineStr">
         <is>
           <t>Gate</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>Voluntary play time</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>5 of 8 playtesters play 30+ minutes without being asked to continue</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Observation + local session log (US-092)</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>M6</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Emergent story</t>
+          <t>Voluntary play time</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>3 of 8 can retell a story that came from the simulation, not from a script</t>
+          <t>5 of 8 playtesters play 30+ minutes without being asked to continue</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>Post-play interview</t>
+          <t>Observation + local session log (US-092)</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
@@ -1211,110 +1221,132 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>Chronicle interest (early)</t>
+          <t>Emergent story</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>2 of 3 readers find a story in the console chronicle</t>
+          <t>3 of 8 can retell a story that came from the simulation, not from a script</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Show printed chronicle</t>
+          <t>Post-play interview</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>M6</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Frame rate</t>
+          <t>Chronicle interest (early)</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>60 FPS with 500 simulated agents in the region on the minimum PC (OPEN-19)</t>
+          <t>2 of 3 readers find a story in the console chronicle</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>FPS overlay (US-082)</t>
+          <t>Show printed chronicle</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M2</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Determinism</t>
+          <t>Frame rate</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Same seed + inputs give the same world hash after 10,000 ticks</t>
+          <t>60 FPS with 500 simulated agents in the region on the minimum PC (OPEN-19)</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Automated test in CI</t>
+          <t>FPS overlay (US-082)</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>M1 onwards</t>
+          <t>M5</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Stability</t>
+          <t>Determinism</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>No crash in a 2-hour play session or a 100-year soak test</t>
+          <t>Same seed + inputs give the same world hash after 10,000 ticks</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Soak test + crash log</t>
+          <t>Automated test in CI</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>M5, M6</t>
+          <t>M2 onwards</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
+          <t>Stability</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>No crash in a 2-hour play session or a 100-year soak test</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Soak test + crash log</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>M5, M6</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
           <t>Kill / pivot rule</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>If M1 or M6 fails: stop adding content; redesign the simulation or the loop first</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>If M2 or M6 fails: stop adding content; redesign the simulation or the loop first</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
         <is>
           <t>Owner decision, recorded</t>
         </is>
       </c>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>M1, M6</t>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>M2, M6</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ19"/>
+  <dimension ref="A1:CQ20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1453,6 +1485,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -1463,6 +1496,7 @@
         <v>46300</v>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -1827,7 +1861,7 @@
         <v/>
       </c>
       <c r="M7" s="9">
-        <f>SUMIFS('User Stories'!$H$5:$H$48,'User Stories'!$J$5:$J$48,A7,'User Stories'!$F$5:$F$48,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$48,'User Stories'!$J$5:$J$48,A7,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$53,'User Stories'!$J$5:$J$53,A7,'User Stories'!$F$5:$F$53,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$53,'User Stories'!$J$5:$J$53,A7,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="N7" s="9" t="inlineStr">
@@ -1887,7 +1921,7 @@
         <v/>
       </c>
       <c r="M8" s="9">
-        <f>SUMIFS('User Stories'!$H$5:$H$48,'User Stories'!$J$5:$J$48,A8,'User Stories'!$F$5:$F$48,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$48,'User Stories'!$J$5:$J$48,A8,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$53,'User Stories'!$J$5:$J$53,A8,'User Stories'!$F$5:$F$53,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$53,'User Stories'!$J$5:$J$53,A8,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="N8" s="9" t="inlineStr">
@@ -1899,24 +1933,24 @@
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M1b</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Console clan simulator (KILL GATE 1)</t>
+          <t>Luna Physics (deterministic 3D)</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D9" s="13" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F9" s="9">
         <f>ROUND((D9+E9)/2,0)</f>
@@ -1947,36 +1981,36 @@
         <v/>
       </c>
       <c r="M9" s="9">
-        <f>SUMIFS('User Stories'!$H$5:$H$48,'User Stories'!$J$5:$J$48,A9,'User Stories'!$F$5:$F$48,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$48,'User Stories'!$J$5:$J$48,A9,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$53,'User Stories'!$J$5:$J$53,A9,'User Stories'!$F$5:$F$53,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$53,'User Stories'!$J$5:$J$53,A9,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="N9" s="9" t="inlineStr">
         <is>
-          <t>The headless runner simulates a 20-person clan for 100 years without crashing; the printed chronicle is shown to 3 people and at least 2 find a story in it; the determinism test passes.</t>
+          <t>Luna Physics passes its math, hit-detection, ballistics and rigid-body tests identically on every build; in the demo the hero throws a spear that flies in an arc with a shadow and hits a target.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M2</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Living clan on screen</t>
+          <t>Console clan simulator (KILL GATE 1)</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="D10" s="13" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E10" s="13" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="F10" s="9">
         <f>ROUND((D10+E10)/2,0)</f>
@@ -2007,36 +2041,36 @@
         <v/>
       </c>
       <c r="M10" s="9">
-        <f>SUMIFS('User Stories'!$H$5:$H$48,'User Stories'!$J$5:$J$48,A10,'User Stories'!$F$5:$F$48,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$48,'User Stories'!$J$5:$J$48,A10,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$53,'User Stories'!$J$5:$J$53,A10,'User Stories'!$F$5:$F$53,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$53,'User Stories'!$J$5:$J$53,A10,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="N10" s="9" t="inlineStr">
         <is>
-          <t>The clan from M2 runs inside the game; NPCs are visible, dressed in layered outfits, and act on their needs.</t>
+          <t>The headless runner simulates a 20-person clan for 100 years without crashing; the printed chronicle is shown to 3 people and at least 2 find a story in it; the determinism test passes.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Region, tools and saves</t>
+          <t>Living clan on screen</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>7-9</t>
+          <t>5-6</t>
         </is>
       </c>
       <c r="D11" s="13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F11" s="9">
         <f>ROUND((D11+E11)/2,0)</f>
@@ -2067,36 +2101,36 @@
         <v/>
       </c>
       <c r="M11" s="9">
-        <f>SUMIFS('User Stories'!$H$5:$H$48,'User Stories'!$J$5:$J$48,A11,'User Stories'!$F$5:$F$48,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$48,'User Stories'!$J$5:$J$48,A11,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$53,'User Stories'!$J$5:$J$53,A11,'User Stories'!$F$5:$F$53,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$53,'User Stories'!$J$5:$J$53,A11,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="N11" s="9" t="inlineStr">
         <is>
-          <t>A region is generated from a seed with biomes, resources and two rival clans; any NPC can be inspected; the game saves and loads.</t>
+          <t>The clan from M2 runs inside the game; NPCs are visible, dressed in layered outfits, and act on their needs.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Vertical slice feature-complete</t>
+          <t>Region, tools and saves</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7-9</t>
         </is>
       </c>
       <c r="D12" s="13" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="E12" s="13" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F12" s="9">
         <f>ROUND((D12+E12)/2,0)</f>
@@ -2127,36 +2161,36 @@
         <v/>
       </c>
       <c r="M12" s="9">
-        <f>SUMIFS('User Stories'!$H$5:$H$48,'User Stories'!$J$5:$J$48,A12,'User Stories'!$F$5:$F$48,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$48,'User Stories'!$J$5:$J$48,A12,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$53,'User Stories'!$J$5:$J$53,A12,'User Stories'!$F$5:$F$53,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$53,'User Stories'!$J$5:$J$53,A12,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>A player can start a new game, live the Growing Period, take a profession, pursue Trade or Religion, and win or lose.</t>
+          <t>A region is generated from a seed with biomes, resources and two rival clans; any NPC can be inspected; the game saves and loads.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Playtest and go/no-go (KILL GATE 2)</t>
+          <t>Vertical slice feature-complete</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D13" s="13" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="E13" s="13" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="F13" s="9">
         <f>ROUND((D13+E13)/2,0)</f>
@@ -2187,60 +2221,72 @@
         <v/>
       </c>
       <c r="M13" s="9">
-        <f>SUMIFS('User Stories'!$H$5:$H$48,'User Stories'!$J$5:$J$48,A13,'User Stories'!$F$5:$F$48,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$48,'User Stories'!$J$5:$J$48,A13,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$53,'User Stories'!$J$5:$J$53,A13,'User Stories'!$F$5:$F$53,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$53,'User Stories'!$J$5:$J$53,A13,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
+          <t>A player can start a new game, live the Growing Period, take a profession, pursue Trade or Religion, and win or lose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Playtest and go/no-go (KILL GATE 2)</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" s="9">
+        <f>ROUND((D14+E14)/2,0)</f>
+        <v/>
+      </c>
+      <c r="G14" s="9">
+        <f>H13+1</f>
+        <v/>
+      </c>
+      <c r="H14" s="9">
+        <f>G14+F14-1</f>
+        <v/>
+      </c>
+      <c r="I14" s="14">
+        <f>$B$4+(G14-1)*7</f>
+        <v/>
+      </c>
+      <c r="J14" s="14">
+        <f>$B$4+H14*7-1</f>
+        <v/>
+      </c>
+      <c r="K14" s="14">
+        <f>$B$4+SUM($D$7:D14)*7-1</f>
+        <v/>
+      </c>
+      <c r="L14" s="14">
+        <f>$B$4+SUM($E$7:E14)*7-1</f>
+        <v/>
+      </c>
+      <c r="M14" s="9">
+        <f>SUMIFS('User Stories'!$H$5:$H$53,'User Stories'!$J$5:$J$53,A14,'User Stories'!$F$5:$F$53,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$53,'User Stories'!$J$5:$J$53,A14,'User Stories'!$F$5:$F$53,"Must")</f>
+        <v/>
+      </c>
+      <c r="N14" s="9" t="inlineStr">
+        <is>
           <t>8 outside playtesters play; success criteria measured; go/no-go decision recorded.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr"/>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>MVP total</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr"/>
-      <c r="D14" s="7">
-        <f>SUM(D7:D13)</f>
-        <v/>
-      </c>
-      <c r="E14" s="7">
-        <f>SUM(E7:E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="7">
-        <f>SUM(F7:F13)</f>
-        <v/>
-      </c>
-      <c r="G14" s="7" t="inlineStr"/>
-      <c r="H14" s="7">
-        <f>H13</f>
-        <v/>
-      </c>
-      <c r="I14" s="15">
-        <f>I7</f>
-        <v/>
-      </c>
-      <c r="J14" s="15">
-        <f>J13</f>
-        <v/>
-      </c>
-      <c r="K14" s="15">
-        <f>K13</f>
-        <v/>
-      </c>
-      <c r="L14" s="15">
-        <f>L13</f>
-        <v/>
-      </c>
-      <c r="M14" s="7" t="inlineStr"/>
-      <c r="N14" s="7" t="inlineStr">
-        <is>
-          <t>Months (likely) = weeks / 4.33</t>
         </is>
       </c>
     </row>
@@ -2248,49 +2294,98 @@
       <c r="A15" s="7" t="inlineStr"/>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>In months</t>
+          <t>MVP total</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr"/>
       <c r="D15" s="7">
-        <f>ROUND(D14/4.33,1)</f>
+        <f>SUM(D7:D14)</f>
         <v/>
       </c>
       <c r="E15" s="7">
-        <f>ROUND(E14/4.33,1)</f>
+        <f>SUM(E7:E14)</f>
         <v/>
       </c>
       <c r="F15" s="7">
-        <f>ROUND(F14/4.33,1)</f>
+        <f>SUM(F7:F14)</f>
         <v/>
       </c>
       <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
-      <c r="I15" s="7" t="inlineStr"/>
-      <c r="J15" s="7" t="inlineStr"/>
-      <c r="K15" s="7" t="inlineStr"/>
-      <c r="L15" s="7" t="inlineStr"/>
+      <c r="H15" s="7">
+        <f>H14</f>
+        <v/>
+      </c>
+      <c r="I15" s="15">
+        <f>I7</f>
+        <v/>
+      </c>
+      <c r="J15" s="15">
+        <f>J14</f>
+        <v/>
+      </c>
+      <c r="K15" s="15">
+        <f>K14</f>
+        <v/>
+      </c>
+      <c r="L15" s="15">
+        <f>L14</f>
+        <v/>
+      </c>
       <c r="M15" s="7" t="inlineStr"/>
-      <c r="N15" s="7" t="inlineStr"/>
-    </row>
-    <row r="17" ht="28" customHeight="1">
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Why the estimate grew: the learning path (requirements, section 8.3) estimated 9-13 months top-down. The bottom-up sum of the MVP stories is higher; this sheet uses the bottom-up figure.</t>
-        </is>
-      </c>
-    </row>
+      <c r="N15" s="7" t="inlineStr">
+        <is>
+          <t>Months (likely) = weeks / 4.33</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr"/>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>In months</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr"/>
+      <c r="D16" s="7">
+        <f>ROUND(D15/4.33,1)</f>
+        <v/>
+      </c>
+      <c r="E16" s="7">
+        <f>ROUND(E15/4.33,1)</f>
+        <v/>
+      </c>
+      <c r="F16" s="7">
+        <f>ROUND(F15/4.33,1)</f>
+        <v/>
+      </c>
+      <c r="G16" s="7" t="inlineStr"/>
+      <c r="H16" s="7" t="inlineStr"/>
+      <c r="I16" s="7" t="inlineStr"/>
+      <c r="J16" s="7" t="inlineStr"/>
+      <c r="K16" s="7" t="inlineStr"/>
+      <c r="L16" s="7" t="inlineStr"/>
+      <c r="M16" s="7" t="inlineStr"/>
+      <c r="N16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17" ht="28" customHeight="1"/>
     <row r="18" ht="28" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Buffer: the 'Should' stories are the cut list if time runs short. Cutting all of them saves about 5-11 weeks.</t>
+          <t>Why the estimate grew: the learning path (requirements, section 8.3) estimated 9-13 months top-down. The bottom-up sum of the MVP stories is higher; this sheet uses the bottom-up figure.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Kill gates: M1 (is the console chronicle interesting?) and M6 (do playtesters stay?). If a gate fails, stop adding content and fix the core first.</t>
+          <t>Buffer: the 'Should' stories are the cut list if time runs short. Cutting all of them saves about 5-11 weeks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Kill gates: M2 (is the console chronicle interesting?) and M6 (do playtesters stay?). Critical path: M0 &gt; M1 &gt; M1b &gt; M2 &gt; M3 &gt; M4 &gt; M5 &gt; M6; the engine and its physics come first (owner decisions 2026-09-29/30).</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2395,7 @@
     <mergeCell ref="B17:N17"/>
     <mergeCell ref="B18:N18"/>
   </mergeCells>
-  <conditionalFormatting sqref="P7:CQ13">
+  <conditionalFormatting sqref="P7:CQ14">
     <cfRule type="expression" priority="1" dxfId="2">
       <formula>AND(P$6&gt;=$G7,P$6&lt;=$H7)</formula>
     </cfRule>
@@ -2341,6 +2436,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -2411,7 +2507,7 @@
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2519,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Side Characters interview: needs, traits, relationships (OPEN-10)</t>
+          <t>Side Characters: needs, traits, relationships (OPEN-10). Decided by Dominus (delegated), 2026-09-30.</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -2448,7 +2544,7 @@
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided</t>
         </is>
       </c>
     </row>
@@ -2485,7 +2581,7 @@
       </c>
       <c r="G7" s="16" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Decided</t>
         </is>
       </c>
     </row>
@@ -2904,7 +3000,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Technical chain: M0 &gt; M1 &gt; M2 &gt; M3 &gt; M4 &gt; M5 &gt; M6 (each milestone needs the previous one)</t>
+          <t>Technical chain: M0 &gt; M1 &gt; M1b &gt; M2 &gt; M3 &gt; M4 &gt; M5 &gt; M6 (each milestone needs the previous one)</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -2963,7 +3059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2992,6 +3088,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -3066,23 +3163,23 @@
         </is>
       </c>
       <c r="E5" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$48,A5)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$53,A5)</f>
         <v/>
       </c>
       <c r="F5" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A5,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A5,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="G5" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A5,'User Stories'!$H$5:$H$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A5,'User Stories'!$H$5:$H$53)</f>
         <v/>
       </c>
       <c r="H5" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A5,'User Stories'!$I$5:$I$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A5,'User Stories'!$I$5:$I$53)</f>
         <v/>
       </c>
       <c r="I5" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A5,'User Stories'!$O$5:$O$48,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A5,'User Stories'!$O$5:$O$53,"Done")</f>
         <v/>
       </c>
       <c r="J5" s="17">
@@ -3112,23 +3209,23 @@
         </is>
       </c>
       <c r="E6" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$48,A6)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$53,A6)</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A6,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A6,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="G6" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A6,'User Stories'!$H$5:$H$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A6,'User Stories'!$H$5:$H$53)</f>
         <v/>
       </c>
       <c r="H6" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A6,'User Stories'!$I$5:$I$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A6,'User Stories'!$I$5:$I$53)</f>
         <v/>
       </c>
       <c r="I6" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A6,'User Stories'!$O$5:$O$48,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A6,'User Stories'!$O$5:$O$53,"Done")</f>
         <v/>
       </c>
       <c r="J6" s="17">
@@ -3158,23 +3255,23 @@
         </is>
       </c>
       <c r="E7" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$48,A7)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$53,A7)</f>
         <v/>
       </c>
       <c r="F7" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A7,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A7,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="G7" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A7,'User Stories'!$H$5:$H$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A7,'User Stories'!$H$5:$H$53)</f>
         <v/>
       </c>
       <c r="H7" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A7,'User Stories'!$I$5:$I$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A7,'User Stories'!$I$5:$I$53)</f>
         <v/>
       </c>
       <c r="I7" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A7,'User Stories'!$O$5:$O$48,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A7,'User Stories'!$O$5:$O$53,"Done")</f>
         <v/>
       </c>
       <c r="J7" s="17">
@@ -3204,23 +3301,23 @@
         </is>
       </c>
       <c r="E8" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$48,A8)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$53,A8)</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A8,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A8,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="G8" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A8,'User Stories'!$H$5:$H$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A8,'User Stories'!$H$5:$H$53)</f>
         <v/>
       </c>
       <c r="H8" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A8,'User Stories'!$I$5:$I$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A8,'User Stories'!$I$5:$I$53)</f>
         <v/>
       </c>
       <c r="I8" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A8,'User Stories'!$O$5:$O$48,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A8,'User Stories'!$O$5:$O$53,"Done")</f>
         <v/>
       </c>
       <c r="J8" s="17">
@@ -3250,23 +3347,23 @@
         </is>
       </c>
       <c r="E9" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$48,A9)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$53,A9)</f>
         <v/>
       </c>
       <c r="F9" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A9,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A9,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="G9" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A9,'User Stories'!$H$5:$H$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A9,'User Stories'!$H$5:$H$53)</f>
         <v/>
       </c>
       <c r="H9" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A9,'User Stories'!$I$5:$I$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A9,'User Stories'!$I$5:$I$53)</f>
         <v/>
       </c>
       <c r="I9" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A9,'User Stories'!$O$5:$O$48,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A9,'User Stories'!$O$5:$O$53,"Done")</f>
         <v/>
       </c>
       <c r="J9" s="17">
@@ -3296,23 +3393,23 @@
         </is>
       </c>
       <c r="E10" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$48,A10)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$53,A10)</f>
         <v/>
       </c>
       <c r="F10" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A10,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A10,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="G10" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A10,'User Stories'!$H$5:$H$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A10,'User Stories'!$H$5:$H$53)</f>
         <v/>
       </c>
       <c r="H10" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A10,'User Stories'!$I$5:$I$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A10,'User Stories'!$I$5:$I$53)</f>
         <v/>
       </c>
       <c r="I10" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A10,'User Stories'!$O$5:$O$48,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A10,'User Stories'!$O$5:$O$53,"Done")</f>
         <v/>
       </c>
       <c r="J10" s="17">
@@ -3342,23 +3439,23 @@
         </is>
       </c>
       <c r="E11" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$48,A11)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$53,A11)</f>
         <v/>
       </c>
       <c r="F11" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A11,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A11,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="G11" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A11,'User Stories'!$H$5:$H$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A11,'User Stories'!$H$5:$H$53)</f>
         <v/>
       </c>
       <c r="H11" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A11,'User Stories'!$I$5:$I$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A11,'User Stories'!$I$5:$I$53)</f>
         <v/>
       </c>
       <c r="I11" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A11,'User Stories'!$O$5:$O$48,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A11,'User Stories'!$O$5:$O$53,"Done")</f>
         <v/>
       </c>
       <c r="J11" s="17">
@@ -3388,23 +3485,23 @@
         </is>
       </c>
       <c r="E12" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$48,A12)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$53,A12)</f>
         <v/>
       </c>
       <c r="F12" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A12,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A12,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="G12" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A12,'User Stories'!$H$5:$H$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A12,'User Stories'!$H$5:$H$53)</f>
         <v/>
       </c>
       <c r="H12" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A12,'User Stories'!$I$5:$I$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A12,'User Stories'!$I$5:$I$53)</f>
         <v/>
       </c>
       <c r="I12" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A12,'User Stories'!$O$5:$O$48,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A12,'User Stories'!$O$5:$O$53,"Done")</f>
         <v/>
       </c>
       <c r="J12" s="17">
@@ -3434,23 +3531,23 @@
         </is>
       </c>
       <c r="E13" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$48,A13)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$53,A13)</f>
         <v/>
       </c>
       <c r="F13" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A13,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A13,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="G13" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A13,'User Stories'!$H$5:$H$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A13,'User Stories'!$H$5:$H$53)</f>
         <v/>
       </c>
       <c r="H13" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A13,'User Stories'!$I$5:$I$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A13,'User Stories'!$I$5:$I$53)</f>
         <v/>
       </c>
       <c r="I13" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A13,'User Stories'!$O$5:$O$48,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A13,'User Stories'!$O$5:$O$53,"Done")</f>
         <v/>
       </c>
       <c r="J13" s="17">
@@ -3480,23 +3577,23 @@
         </is>
       </c>
       <c r="E14" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$48,A14)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$53,A14)</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A14,'User Stories'!$F$5:$F$48,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A14,'User Stories'!$F$5:$F$53,"Must")</f>
         <v/>
       </c>
       <c r="G14" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A14,'User Stories'!$H$5:$H$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A14,'User Stories'!$H$5:$H$53)</f>
         <v/>
       </c>
       <c r="H14" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$48,A14,'User Stories'!$I$5:$I$48)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$53,A14,'User Stories'!$I$5:$I$53)</f>
         <v/>
       </c>
       <c r="I14" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$48,A14,'User Stories'!$O$5:$O$48,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A14,'User Stories'!$O$5:$O$53,"Done")</f>
         <v/>
       </c>
       <c r="J14" s="17">
@@ -3505,36 +3602,82 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr"/>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Luna physics</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>Luna simulates hits, throws and bodies with deterministic 3D physics.</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>M1b</t>
+        </is>
+      </c>
+      <c r="E15" s="9">
+        <f>COUNTIF('User Stories'!$B$5:$B$53,A15)</f>
+        <v/>
+      </c>
+      <c r="F15" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A15,'User Stories'!$F$5:$F$53,"Must")</f>
+        <v/>
+      </c>
+      <c r="G15" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$53,A15,'User Stories'!$H$5:$H$53)</f>
+        <v/>
+      </c>
+      <c r="H15" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$53,A15,'User Stories'!$I$5:$I$53)</f>
+        <v/>
+      </c>
+      <c r="I15" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$53,A15,'User Stories'!$O$5:$O$53,"Done")</f>
+        <v/>
+      </c>
+      <c r="J15" s="17">
+        <f>IFERROR(I15/E15,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr"/>
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr"/>
-      <c r="D15" s="7" t="inlineStr"/>
-      <c r="E15" s="7">
-        <f>SUM(E5:E14)</f>
-        <v/>
-      </c>
-      <c r="F15" s="7">
-        <f>SUM(F5:F14)</f>
-        <v/>
-      </c>
-      <c r="G15" s="7">
-        <f>SUM(G5:G14)</f>
-        <v/>
-      </c>
-      <c r="H15" s="7">
-        <f>SUM(H5:H14)</f>
-        <v/>
-      </c>
-      <c r="I15" s="7">
-        <f>SUM(I5:I14)</f>
-        <v/>
-      </c>
-      <c r="J15" s="18">
-        <f>IFERROR(I15/E15,0)</f>
+      <c r="C16" s="7" t="inlineStr"/>
+      <c r="D16" s="7" t="inlineStr"/>
+      <c r="E16" s="7">
+        <f>SUM(E5:E15)</f>
+        <v/>
+      </c>
+      <c r="F16" s="7">
+        <f>SUM(F5:F15)</f>
+        <v/>
+      </c>
+      <c r="G16" s="7">
+        <f>SUM(G5:G15)</f>
+        <v/>
+      </c>
+      <c r="H16" s="7">
+        <f>SUM(H5:H15)</f>
+        <v/>
+      </c>
+      <c r="I16" s="7">
+        <f>SUM(I5:I15)</f>
+        <v/>
+      </c>
+      <c r="J16" s="18">
+        <f>IFERROR(I16/E16,0)</f>
         <v/>
       </c>
     </row>
@@ -3549,7 +3692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O48"/>
+  <dimension ref="A1:O53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3583,6 +3726,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -7199,6 +7343,416 @@
       </c>
       <c r="N48" s="9" t="inlineStr"/>
       <c r="O48" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="124.2" customHeight="1">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>US-025</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>Build deterministic 3D math</t>
+        </is>
+      </c>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>As a developer, I want fixed-point numbers, 3D vectors and rotations in Luna Physics, so that physics gives identical results on every computer and every run.</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Exact arithmetic
+  Given two fixed-point values
+  When they are added, multiplied and divided
+  Then the results equal the expected values bit for bit in Debug, Release and CI
+Scenario: Rotations
+  Given a vector rotated by 90 degrees about the up axis four times
+  When the rotations are applied as quaternions
+  Then it returns to the starting vector within 1/65536 of a unit
+Scenario: Determinism
+  Given two runs of 1,000,000 mixed math operations with the same inputs
+  When both finish
+  Then both produce the same hash</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G49" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H49" s="9">
+        <f>VLOOKUP(G49,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I49" s="9">
+        <f>VLOOKUP(G49,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J49" s="9" t="inlineStr">
+        <is>
+          <t>M1b</t>
+        </is>
+      </c>
+      <c r="K49" s="9" t="inlineStr">
+        <is>
+          <t>US-003</t>
+        </is>
+      </c>
+      <c r="L49" s="9" t="inlineStr">
+        <is>
+          <t>PHY-01, ARC-10, ADR-017</t>
+        </is>
+      </c>
+      <c r="M49" s="9" t="inlineStr">
+        <is>
+          <t>Fixed-point arithmetic; operator overloading; quaternions</t>
+        </is>
+      </c>
+      <c r="N49" s="9" t="n"/>
+      <c r="O49" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="124.2" customHeight="1">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>US-026</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>Detect hits between shapes</t>
+        </is>
+      </c>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>As a developer, I want spheres, capsules and boxes to report overlaps, ray hits and swept hits, so that every hit is found and a fast spear never passes through its target.</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Overlap
+  Given a sphere and a box that touch
+  When their overlap is tested
+  Then a hit is reported with the contact point and normal
+Scenario: No tunnelling
+  Given a projectile moving 10 m per tick towards a 0.2 m target
+  When its path is swept
+  Then the hit is found at the correct time of impact
+Scenario: Many bodies
+  Given 1,000 bodies in a region
+  When one physics step checks them through the spatial grid
+  Then only nearby pairs are tested and the step takes under 2 ms on the development PC</t>
+        </is>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H50" s="9">
+        <f>VLOOKUP(G50,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I50" s="9">
+        <f>VLOOKUP(G50,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J50" s="9" t="inlineStr">
+        <is>
+          <t>M1b</t>
+        </is>
+      </c>
+      <c r="K50" s="9" t="inlineStr">
+        <is>
+          <t>US-025</t>
+        </is>
+      </c>
+      <c r="L50" s="9" t="inlineStr">
+        <is>
+          <t>PHY-02, ARC-10</t>
+        </is>
+      </c>
+      <c r="M50" s="9" t="inlineStr">
+        <is>
+          <t>Structs and pure functions; geometry; spatial grids</t>
+        </is>
+      </c>
+      <c r="N50" s="9" t="n"/>
+      <c r="O50" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="124.2" customHeight="1">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>US-027</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
+        <is>
+          <t>Fly projectiles with real ballistics</t>
+        </is>
+      </c>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>As a hunter, I want thrown spears and darts to fly in true arcs under gravity, drag and wind, so that aim, strength and distance matter.</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Arc
+  Given a spear thrown at 45 degrees and 20 m/s over flat ground without drag
+  When it lands
+  Then its range is v^2/g = 40.8 m within 1%
+Scenario: Drag and wind
+  Given the same throw with air drag and a crosswind
+  When it lands
+  Then it falls short and drifts downwind by the amounts the formulas predict
+Scenario: Aim
+  Given a target 25 m away
+  When the aim solver computes the launch angle for a given speed
+  Then the thrown projectile hits the target</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G51" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H51" s="9">
+        <f>VLOOKUP(G51,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I51" s="9">
+        <f>VLOOKUP(G51,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J51" s="9" t="inlineStr">
+        <is>
+          <t>M1b</t>
+        </is>
+      </c>
+      <c r="K51" s="9" t="inlineStr">
+        <is>
+          <t>US-026</t>
+        </is>
+      </c>
+      <c r="L51" s="9" t="inlineStr">
+        <is>
+          <t>PHY-03, ADR-017</t>
+        </is>
+      </c>
+      <c r="M51" s="9" t="inlineStr">
+        <is>
+          <t>Numerical integration; units</t>
+        </is>
+      </c>
+      <c r="N51" s="9" t="n"/>
+      <c r="O51" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="124.2" customHeight="1">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>US-028</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
+        <is>
+          <t>Push and bounce bodies</t>
+        </is>
+      </c>
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>As a player, I want bodies to have mass, be pushed, slide, bounce and come to rest, so that knockback and thrown or falling objects feel physical.</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Impulse
+  Given a 70 kg body at rest
+  When an impulse of 140 N s pushes it
+  Then its velocity becomes 2 m/s in the impulse direction
+Scenario: Bounce and rest
+  Given a ball dropped onto the ground with restitution 0.5
+  When it bounces
+  Then each bounce reaches a quarter of the previous height and it comes to rest
+Scenario: Friction
+  Given a crate sliding on grass
+  When no force pushes it any more
+  Then it stops within the distance friction predicts</t>
+        </is>
+      </c>
+      <c r="F52" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G52" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H52" s="9">
+        <f>VLOOKUP(G52,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I52" s="9">
+        <f>VLOOKUP(G52,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J52" s="9" t="inlineStr">
+        <is>
+          <t>M1b</t>
+        </is>
+      </c>
+      <c r="K52" s="9" t="inlineStr">
+        <is>
+          <t>US-026</t>
+        </is>
+      </c>
+      <c r="L52" s="9" t="inlineStr">
+        <is>
+          <t>PHY-04, ADR-017</t>
+        </is>
+      </c>
+      <c r="M52" s="9" t="inlineStr">
+        <is>
+          <t>Classes with invariants; fixed-timestep integration</t>
+        </is>
+      </c>
+      <c r="N52" s="9" t="n"/>
+      <c r="O52" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="124.2" customHeight="1">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>US-029</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
+        <is>
+          <t>Throw a spear in the demo</t>
+        </is>
+      </c>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>As a player, I want to throw a spear at a target in the walking skeleton, so that Luna Physics is proven end to end in the real game.</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Throw
+  Given the hero facing a straw target 8 tiles away
+  When I press Interact
+  Then a spear flies in a visible arc with a shadow and hits the target
+Scenario: Material
+  Given a flint-tipped and a wooden spear (materials.json)
+  When each hits the target
+  Then the damage differs by the materials' hardness and density as configured
+Scenario: Blocked
+  Given a target behind a rock
+  When I throw at it
+  Then the spear hits the rock and stops; the target is unharmed</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G53" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H53" s="9">
+        <f>VLOOKUP(G53,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I53" s="9">
+        <f>VLOOKUP(G53,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J53" s="9" t="inlineStr">
+        <is>
+          <t>M1b</t>
+        </is>
+      </c>
+      <c r="K53" s="9" t="inlineStr">
+        <is>
+          <t>US-024, US-027, US-028</t>
+        </is>
+      </c>
+      <c r="L53" s="9" t="inlineStr">
+        <is>
+          <t>PHY-02, PHY-03, PHY-05</t>
+        </is>
+      </c>
+      <c r="M53" s="9" t="inlineStr">
+        <is>
+          <t>Putting it together; content as data (materials.json)</t>
+        </is>
+      </c>
+      <c r="N53" s="9" t="n"/>
+      <c r="O53" s="16" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
@@ -7229,7 +7783,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 O41 O42 O43 O44 O45 O46 O47 O48" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 O41 O42 O43 O44 O45 O46 O47 O48 O49 O50 O51 O52 O53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"To do,In progress,Blocked,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7243,7 +7797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -7265,6 +7819,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -7432,6 +7987,23 @@
       <c r="C13" s="9" t="inlineStr">
         <is>
           <t>Launch</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Advanced physics and chemistry (explosions, vehicles, orbits, heat, fire spread, reactions)</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Age 1 needs hit detection, ballistics, basic bodies and material properties only; the rest belongs to later Ages.</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>With the Age that needs it (PHY-05, PHY-06)</t>
         </is>
       </c>
     </row>
@@ -7466,6 +8038,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -7501,6 +8074,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Docs: sync workspace files from Drive (requirements v1.6, backlog: M2b Story engine)
</commit_message>
<xml_diff>
--- a/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
+++ b/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
@@ -603,7 +603,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -646,7 +645,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
@@ -765,7 +763,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -780,7 +777,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
@@ -1166,7 +1162,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
@@ -1253,12 +1248,12 @@
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Show printed chronicle</t>
+          <t>Show printed chronicle (M2: 3 readers, failed 2026-09-30; M2b retry: the owner reads and judges)</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>M2</t>
+          <t>M2, retried at M2b</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CQ20"/>
+  <dimension ref="A1:CQ21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1485,7 +1480,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -1496,7 +1490,6 @@
         <v>46300</v>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -1861,7 +1854,7 @@
         <v/>
       </c>
       <c r="M7" s="9">
-        <f>SUMIFS('User Stories'!$H$5:$H$53,'User Stories'!$J$5:$J$53,A7,'User Stories'!$F$5:$F$53,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$53,'User Stories'!$J$5:$J$53,A7,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$59,'User Stories'!$J$5:$J$59,A7,'User Stories'!$F$5:$F$59,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$59,'User Stories'!$J$5:$J$59,A7,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="N7" s="9" t="inlineStr">
@@ -1921,7 +1914,7 @@
         <v/>
       </c>
       <c r="M8" s="9">
-        <f>SUMIFS('User Stories'!$H$5:$H$53,'User Stories'!$J$5:$J$53,A8,'User Stories'!$F$5:$F$53,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$53,'User Stories'!$J$5:$J$53,A8,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$59,'User Stories'!$J$5:$J$59,A8,'User Stories'!$F$5:$F$59,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$59,'User Stories'!$J$5:$J$59,A8,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="N8" s="9" t="inlineStr">
@@ -1981,7 +1974,7 @@
         <v/>
       </c>
       <c r="M9" s="9">
-        <f>SUMIFS('User Stories'!$H$5:$H$53,'User Stories'!$J$5:$J$53,A9,'User Stories'!$F$5:$F$53,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$53,'User Stories'!$J$5:$J$53,A9,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$59,'User Stories'!$J$5:$J$59,A9,'User Stories'!$F$5:$F$59,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$59,'User Stories'!$J$5:$J$59,A9,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="N9" s="9" t="inlineStr">
@@ -2041,7 +2034,7 @@
         <v/>
       </c>
       <c r="M10" s="9">
-        <f>SUMIFS('User Stories'!$H$5:$H$53,'User Stories'!$J$5:$J$53,A10,'User Stories'!$F$5:$F$53,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$53,'User Stories'!$J$5:$J$53,A10,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$59,'User Stories'!$J$5:$J$59,A10,'User Stories'!$F$5:$F$59,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$59,'User Stories'!$J$5:$J$59,A10,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="N10" s="9" t="inlineStr">
@@ -2053,24 +2046,24 @@
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>M3</t>
+          <t>M2b</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Living clan on screen</t>
+          <t>Story engine (KILL GATE 1 retry)</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>5-6</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="D11" s="13" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E11" s="13" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="F11" s="9">
         <f>ROUND((D11+E11)/2,0)</f>
@@ -2101,36 +2094,36 @@
         <v/>
       </c>
       <c r="M11" s="9">
-        <f>SUMIFS('User Stories'!$H$5:$H$53,'User Stories'!$J$5:$J$53,A11,'User Stories'!$F$5:$F$53,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$53,'User Stories'!$J$5:$J$53,A11,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$59,'User Stories'!$J$5:$J$59,A11,'User Stories'!$F$5:$F$59,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$59,'User Stories'!$J$5:$J$59,A11,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="N11" s="9" t="inlineStr">
         <is>
-          <t>The clan from M2 runs inside the game; NPCs are visible, dressed in layered outfits, and act on their needs.</t>
+          <t>The chronicle tells the clan's story in fewer, bigger episodes with reasons; every death and feud says why; the 100-year soak still runs without crashing and the determinism test passes; the owner reads the printed story and judges whether it is a story (Kill Gate 1 retry).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Region, tools and saves</t>
+          <t>Living clan on screen</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>7-9</t>
+          <t>5-6</t>
         </is>
       </c>
       <c r="D12" s="13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E12" s="13" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F12" s="9">
         <f>ROUND((D12+E12)/2,0)</f>
@@ -2161,36 +2154,36 @@
         <v/>
       </c>
       <c r="M12" s="9">
-        <f>SUMIFS('User Stories'!$H$5:$H$53,'User Stories'!$J$5:$J$53,A12,'User Stories'!$F$5:$F$53,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$53,'User Stories'!$J$5:$J$53,A12,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$59,'User Stories'!$J$5:$J$59,A12,'User Stories'!$F$5:$F$59,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$59,'User Stories'!$J$5:$J$59,A12,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="N12" s="9" t="inlineStr">
         <is>
-          <t>A region is generated from a seed with biomes, resources and two rival clans; any NPC can be inspected; the game saves and loads.</t>
+          <t>The clan from M2 and M2b runs inside the game; NPCs are visible, dressed in layered outfits, and act on their needs.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M4</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>Vertical slice feature-complete</t>
+          <t>Region, tools and saves</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7-9</t>
         </is>
       </c>
       <c r="D13" s="13" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="E13" s="13" t="n">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F13" s="9">
         <f>ROUND((D13+E13)/2,0)</f>
@@ -2221,36 +2214,36 @@
         <v/>
       </c>
       <c r="M13" s="9">
-        <f>SUMIFS('User Stories'!$H$5:$H$53,'User Stories'!$J$5:$J$53,A13,'User Stories'!$F$5:$F$53,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$53,'User Stories'!$J$5:$J$53,A13,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$59,'User Stories'!$J$5:$J$59,A13,'User Stories'!$F$5:$F$59,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$59,'User Stories'!$J$5:$J$59,A13,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
-          <t>A player can start a new game, live the Growing Period, take a profession, pursue Trade or Religion, and win or lose.</t>
+          <t>A region is generated from a seed with biomes, resources and two rival clans; any NPC can be inspected; the game saves and loads.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>M5</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Playtest and go/no-go (KILL GATE 2)</t>
+          <t>Vertical slice feature-complete</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D14" s="13" t="n">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="E14" s="13" t="n">
-        <v>4</v>
+        <v>31</v>
       </c>
       <c r="F14" s="9">
         <f>ROUND((D14+E14)/2,0)</f>
@@ -2281,60 +2274,72 @@
         <v/>
       </c>
       <c r="M14" s="9">
-        <f>SUMIFS('User Stories'!$H$5:$H$53,'User Stories'!$J$5:$J$53,A14,'User Stories'!$F$5:$F$53,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$53,'User Stories'!$J$5:$J$53,A14,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$59,'User Stories'!$J$5:$J$59,A14,'User Stories'!$F$5:$F$59,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$59,'User Stories'!$J$5:$J$59,A14,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="N14" s="9" t="inlineStr">
         <is>
+          <t>A player can start a new game, live the Growing Period, take a profession, pursue Trade or Religion, and win or lose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Playtest and go/no-go (KILL GATE 2)</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D15" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="F15" s="9">
+        <f>ROUND((D15+E15)/2,0)</f>
+        <v/>
+      </c>
+      <c r="G15" s="9">
+        <f>H14+1</f>
+        <v/>
+      </c>
+      <c r="H15" s="9">
+        <f>G15+F15-1</f>
+        <v/>
+      </c>
+      <c r="I15" s="14">
+        <f>$B$4+(G15-1)*7</f>
+        <v/>
+      </c>
+      <c r="J15" s="14">
+        <f>$B$4+H15*7-1</f>
+        <v/>
+      </c>
+      <c r="K15" s="14">
+        <f>$B$4+SUM($D$7:D15)*7-1</f>
+        <v/>
+      </c>
+      <c r="L15" s="14">
+        <f>$B$4+SUM($E$7:E15)*7-1</f>
+        <v/>
+      </c>
+      <c r="M15" s="9">
+        <f>SUMIFS('User Stories'!$H$5:$H$59,'User Stories'!$J$5:$J$59,A15,'User Stories'!$F$5:$F$59,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$59,'User Stories'!$J$5:$J$59,A15,'User Stories'!$F$5:$F$59,"Must")</f>
+        <v/>
+      </c>
+      <c r="N15" s="9" t="inlineStr">
+        <is>
           <t>8 outside playtesters play; success criteria measured; go/no-go decision recorded.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr"/>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>MVP total</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr"/>
-      <c r="D15" s="7">
-        <f>SUM(D7:D14)</f>
-        <v/>
-      </c>
-      <c r="E15" s="7">
-        <f>SUM(E7:E14)</f>
-        <v/>
-      </c>
-      <c r="F15" s="7">
-        <f>SUM(F7:F14)</f>
-        <v/>
-      </c>
-      <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="7">
-        <f>H14</f>
-        <v/>
-      </c>
-      <c r="I15" s="15">
-        <f>I7</f>
-        <v/>
-      </c>
-      <c r="J15" s="15">
-        <f>J14</f>
-        <v/>
-      </c>
-      <c r="K15" s="15">
-        <f>K14</f>
-        <v/>
-      </c>
-      <c r="L15" s="15">
-        <f>L14</f>
-        <v/>
-      </c>
-      <c r="M15" s="7" t="inlineStr"/>
-      <c r="N15" s="7" t="inlineStr">
-        <is>
-          <t>Months (likely) = weeks / 4.33</t>
         </is>
       </c>
     </row>
@@ -2342,60 +2347,108 @@
       <c r="A16" s="7" t="inlineStr"/>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>In months</t>
+          <t>MVP total</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr"/>
       <c r="D16" s="7">
-        <f>ROUND(D15/4.33,1)</f>
+        <f>SUM(D7:D15)</f>
         <v/>
       </c>
       <c r="E16" s="7">
-        <f>ROUND(E15/4.33,1)</f>
+        <f>SUM(E7:E15)</f>
         <v/>
       </c>
       <c r="F16" s="7">
-        <f>ROUND(F15/4.33,1)</f>
+        <f>SUM(F7:F15)</f>
         <v/>
       </c>
       <c r="G16" s="7" t="inlineStr"/>
-      <c r="H16" s="7" t="inlineStr"/>
-      <c r="I16" s="7" t="inlineStr"/>
-      <c r="J16" s="7" t="inlineStr"/>
-      <c r="K16" s="7" t="inlineStr"/>
-      <c r="L16" s="7" t="inlineStr"/>
+      <c r="H16" s="7">
+        <f>H15</f>
+        <v/>
+      </c>
+      <c r="I16" s="15">
+        <f>I7</f>
+        <v/>
+      </c>
+      <c r="J16" s="15">
+        <f>J15</f>
+        <v/>
+      </c>
+      <c r="K16" s="15">
+        <f>K15</f>
+        <v/>
+      </c>
+      <c r="L16" s="15">
+        <f>L15</f>
+        <v/>
+      </c>
       <c r="M16" s="7" t="inlineStr"/>
-      <c r="N16" s="7" t="inlineStr"/>
-    </row>
-    <row r="17" ht="28" customHeight="1"/>
-    <row r="18" ht="28" customHeight="1">
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Why the estimate grew: the learning path (requirements, section 8.3) estimated 9-13 months top-down. The bottom-up sum of the MVP stories is higher; this sheet uses the bottom-up figure.</t>
-        </is>
-      </c>
-    </row>
+      <c r="N16" s="7" t="inlineStr">
+        <is>
+          <t>Months (likely) = weeks / 4.33</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="7" t="inlineStr"/>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>In months</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr"/>
+      <c r="D17" s="7">
+        <f>ROUND(D16/4.33,1)</f>
+        <v/>
+      </c>
+      <c r="E17" s="7">
+        <f>ROUND(E16/4.33,1)</f>
+        <v/>
+      </c>
+      <c r="F17" s="7">
+        <f>ROUND(F16/4.33,1)</f>
+        <v/>
+      </c>
+      <c r="G17" s="7" t="inlineStr"/>
+      <c r="H17" s="7" t="inlineStr"/>
+      <c r="I17" s="7" t="inlineStr"/>
+      <c r="J17" s="7" t="inlineStr"/>
+      <c r="K17" s="7" t="inlineStr"/>
+      <c r="L17" s="7" t="inlineStr"/>
+      <c r="M17" s="7" t="inlineStr"/>
+      <c r="N17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18" ht="28" customHeight="1"/>
     <row r="19" ht="28" customHeight="1">
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Buffer: the 'Should' stories are the cut list if time runs short. Cutting all of them saves about 5-11 weeks.</t>
+          <t>Why the estimate grew: the learning path (requirements, section 8.3) estimated 9-13 months top-down. The bottom-up sum of the MVP stories is higher; this sheet uses the bottom-up figure.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Kill gates: M2 (is the console chronicle interesting?) and M6 (do playtesters stay?). Critical path: M0 &gt; M1 &gt; M1b &gt; M2 &gt; M3 &gt; M4 &gt; M5 &gt; M6; the engine and its physics come first (owner decisions 2026-09-29/30).</t>
+          <t>Buffer: the 'Should' stories are the cut list if time runs short. Cutting all of them saves about 5-11 weeks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Kill gates: M2 (is the console chronicle interesting? failed 2026-09-30; retried at M2b) and M6 (do playtesters stay?). Critical path: M0 &gt; M1 &gt; M1b &gt; M2 &gt; M2b &gt; M3 &gt; M4 &gt; M5 &gt; M6; the engine and its physics come first (owner decisions 2026-09-29/30).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B19:N19"/>
-    <mergeCell ref="B17:N17"/>
+    <mergeCell ref="B20:N20"/>
     <mergeCell ref="B18:N18"/>
   </mergeCells>
-  <conditionalFormatting sqref="P7:CQ14">
+  <conditionalFormatting sqref="P7:CQ15">
     <cfRule type="expression" priority="1" dxfId="2">
       <formula>AND(P$6&gt;=$G7,P$6&lt;=$H7)</formula>
     </cfRule>
@@ -2410,7 +2463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2436,7 +2489,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -3000,7 +3052,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Technical chain: M0 &gt; M1 &gt; M1b &gt; M2 &gt; M3 &gt; M4 &gt; M5 &gt; M6 (each milestone needs the previous one)</t>
+          <t>Technical chain: M0 &gt; M1 &gt; M1b &gt; M2 &gt; M2b &gt; M3 &gt; M4 &gt; M5 &gt; M6 (each milestone needs the previous one)</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -3026,6 +3078,117 @@
       <c r="G19" s="16" t="inlineStr">
         <is>
           <t>Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>D-GATE-M2</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Kill Gate 1 result: did 2 of 3 readers find a story in the console chronicle?</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>External / people</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>M2 exit</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>M3 (all)</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G20" s="16" t="inlineStr">
+        <is>
+          <t>Decided: Pivot</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>D-18</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Story pivot design: story arcs on a richer social simulation; quarrels, blame, revenge; sharing and nursing; courtship and rivals; teaching and hunting parties; episodes plus lines with reasons; the owner judges the retry alone</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Design decision</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>M2b</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>US-110..US-115</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G21" s="16" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>D-GATE-M2b</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Kill Gate 1 retry: the owner reads the M2b story and judges whether it is a story</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>External / people</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>M2b exit</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>M3 (all)</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G22" s="16" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3059,7 +3222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3088,7 +3251,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -3163,23 +3325,23 @@
         </is>
       </c>
       <c r="E5" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$53,A5)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$59,A5)</f>
         <v/>
       </c>
       <c r="F5" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A5,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A5,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="G5" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A5,'User Stories'!$H$5:$H$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A5,'User Stories'!$H$5:$H$59)</f>
         <v/>
       </c>
       <c r="H5" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A5,'User Stories'!$I$5:$I$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A5,'User Stories'!$I$5:$I$59)</f>
         <v/>
       </c>
       <c r="I5" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A5,'User Stories'!$O$5:$O$53,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A5,'User Stories'!$O$5:$O$59,"Done")</f>
         <v/>
       </c>
       <c r="J5" s="17">
@@ -3209,23 +3371,23 @@
         </is>
       </c>
       <c r="E6" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$53,A6)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$59,A6)</f>
         <v/>
       </c>
       <c r="F6" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A6,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A6,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="G6" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A6,'User Stories'!$H$5:$H$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A6,'User Stories'!$H$5:$H$59)</f>
         <v/>
       </c>
       <c r="H6" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A6,'User Stories'!$I$5:$I$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A6,'User Stories'!$I$5:$I$59)</f>
         <v/>
       </c>
       <c r="I6" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A6,'User Stories'!$O$5:$O$53,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A6,'User Stories'!$O$5:$O$59,"Done")</f>
         <v/>
       </c>
       <c r="J6" s="17">
@@ -3255,23 +3417,23 @@
         </is>
       </c>
       <c r="E7" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$53,A7)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$59,A7)</f>
         <v/>
       </c>
       <c r="F7" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A7,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A7,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="G7" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A7,'User Stories'!$H$5:$H$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A7,'User Stories'!$H$5:$H$59)</f>
         <v/>
       </c>
       <c r="H7" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A7,'User Stories'!$I$5:$I$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A7,'User Stories'!$I$5:$I$59)</f>
         <v/>
       </c>
       <c r="I7" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A7,'User Stories'!$O$5:$O$53,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A7,'User Stories'!$O$5:$O$59,"Done")</f>
         <v/>
       </c>
       <c r="J7" s="17">
@@ -3301,23 +3463,23 @@
         </is>
       </c>
       <c r="E8" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$53,A8)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$59,A8)</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A8,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A8,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="G8" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A8,'User Stories'!$H$5:$H$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A8,'User Stories'!$H$5:$H$59)</f>
         <v/>
       </c>
       <c r="H8" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A8,'User Stories'!$I$5:$I$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A8,'User Stories'!$I$5:$I$59)</f>
         <v/>
       </c>
       <c r="I8" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A8,'User Stories'!$O$5:$O$53,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A8,'User Stories'!$O$5:$O$59,"Done")</f>
         <v/>
       </c>
       <c r="J8" s="17">
@@ -3347,23 +3509,23 @@
         </is>
       </c>
       <c r="E9" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$53,A9)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$59,A9)</f>
         <v/>
       </c>
       <c r="F9" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A9,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A9,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="G9" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A9,'User Stories'!$H$5:$H$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A9,'User Stories'!$H$5:$H$59)</f>
         <v/>
       </c>
       <c r="H9" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A9,'User Stories'!$I$5:$I$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A9,'User Stories'!$I$5:$I$59)</f>
         <v/>
       </c>
       <c r="I9" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A9,'User Stories'!$O$5:$O$53,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A9,'User Stories'!$O$5:$O$59,"Done")</f>
         <v/>
       </c>
       <c r="J9" s="17">
@@ -3393,23 +3555,23 @@
         </is>
       </c>
       <c r="E10" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$53,A10)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$59,A10)</f>
         <v/>
       </c>
       <c r="F10" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A10,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A10,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="G10" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A10,'User Stories'!$H$5:$H$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A10,'User Stories'!$H$5:$H$59)</f>
         <v/>
       </c>
       <c r="H10" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A10,'User Stories'!$I$5:$I$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A10,'User Stories'!$I$5:$I$59)</f>
         <v/>
       </c>
       <c r="I10" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A10,'User Stories'!$O$5:$O$53,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A10,'User Stories'!$O$5:$O$59,"Done")</f>
         <v/>
       </c>
       <c r="J10" s="17">
@@ -3439,23 +3601,23 @@
         </is>
       </c>
       <c r="E11" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$53,A11)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$59,A11)</f>
         <v/>
       </c>
       <c r="F11" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A11,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A11,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="G11" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A11,'User Stories'!$H$5:$H$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A11,'User Stories'!$H$5:$H$59)</f>
         <v/>
       </c>
       <c r="H11" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A11,'User Stories'!$I$5:$I$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A11,'User Stories'!$I$5:$I$59)</f>
         <v/>
       </c>
       <c r="I11" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A11,'User Stories'!$O$5:$O$53,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A11,'User Stories'!$O$5:$O$59,"Done")</f>
         <v/>
       </c>
       <c r="J11" s="17">
@@ -3485,23 +3647,23 @@
         </is>
       </c>
       <c r="E12" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$53,A12)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$59,A12)</f>
         <v/>
       </c>
       <c r="F12" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A12,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A12,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="G12" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A12,'User Stories'!$H$5:$H$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A12,'User Stories'!$H$5:$H$59)</f>
         <v/>
       </c>
       <c r="H12" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A12,'User Stories'!$I$5:$I$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A12,'User Stories'!$I$5:$I$59)</f>
         <v/>
       </c>
       <c r="I12" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A12,'User Stories'!$O$5:$O$53,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A12,'User Stories'!$O$5:$O$59,"Done")</f>
         <v/>
       </c>
       <c r="J12" s="17">
@@ -3531,23 +3693,23 @@
         </is>
       </c>
       <c r="E13" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$53,A13)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$59,A13)</f>
         <v/>
       </c>
       <c r="F13" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A13,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A13,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="G13" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A13,'User Stories'!$H$5:$H$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A13,'User Stories'!$H$5:$H$59)</f>
         <v/>
       </c>
       <c r="H13" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A13,'User Stories'!$I$5:$I$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A13,'User Stories'!$I$5:$I$59)</f>
         <v/>
       </c>
       <c r="I13" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A13,'User Stories'!$O$5:$O$53,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A13,'User Stories'!$O$5:$O$59,"Done")</f>
         <v/>
       </c>
       <c r="J13" s="17">
@@ -3577,23 +3739,23 @@
         </is>
       </c>
       <c r="E14" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$53,A14)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$59,A14)</f>
         <v/>
       </c>
       <c r="F14" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A14,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A14,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="G14" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A14,'User Stories'!$H$5:$H$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A14,'User Stories'!$H$5:$H$59)</f>
         <v/>
       </c>
       <c r="H14" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A14,'User Stories'!$I$5:$I$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A14,'User Stories'!$I$5:$I$59)</f>
         <v/>
       </c>
       <c r="I14" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A14,'User Stories'!$O$5:$O$53,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A14,'User Stories'!$O$5:$O$59,"Done")</f>
         <v/>
       </c>
       <c r="J14" s="17">
@@ -3623,23 +3785,23 @@
         </is>
       </c>
       <c r="E15" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$53,A15)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$59,A15)</f>
         <v/>
       </c>
       <c r="F15" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A15,'User Stories'!$F$5:$F$53,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A15,'User Stories'!$F$5:$F$59,"Must")</f>
         <v/>
       </c>
       <c r="G15" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A15,'User Stories'!$H$5:$H$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A15,'User Stories'!$H$5:$H$59)</f>
         <v/>
       </c>
       <c r="H15" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$53,A15,'User Stories'!$I$5:$I$53)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$59,A15,'User Stories'!$I$5:$I$59)</f>
         <v/>
       </c>
       <c r="I15" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$53,A15,'User Stories'!$O$5:$O$53,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A15,'User Stories'!$O$5:$O$59,"Done")</f>
         <v/>
       </c>
       <c r="J15" s="17">
@@ -3648,36 +3810,82 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr"/>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>E11</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Story engine</t>
+        </is>
+      </c>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>The clan's life becomes a readable story: episodes with causes, people and consequences.</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>M2b</t>
+        </is>
+      </c>
+      <c r="E16" s="9">
+        <f>COUNTIF('User Stories'!$B$5:$B$59,A16)</f>
+        <v/>
+      </c>
+      <c r="F16" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A16,'User Stories'!$F$5:$F$59,"Must")</f>
+        <v/>
+      </c>
+      <c r="G16" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$59,A16,'User Stories'!$H$5:$H$59)</f>
+        <v/>
+      </c>
+      <c r="H16" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$59,A16,'User Stories'!$I$5:$I$59)</f>
+        <v/>
+      </c>
+      <c r="I16" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$59,A16,'User Stories'!$O$5:$O$59,"Done")</f>
+        <v/>
+      </c>
+      <c r="J16" s="17">
+        <f>IFERROR(I16/E16,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr"/>
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr"/>
-      <c r="D16" s="7" t="inlineStr"/>
-      <c r="E16" s="7">
-        <f>SUM(E5:E15)</f>
-        <v/>
-      </c>
-      <c r="F16" s="7">
-        <f>SUM(F5:F15)</f>
-        <v/>
-      </c>
-      <c r="G16" s="7">
-        <f>SUM(G5:G15)</f>
-        <v/>
-      </c>
-      <c r="H16" s="7">
-        <f>SUM(H5:H15)</f>
-        <v/>
-      </c>
-      <c r="I16" s="7">
-        <f>SUM(I5:I15)</f>
-        <v/>
-      </c>
-      <c r="J16" s="18">
-        <f>IFERROR(I16/E16,0)</f>
+      <c r="C17" s="7" t="inlineStr"/>
+      <c r="D17" s="7" t="inlineStr"/>
+      <c r="E17" s="7">
+        <f>SUM(E5:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="7">
+        <f>SUM(F5:F16)</f>
+        <v/>
+      </c>
+      <c r="G17" s="7">
+        <f>SUM(G5:G16)</f>
+        <v/>
+      </c>
+      <c r="H17" s="7">
+        <f>SUM(H5:H16)</f>
+        <v/>
+      </c>
+      <c r="I17" s="7">
+        <f>SUM(I5:I16)</f>
+        <v/>
+      </c>
+      <c r="J17" s="18">
+        <f>IFERROR(I17/E17,0)</f>
         <v/>
       </c>
     </row>
@@ -3692,7 +3900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O53"/>
+  <dimension ref="A1:O59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3726,7 +3934,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -7758,9 +7965,525 @@
         </is>
       </c>
     </row>
+    <row r="54" ht="124.2" customHeight="1">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>US-110</t>
+        </is>
+      </c>
+      <c r="B54" s="9" t="inlineStr">
+        <is>
+          <t>E11</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
+        <is>
+          <t>Give every death and feud a reason</t>
+        </is>
+      </c>
+      <c r="D54" s="9" t="inlineStr">
+        <is>
+          <t>As a reader, I want every death and feud in the chronicle to say why it happened, so that events connect into a story.</t>
+        </is>
+      </c>
+      <c r="E54" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Death with a cause
+  Given a person who starves after the food store was robbed or ran empty
+  When the death is recorded
+  Then the sentence names the cause and the event behind it, e.g. 'Winter, year 74: Hano died of hunger in the hard winter, after Brak stole from the store.'
+Scenario: Feud with a reason
+  Given two people whose opinions fell through thefts, quarrels or blame
+  When their feud begins
+  Then the sentence names what turned them, e.g. 'A feud broke out between Tok and Brak over stolen meat.'
+Scenario: Traceable
+  Given any death or feud in the chronicle
+  When I inspect it in the headless runner
+  Then it lists the earlier events that caused it</t>
+        </is>
+      </c>
+      <c r="F54" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G54" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H54" s="9">
+        <f>VLOOKUP(G54,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I54" s="9">
+        <f>VLOOKUP(G54,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J54" s="9" t="inlineStr">
+        <is>
+          <t>M2b</t>
+        </is>
+      </c>
+      <c r="K54" s="9" t="inlineStr">
+        <is>
+          <t>US-014</t>
+        </is>
+      </c>
+      <c r="L54" s="9" t="inlineStr">
+        <is>
+          <t>STO-03, NA-02</t>
+        </is>
+      </c>
+      <c r="M54" s="9" t="inlineStr">
+        <is>
+          <t>Small structs that point to other data (event ids); enums</t>
+        </is>
+      </c>
+      <c r="N54" s="9" t="inlineStr">
+        <is>
+          <t>Kill Gate 1 pivot (owner, 2026-09-30, D-18)</t>
+        </is>
+      </c>
+      <c r="O54" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="124.2" customHeight="1">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>US-111</t>
+        </is>
+      </c>
+      <c r="B55" s="9" t="inlineStr">
+        <is>
+          <t>E11</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
+        <is>
+          <t>Quarrel, blame and take revenge</t>
+        </is>
+      </c>
+      <c r="D55" s="9" t="inlineStr">
+        <is>
+          <t>As a player, I want people to quarrel, blame each other for losses and seek revenge, so that conflicts have causes and consequences.</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Quarrel
+  Given two tired or hungry people who dislike each other
+  When they meet
+  Then they may quarrel; both remember it and think less of each other
+Scenario: Blame
+  Given a person whose close kin died after a theft they know of, or on a hunt someone led
+  When they grieve
+  Then they blame the person linked to the cause and remember it for life
+Scenario: Revenge
+  Given a feud that keeps worsening
+  When revenge is taken
+  Then it ends in a fight (injury or death) or the clan exiles the aggressor, and the chronicle tells which and why</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G55" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H55" s="9">
+        <f>VLOOKUP(G55,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I55" s="9">
+        <f>VLOOKUP(G55,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J55" s="9" t="inlineStr">
+        <is>
+          <t>M2b</t>
+        </is>
+      </c>
+      <c r="K55" s="9" t="inlineStr">
+        <is>
+          <t>US-110</t>
+        </is>
+      </c>
+      <c r="L55" s="9" t="inlineStr">
+        <is>
+          <t>SDC-02, GD-03</t>
+        </is>
+      </c>
+      <c r="M55" s="9" t="inlineStr">
+        <is>
+          <t>State machines with enums; std::optional</t>
+        </is>
+      </c>
+      <c r="N55" s="9" t="inlineStr">
+        <is>
+          <t>Kill Gate 1 pivot (owner, 2026-09-30, D-18)</t>
+        </is>
+      </c>
+      <c r="O55" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="124.2" customHeight="1">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>US-112</t>
+        </is>
+      </c>
+      <c r="B56" s="9" t="inlineStr">
+        <is>
+          <t>E11</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
+        <is>
+          <t>Share food and nurse the sick</t>
+        </is>
+      </c>
+      <c r="D56" s="9" t="inlineStr">
+        <is>
+          <t>As a player, I want people to share food in hard times and care for the sick and injured, so that kindness has weight and debts of gratitude form.</t>
+        </is>
+      </c>
+      <c r="E56" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Sickness
+  Given a person weakened by cold, hunger or a hunting wound
+  When sickness or injury strikes
+  Then they are sick or injured for some days and may die of it
+Scenario: Nursing
+  Given a sick person and a kind or close person nearby
+  When they are nursed
+  Then recovery is likelier and the patient remembers the carer with gratitude
+Scenario: Sharing and adoption
+  Given a hungry child or an orphan
+  When a relative or friend has food or room
+  Then they share or adopt, and the one helped remembers it</t>
+        </is>
+      </c>
+      <c r="F56" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G56" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H56" s="9">
+        <f>VLOOKUP(G56,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I56" s="9">
+        <f>VLOOKUP(G56,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J56" s="9" t="inlineStr">
+        <is>
+          <t>M2b</t>
+        </is>
+      </c>
+      <c r="K56" s="9" t="inlineStr">
+        <is>
+          <t>US-110</t>
+        </is>
+      </c>
+      <c r="L56" s="9" t="inlineStr">
+        <is>
+          <t>SDC-02</t>
+        </is>
+      </c>
+      <c r="M56" s="9" t="inlineStr">
+        <is>
+          <t>Standard algorithms: std::find_if, std::max_element, std::sort</t>
+        </is>
+      </c>
+      <c r="N56" s="9" t="inlineStr">
+        <is>
+          <t>Kill Gate 1 pivot (owner, 2026-09-30, D-18)</t>
+        </is>
+      </c>
+      <c r="O56" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="124.2" customHeight="1">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>US-113</t>
+        </is>
+      </c>
+      <c r="B57" s="9" t="inlineStr">
+        <is>
+          <t>E11</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
+        <is>
+          <t>Court and compete for a partner</t>
+        </is>
+      </c>
+      <c r="D57" s="9" t="inlineStr">
+        <is>
+          <t>As a player, I want courtship with rivals and broken pairings, so that love brings drama as well as children.</t>
+        </is>
+      </c>
+      <c r="E57" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Courtship
+  Given an unpaired adult who favours another
+  When they court (gifts, time together)
+  Then the other's opinion rises, and they pair only when both agree
+Scenario: Rivals
+  Given two suitors courting the same person
+  When one is chosen
+  Then the rivals become jealous and may quarrel, and the one not chosen remembers it
+Scenario: Parting
+  Given partners whose opinions of each other fall below the parting threshold
+  When a day ends
+  Then they part, and the chronicle records why</t>
+        </is>
+      </c>
+      <c r="F57" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G57" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H57" s="9">
+        <f>VLOOKUP(G57,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I57" s="9">
+        <f>VLOOKUP(G57,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J57" s="9" t="inlineStr">
+        <is>
+          <t>M2b</t>
+        </is>
+      </c>
+      <c r="K57" s="9" t="inlineStr">
+        <is>
+          <t>US-111</t>
+        </is>
+      </c>
+      <c r="L57" s="9" t="inlineStr">
+        <is>
+          <t>SDC-02</t>
+        </is>
+      </c>
+      <c r="M57" s="9" t="inlineStr">
+        <is>
+          <t>Comparators and ranking (std::sort with a lambda)</t>
+        </is>
+      </c>
+      <c r="N57" s="9" t="inlineStr">
+        <is>
+          <t>Kill Gate 1 pivot (owner, 2026-09-30, D-18)</t>
+        </is>
+      </c>
+      <c r="O57" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="124.2" customHeight="1">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>US-114</t>
+        </is>
+      </c>
+      <c r="B58" s="9" t="inlineStr">
+        <is>
+          <t>E11</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>Teach the young and hunt together</t>
+        </is>
+      </c>
+      <c r="D58" s="9" t="inlineStr">
+        <is>
+          <t>As a player, I want masters to teach apprentices and hunters to go out in parties, so that skills pass down and hunts create heroes and cowards.</t>
+        </is>
+      </c>
+      <c r="E58" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Apprenticeship
+  Given a skilled adult and a youth of working age
+  When the adult takes the youth as apprentice
+  Then the youth's skill grows faster and they grow close
+Scenario: Hunting party
+  Given a mammoth sighting
+  When a party of 3 to 5 hunters forms and hunts
+  Then roles emerge (leader, hero, coward), the outcome depends on the party, and each member remembers what the others did
+Scenario: Rescue
+  Given a hunter in danger
+  When another hunter saves them
+  Then the rescued owes a debt of gratitude and the chronicle tells of it</t>
+        </is>
+      </c>
+      <c r="F58" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G58" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H58" s="9">
+        <f>VLOOKUP(G58,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I58" s="9">
+        <f>VLOOKUP(G58,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J58" s="9" t="inlineStr">
+        <is>
+          <t>M2b</t>
+        </is>
+      </c>
+      <c r="K58" s="9" t="inlineStr">
+        <is>
+          <t>US-111</t>
+        </is>
+      </c>
+      <c r="L58" s="9" t="inlineStr">
+        <is>
+          <t>SDC-02</t>
+        </is>
+      </c>
+      <c r="M58" s="9" t="inlineStr">
+        <is>
+          <t>A class that coordinates others (the hunting party)</t>
+        </is>
+      </c>
+      <c r="N58" s="9" t="inlineStr">
+        <is>
+          <t>Kill Gate 1 pivot (owner, 2026-09-30, D-18)</t>
+        </is>
+      </c>
+      <c r="O58" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="124.2" customHeight="1">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>US-115</t>
+        </is>
+      </c>
+      <c r="B59" s="9" t="inlineStr">
+        <is>
+          <t>E11</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
+        <is>
+          <t>Tell the clan's story in episodes</t>
+        </is>
+      </c>
+      <c r="D59" s="9" t="inlineStr">
+        <is>
+          <t>As a reader, I want the chronicle to tell fewer, bigger episodes with a beginning, a turn and an end, so that I can follow the clan's story.</t>
+        </is>
+      </c>
+      <c r="E59" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Episode
+  Given linked events (a lean autumn, thefts, blame, a feud, deaths)
+  When the episode ends
+  Then the chronicle writes it as one short named paragraph ('The Hard Winter of year 74') saying who, why and what came of it
+Scenario: Fewer, bigger
+  Given a 100-year run
+  When I print the story
+  Then it tells at most 40 episodes, each naming its people and causes, followed by the births, deaths, pairings and feuds with their reasons
+Scenario: Both views
+  Given the headless runner
+  When I ask for the story or for the full chronicle
+  Then --story prints the episodes and --chronicle still prints every event</t>
+        </is>
+      </c>
+      <c r="F59" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G59" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H59" s="9">
+        <f>VLOOKUP(G59,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I59" s="9">
+        <f>VLOOKUP(G59,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J59" s="9" t="inlineStr">
+        <is>
+          <t>M2b</t>
+        </is>
+      </c>
+      <c r="K59" s="9" t="inlineStr">
+        <is>
+          <t>US-110, US-111, US-112, US-113, US-114</t>
+        </is>
+      </c>
+      <c r="L59" s="9" t="inlineStr">
+        <is>
+          <t>STO-02, STO-03, NA-02</t>
+        </is>
+      </c>
+      <c r="M59" s="9" t="inlineStr">
+        <is>
+          <t>Designing with data: grouping and summarising</t>
+        </is>
+      </c>
+      <c r="N59" s="9" t="inlineStr">
+        <is>
+          <t>Kill Gate 1 pivot (owner, 2026-09-30, D-18)</t>
+        </is>
+      </c>
+      <c r="O59" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:O48"/>
-  <conditionalFormatting sqref="F5:F48">
+  <conditionalFormatting sqref="F5:F59">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>"Must"</formula>
     </cfRule>
@@ -7771,7 +8494,7 @@
       <formula>"Could"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O5:O48">
+  <conditionalFormatting sqref="O5:O59">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
       <formula>"Done"</formula>
     </cfRule>
@@ -7783,7 +8506,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 O41 O42 O43 O44 O45 O46 O47 O48 O49 O50 O51 O52 O53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="O5 O6 O7 O8 O9 O10 O11 O12 O13 O14 O15 O16 O17 O18 O19 O20 O21 O22 O23 O24 O25 O26 O27 O28 O29 O30 O31 O32 O33 O34 O35 O36 O37 O38 O39 O40 O41 O42 O43 O44 O45 O46 O47 O48 O49 O50 O51 O52 O53 O54:O59" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"To do,In progress,Blocked,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7819,7 +8542,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -8038,7 +8760,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -8074,7 +8795,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Docs: M2d brief, requirements v1.8 and Codex v1.8 (content and combat)
</commit_message>
<xml_diff>
--- a/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
+++ b/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\~gamerrr\Project Odysseus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE7448E4-0179-4E8E-BC03-F8F7D27F764A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{623BF406-4428-4723-998E-0CE960D394F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1223" uniqueCount="757">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1361" uniqueCount="823">
   <si>
     <t>Project Odyssey - MVP Backlog</t>
   </si>
@@ -2915,6 +2915,267 @@
   </si>
   <si>
     <t>US-120..US-126</t>
+  </si>
+  <si>
+    <t>US-130</t>
+  </si>
+  <si>
+    <t>E13</t>
+  </si>
+  <si>
+    <t>Content catalogs from the new sheets</t>
+  </si>
+  <si>
+    <t>As the owner, I want my seven new sprite sheets cut into game atlases and catalogs, so that weapons, plants, animals, effects and weather can be used in the game.</t>
+  </si>
+  <si>
+    <t>Scenario: Cut
+Given the seven sheets and cuts.json
+When the atlas tool runs
+Then atlases and JSON catalogs exist for weapons, plants, animals, effects and weather, backgrounds removed
+Scenario: Review
+Given the owner
+When the owner opens the numbered contact sheets
+Then every item is shown with its catalog name</t>
+  </si>
+  <si>
+    <t>M2d</t>
+  </si>
+  <si>
+    <t>D-05, D-21, ARC-08</t>
+  </si>
+  <si>
+    <t>Reading data tables with std::map and validating them</t>
+  </si>
+  <si>
+    <t>Content and combat (owner, 2026-09-30, D-21)</t>
+  </si>
+  <si>
+    <t>US-131</t>
+  </si>
+  <si>
+    <t>Hero HP, fighting back and death</t>
+  </si>
+  <si>
+    <t>As the player, I want enemies to strike back when I hit them, so that fighting has risk.</t>
+  </si>
+  <si>
+    <t>Scenario: Strike back
+Given an enemy the hero hits while standing within 1.5 m
+When 0.5 s pass with a warning flash
+Then the hero loses the enemy kind's damage
+Scenario: Death
+Given the hero or an enemy at 0 HP
+When it happens
+Then the hero respawns at the start with 100 HP; the enemy dies and is gone until the level restarts</t>
+  </si>
+  <si>
+    <t>D-21</t>
+  </si>
+  <si>
+    <t>A small state machine with enum class</t>
+  </si>
+  <si>
+    <t>US-132</t>
+  </si>
+  <si>
+    <t>Effect player</t>
+  </si>
+  <si>
+    <t>As the player, I want hits, deaths and projectiles to show effects, so that combat reads clearly.</t>
+  </si>
+  <si>
+    <t>Scenario: One-shot
+Given an effect started in the world
+When its frames have played
+Then it disappears
+Scenario: Combat
+Given a sword hit, a death or an arrow in flight
+When it happens
+Then a hit spark, a smoke puff or a trail plays</t>
+  </si>
+  <si>
+    <t>D-21, ARC-09</t>
+  </si>
+  <si>
+    <t>Timers and animation frames in a fixed timestep</t>
+  </si>
+  <si>
+    <t>US-133</t>
+  </si>
+  <si>
+    <t>Weapon classes and the starter set</t>
+  </si>
+  <si>
+    <t>As the player, I want each kind of weapon to fight differently, so that choosing a weapon matters.</t>
+  </si>
+  <si>
+    <t>Scenario: Classes
+Given each of the 8 classes
+When the hero attacks
+Then its own attack shape, speed and range are used from JSON
+Scenario: In hand
+Given a weapon selected
+When the hero walks
+Then the weapon icon is drawn in the hero's hand</t>
+  </si>
+  <si>
+    <t>US-130, US-132</t>
+  </si>
+  <si>
+    <t>Virtual functions or std::variant for weapon classes</t>
+  </si>
+  <si>
+    <t>US-134</t>
+  </si>
+  <si>
+    <t>Pickups and the hotbar</t>
+  </si>
+  <si>
+    <t>As a level designer, I want to place weapons in my levels for the hero to find, so that levels have rewards.</t>
+  </si>
+  <si>
+    <t>Scenario: Pick up
+Given the hero walks over a pickup
+When it happens
+Then the weapon goes into the first free of 9 hotbar slots
+Scenario: Select
+Given weapons in the hotbar
+When I press 1-9 or Shift
+Then that weapon, or the next one, is held</t>
+  </si>
+  <si>
+    <t>D-21, ADR-010</t>
+  </si>
+  <si>
+    <t>Upgrading a saved file format (version 1 to 2)</t>
+  </si>
+  <si>
+    <t>US-135</t>
+  </si>
+  <si>
+    <t>Elements</t>
+  </si>
+  <si>
+    <t>As the player, I want elemental weapons to do something special, so that they feel different.</t>
+  </si>
+  <si>
+    <t>Scenario: Over time
+Given a hit with a fire or poison weapon
+When seconds pass
+Then the target loses HP over time with its effect showing
+Scenario: Lightning
+Given a hit with a lightning weapon and a second enemy nearby
+When it happens
+Then the lightning jumps to that enemy</t>
+  </si>
+  <si>
+    <t>Components: small structs attached to characters</t>
+  </si>
+  <si>
+    <t>US-136</t>
+  </si>
+  <si>
+    <t>Plants</t>
+  </si>
+  <si>
+    <t>As a level designer and player, I want plants in the world that block, can be looked at, chopped and eaten, so that the world feels alive.</t>
+  </si>
+  <si>
+    <t>Scenario: Chop
+Given the hero next to a plant
+When the player hits it with a weapon
+Then it is destroyed with a leaf burst; an edible plant heals 10 HP
+Scenario: Regrow
+Given a destroyed plant
+When 15 s pass
+Then the same plant grows back at a random free spot in the camera view</t>
+  </si>
+  <si>
+    <t>US-130, US-132, US-134</t>
+  </si>
+  <si>
+    <t>Random numbers from a seeded stream; spatial queries</t>
+  </si>
+  <si>
+    <t>US-137</t>
+  </si>
+  <si>
+    <t>Animals in the Editor</t>
+  </si>
+  <si>
+    <t>As a level designer, I want to place animals, so that my levels have wildlife and dangers.</t>
+  </si>
+  <si>
+    <t>Scenario: Enemies
+Given a predator or boar
+When the hero hits it
+Then it takes damage and strikes back like a goblin
+Scenario: Bystanders
+Given a deer, cow or rabbit
+When the hero walks by
+Then it does nothing and cannot be hit</t>
+  </si>
+  <si>
+    <t>US-130, US-131</t>
+  </si>
+  <si>
+    <t>Data-driven behaviour flags</t>
+  </si>
+  <si>
+    <t>US-138</t>
+  </si>
+  <si>
+    <t>Placed effects and random weather</t>
+  </si>
+  <si>
+    <t>As the owner, I want ambient effects and changing weather, so that the world has atmosphere.</t>
+  </si>
+  <si>
+    <t>Scenario: Weather
+Given Game mode
+When 60-120 s pass
+Then a random weather fades in over 3 s; clear sky comes about 1 in 3
+Scenario: Repeatable
+Given the same seed
+When the game runs twice
+Then the same weathers come in the same order</t>
+  </si>
+  <si>
+    <t>D-21, ADR-011</t>
+  </si>
+  <si>
+    <t>Blending two overlays with alpha</t>
+  </si>
+  <si>
+    <t>Content and combat</t>
+  </si>
+  <si>
+    <t>The owner's weapons, plants, animals, effects and weather are in the game and playable.</t>
+  </si>
+  <si>
+    <t>Content and combat (weapons, nature, effects, weather)</t>
+  </si>
+  <si>
+    <t>The hero fights with 16 starter weapons of 8 classes and elements; enemies strike back; plants block, are chopped and eaten and regrow; animals and effects are placed in the Editor; the weather changes by itself.</t>
+  </si>
+  <si>
+    <t>M2d content and combat: full gameplay; 16 starter weapons as pickups with a 9-slot hotbar; 8 weapon classes; elements; hero 100 HP; enemies strike back within 1.5 m after 0.5 s; plants block, chop, heal 10, regrow in 15 s in camera view; predators and boars are enemies; effects; random weather every 60-120 s</t>
+  </si>
+  <si>
+    <t>US-130..US-138</t>
+  </si>
+  <si>
+    <t>D-22</t>
+  </si>
+  <si>
+    <t>Design decisions are taken by the owner in interactive question rounds in chat; Dominus no longer delegates design or scope questions</t>
+  </si>
+  <si>
+    <t>Process decision</t>
+  </si>
+  <si>
+    <t>all</t>
   </si>
 </sst>
 </file>
@@ -3022,7 +3283,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3072,6 +3333,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="16" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3994,7 +4258,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:CQ22"/>
+  <dimension ref="A1:CQ23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -4329,22 +4593,22 @@
         <v>4</v>
       </c>
       <c r="F7" s="9">
-        <f t="shared" ref="F7:F16" si="0">ROUND((D7+E7)/2,0)</f>
+        <f t="shared" ref="F7:F17" si="0">ROUND((D7+E7)/2,0)</f>
         <v>3</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>134</v>
       </c>
       <c r="H7" s="9">
-        <f t="shared" ref="H7:H16" si="1">G7+F7-1</f>
+        <f t="shared" ref="H7:H17" si="1">G7+F7-1</f>
         <v>3</v>
       </c>
       <c r="I7" s="14">
-        <f t="shared" ref="I7:I16" si="2">$B$4+(G7-1)*7</f>
+        <f t="shared" ref="I7:I17" si="2">$B$4+(G7-1)*7</f>
         <v>46300</v>
       </c>
       <c r="J7" s="14">
-        <f t="shared" ref="J7:J16" si="3">$B$4+H7*7-1</f>
+        <f t="shared" ref="J7:J17" si="3">$B$4+H7*7-1</f>
         <v>46320</v>
       </c>
       <c r="K7" s="14">
@@ -4356,7 +4620,7 @@
         <v>46327</v>
       </c>
       <c r="M7" s="9" t="str">
-        <f>SUMIFS('User Stories'!$H$5:$H$66,'User Stories'!$J$5:$J$66,A7,'User Stories'!$F$5:$F$66,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$66,'User Stories'!$J$5:$J$66,A7,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$75,'User Stories'!$J$5:$J$75,A7,'User Stories'!$F$5:$F$75,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$75,'User Stories'!$J$5:$J$75,A7,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>2 - 4</v>
       </c>
       <c r="N7" s="9" t="s">
@@ -4384,7 +4648,7 @@
         <v>7</v>
       </c>
       <c r="G8" s="9">
-        <f t="shared" ref="G8:G16" si="4">H7+1</f>
+        <f t="shared" ref="G8:G17" si="4">H7+1</f>
         <v>4</v>
       </c>
       <c r="H8" s="9">
@@ -4408,7 +4672,7 @@
         <v>46390</v>
       </c>
       <c r="M8" s="9" t="str">
-        <f>SUMIFS('User Stories'!$H$5:$H$66,'User Stories'!$J$5:$J$66,A8,'User Stories'!$F$5:$F$66,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$66,'User Stories'!$J$5:$J$66,A8,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$75,'User Stories'!$J$5:$J$75,A8,'User Stories'!$F$5:$F$75,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$75,'User Stories'!$J$5:$J$75,A8,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>4.5 - 9</v>
       </c>
       <c r="N8" s="9" t="s">
@@ -4460,7 +4724,7 @@
         <v>46474</v>
       </c>
       <c r="M9" s="9" t="str">
-        <f>SUMIFS('User Stories'!$H$5:$H$66,'User Stories'!$J$5:$J$66,A9,'User Stories'!$F$5:$F$66,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$66,'User Stories'!$J$5:$J$66,A9,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$75,'User Stories'!$J$5:$J$75,A9,'User Stories'!$F$5:$F$75,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$75,'User Stories'!$J$5:$J$75,A9,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>6 - 12</v>
       </c>
       <c r="N9" s="9" t="s">
@@ -4512,7 +4776,7 @@
         <v>46579</v>
       </c>
       <c r="M10" s="9" t="str">
-        <f>SUMIFS('User Stories'!$H$5:$H$66,'User Stories'!$J$5:$J$66,A10,'User Stories'!$F$5:$F$66,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$66,'User Stories'!$J$5:$J$66,A10,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$75,'User Stories'!$J$5:$J$75,A10,'User Stories'!$F$5:$F$75,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$75,'User Stories'!$J$5:$J$75,A10,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>7.5 - 15</v>
       </c>
       <c r="N10" s="9" t="s">
@@ -4564,7 +4828,7 @@
         <v>46719</v>
       </c>
       <c r="M11" s="9" t="str">
-        <f>SUMIFS('User Stories'!$H$5:$H$66,'User Stories'!$J$5:$J$66,A11,'User Stories'!$F$5:$F$66,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$66,'User Stories'!$J$5:$J$66,A11,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$75,'User Stories'!$J$5:$J$75,A11,'User Stories'!$F$5:$F$75,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$75,'User Stories'!$J$5:$J$75,A11,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>10 - 20</v>
       </c>
       <c r="N11" s="9" t="s">
@@ -4616,7 +4880,7 @@
         <v>46775</v>
       </c>
       <c r="M12" s="9" t="str">
-        <f>SUMIFS('User Stories'!$H$5:$H$66,'User Stories'!$J$5:$J$66,A12,'User Stories'!$F$5:$F$66,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$66,'User Stories'!$J$5:$J$66,A12,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>SUMIFS('User Stories'!$H$5:$H$75,'User Stories'!$J$5:$J$75,A12,'User Stories'!$F$5:$F$75,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$75,'User Stories'!$J$5:$J$75,A12,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>7 - 14</v>
       </c>
       <c r="N12" s="9" t="s">
@@ -4625,302 +4889,337 @@
     </row>
     <row r="13" spans="1:95" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
+        <v>762</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>815</v>
+      </c>
+      <c r="C13" s="21">
+        <v>46024</v>
+      </c>
+      <c r="D13" s="13">
+        <v>4</v>
+      </c>
+      <c r="E13" s="13">
+        <v>9</v>
+      </c>
+      <c r="F13" s="9">
+        <f t="shared" ref="F13" si="9">ROUND((D13+E13)/2,0)</f>
+        <v>7</v>
+      </c>
+      <c r="G13" s="9">
+        <f t="shared" ref="G13" si="10">H12+1</f>
+        <v>53</v>
+      </c>
+      <c r="H13" s="9">
+        <f t="shared" ref="H13" si="11">G13+F13-1</f>
+        <v>59</v>
+      </c>
+      <c r="I13" s="14">
+        <f t="shared" ref="I13" si="12">$B$4+(G13-1)*7</f>
+        <v>46664</v>
+      </c>
+      <c r="J13" s="14">
+        <f t="shared" ref="J13" si="13">$B$4+H13*7-1</f>
+        <v>46712</v>
+      </c>
+      <c r="K13" s="14">
+        <f>$B$4+SUM($D$7:D13)*7-1</f>
+        <v>46565</v>
+      </c>
+      <c r="L13" s="14">
+        <f>$B$4+SUM($E$7:E13)*7-1</f>
+        <v>46838</v>
+      </c>
+      <c r="M13" s="9" t="str">
+        <f>SUMIFS('User Stories'!$H$5:$H$75,'User Stories'!$J$5:$J$75,A13,'User Stories'!$F$5:$F$75,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$75,'User Stories'!$J$5:$J$75,A13,'User Stories'!$F$5:$F$75,"Must")</f>
+        <v>9.5 - 19</v>
+      </c>
+      <c r="N13" s="9" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="14" spans="1:95" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B14" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C14" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="D13" s="13">
+      <c r="D14" s="13">
         <v>3</v>
       </c>
-      <c r="E13" s="13">
+      <c r="E14" s="13">
         <v>6</v>
       </c>
-      <c r="F13" s="9">
+      <c r="F14" s="9">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="G13" s="9">
-        <f>H12+1</f>
-        <v>53</v>
-      </c>
-      <c r="H13" s="9">
+      <c r="G14" s="9">
+        <f>H13+1</f>
+        <v>60</v>
+      </c>
+      <c r="H14" s="9">
         <f t="shared" si="1"/>
-        <v>57</v>
-      </c>
-      <c r="I13" s="14">
+        <v>64</v>
+      </c>
+      <c r="I14" s="14">
         <f t="shared" si="2"/>
-        <v>46664</v>
-      </c>
-      <c r="J13" s="14">
+        <v>46713</v>
+      </c>
+      <c r="J14" s="14">
         <f t="shared" si="3"/>
-        <v>46698</v>
-      </c>
-      <c r="K13" s="14">
-        <f>$B$4+SUM($D$7:D13)*7-1</f>
-        <v>46558</v>
-      </c>
-      <c r="L13" s="14">
-        <f>$B$4+SUM($E$7:E13)*7-1</f>
-        <v>46817</v>
-      </c>
-      <c r="M13" s="9" t="str">
-        <f>SUMIFS('User Stories'!$H$5:$H$66,'User Stories'!$J$5:$J$66,A13,'User Stories'!$F$5:$F$66,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$66,'User Stories'!$J$5:$J$66,A13,'User Stories'!$F$5:$F$66,"Must")</f>
+        <v>46747</v>
+      </c>
+      <c r="K14" s="14">
+        <f>$B$4+SUM($D$7:D14)*7-1</f>
+        <v>46586</v>
+      </c>
+      <c r="L14" s="14">
+        <f>$B$4+SUM($E$7:E14)*7-1</f>
+        <v>46880</v>
+      </c>
+      <c r="M14" s="9" t="str">
+        <f>SUMIFS('User Stories'!$H$5:$H$75,'User Stories'!$J$5:$J$75,A14,'User Stories'!$F$5:$F$75,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$75,'User Stories'!$J$5:$J$75,A14,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>3 - 6</v>
       </c>
-      <c r="N13" s="9" t="s">
+      <c r="N14" s="9" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="14" spans="1:95" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
+    <row r="15" spans="1:95" ht="42" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B15" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C15" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="D14" s="13">
+      <c r="D15" s="13">
         <v>5</v>
       </c>
-      <c r="E14" s="13">
+      <c r="E15" s="13">
         <v>10</v>
       </c>
-      <c r="F14" s="9">
+      <c r="F15" s="9">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G15" s="9">
         <f t="shared" si="4"/>
-        <v>58</v>
-      </c>
-      <c r="H14" s="9">
+        <v>65</v>
+      </c>
+      <c r="H15" s="9">
         <f t="shared" si="1"/>
-        <v>65</v>
-      </c>
-      <c r="I14" s="14">
+        <v>72</v>
+      </c>
+      <c r="I15" s="14">
         <f t="shared" si="2"/>
-        <v>46699</v>
-      </c>
-      <c r="J14" s="14">
+        <v>46748</v>
+      </c>
+      <c r="J15" s="14">
         <f t="shared" si="3"/>
-        <v>46754</v>
-      </c>
-      <c r="K14" s="14">
-        <f>$B$4+SUM($D$7:D14)*7-1</f>
-        <v>46593</v>
-      </c>
-      <c r="L14" s="14">
-        <f>$B$4+SUM($E$7:E14)*7-1</f>
-        <v>46887</v>
-      </c>
-      <c r="M14" s="9" t="str">
-        <f>SUMIFS('User Stories'!$H$5:$H$66,'User Stories'!$J$5:$J$66,A14,'User Stories'!$F$5:$F$66,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$66,'User Stories'!$J$5:$J$66,A14,'User Stories'!$F$5:$F$66,"Must")</f>
+        <v>46803</v>
+      </c>
+      <c r="K15" s="14">
+        <f>$B$4+SUM($D$7:D15)*7-1</f>
+        <v>46621</v>
+      </c>
+      <c r="L15" s="14">
+        <f>$B$4+SUM($E$7:E15)*7-1</f>
+        <v>46950</v>
+      </c>
+      <c r="M15" s="9" t="str">
+        <f>SUMIFS('User Stories'!$H$5:$H$75,'User Stories'!$J$5:$J$75,A15,'User Stories'!$F$5:$F$75,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$75,'User Stories'!$J$5:$J$75,A15,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>5 - 10</v>
       </c>
-      <c r="N14" s="9" t="s">
+      <c r="N15" s="9" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="15" spans="1:95" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
+    <row r="16" spans="1:95" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B16" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C16" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="D15" s="13">
+      <c r="D16" s="13">
         <v>16</v>
       </c>
-      <c r="E15" s="13">
+      <c r="E16" s="13">
         <v>31</v>
       </c>
-      <c r="F15" s="9">
+      <c r="F16" s="9">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="G15" s="9">
+      <c r="G16" s="9">
         <f t="shared" si="4"/>
-        <v>66</v>
-      </c>
-      <c r="H15" s="9">
+        <v>73</v>
+      </c>
+      <c r="H16" s="9">
         <f t="shared" si="1"/>
-        <v>89</v>
-      </c>
-      <c r="I15" s="14">
+        <v>96</v>
+      </c>
+      <c r="I16" s="14">
         <f t="shared" si="2"/>
-        <v>46755</v>
-      </c>
-      <c r="J15" s="14">
+        <v>46804</v>
+      </c>
+      <c r="J16" s="14">
         <f t="shared" si="3"/>
-        <v>46922</v>
-      </c>
-      <c r="K15" s="14">
-        <f>$B$4+SUM($D$7:D15)*7-1</f>
-        <v>46705</v>
-      </c>
-      <c r="L15" s="14">
-        <f>$B$4+SUM($E$7:E15)*7-1</f>
-        <v>47104</v>
-      </c>
-      <c r="M15" s="9" t="str">
-        <f>SUMIFS('User Stories'!$H$5:$H$66,'User Stories'!$J$5:$J$66,A15,'User Stories'!$F$5:$F$66,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$66,'User Stories'!$J$5:$J$66,A15,'User Stories'!$F$5:$F$66,"Must")</f>
+        <v>46971</v>
+      </c>
+      <c r="K16" s="14">
+        <f>$B$4+SUM($D$7:D16)*7-1</f>
+        <v>46733</v>
+      </c>
+      <c r="L16" s="14">
+        <f>$B$4+SUM($E$7:E16)*7-1</f>
+        <v>47167</v>
+      </c>
+      <c r="M16" s="9" t="str">
+        <f>SUMIFS('User Stories'!$H$5:$H$75,'User Stories'!$J$5:$J$75,A16,'User Stories'!$F$5:$F$75,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$75,'User Stories'!$J$5:$J$75,A16,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>15.5 - 31</v>
       </c>
-      <c r="N15" s="9" t="s">
+      <c r="N16" s="9" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="16" spans="1:95" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
+    <row r="17" spans="1:14" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="B17" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C17" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="D16" s="13">
+      <c r="D17" s="13">
         <v>3</v>
       </c>
-      <c r="E16" s="13">
+      <c r="E17" s="13">
         <v>4</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F17" s="9">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="G16" s="9">
+      <c r="G17" s="9">
         <f t="shared" si="4"/>
-        <v>90</v>
-      </c>
-      <c r="H16" s="9">
+        <v>97</v>
+      </c>
+      <c r="H17" s="9">
         <f t="shared" si="1"/>
-        <v>93</v>
-      </c>
-      <c r="I16" s="14">
+        <v>100</v>
+      </c>
+      <c r="I17" s="14">
         <f t="shared" si="2"/>
-        <v>46923</v>
-      </c>
-      <c r="J16" s="14">
+        <v>46972</v>
+      </c>
+      <c r="J17" s="14">
         <f t="shared" si="3"/>
-        <v>46950</v>
-      </c>
-      <c r="K16" s="14">
-        <f>$B$4+SUM($D$7:D16)*7-1</f>
-        <v>46726</v>
-      </c>
-      <c r="L16" s="14">
-        <f>$B$4+SUM($E$7:E16)*7-1</f>
-        <v>47132</v>
-      </c>
-      <c r="M16" s="9" t="str">
-        <f>SUMIFS('User Stories'!$H$5:$H$66,'User Stories'!$J$5:$J$66,A16,'User Stories'!$F$5:$F$66,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$66,'User Stories'!$J$5:$J$66,A16,'User Stories'!$F$5:$F$66,"Must")</f>
+        <v>46999</v>
+      </c>
+      <c r="K17" s="14">
+        <f>$B$4+SUM($D$7:D17)*7-1</f>
+        <v>46754</v>
+      </c>
+      <c r="L17" s="14">
+        <f>$B$4+SUM($E$7:E17)*7-1</f>
+        <v>47195</v>
+      </c>
+      <c r="M17" s="9" t="str">
+        <f>SUMIFS('User Stories'!$H$5:$H$75,'User Stories'!$J$5:$J$75,A17,'User Stories'!$F$5:$F$75,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$75,'User Stories'!$J$5:$J$75,A17,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>0.5 - 1</v>
       </c>
-      <c r="N16" s="9" t="s">
+      <c r="N17" s="9" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7" t="s">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" s="7"/>
+      <c r="B18" s="7" t="s">
         <v>165</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7">
-        <f>SUM(D7:D16)</f>
-        <v>61</v>
-      </c>
-      <c r="E17" s="7">
-        <f>SUM(E7:E16)</f>
-        <v>119</v>
-      </c>
-      <c r="F17" s="7">
-        <f>SUM(F7:F16)</f>
-        <v>93</v>
-      </c>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7">
-        <f>H16</f>
-        <v>93</v>
-      </c>
-      <c r="I17" s="15">
+      <c r="C18" s="7"/>
+      <c r="D18" s="7">
+        <f>SUM(D7:D17)</f>
+        <v>65</v>
+      </c>
+      <c r="E18" s="7">
+        <f>SUM(E7:E17)</f>
+        <v>128</v>
+      </c>
+      <c r="F18" s="7">
+        <f>SUM(F7:F17)</f>
+        <v>100</v>
+      </c>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7">
+        <f>H17</f>
+        <v>100</v>
+      </c>
+      <c r="I18" s="15">
         <f>I7</f>
         <v>46300</v>
       </c>
-      <c r="J17" s="15">
-        <f>J16</f>
-        <v>46950</v>
-      </c>
-      <c r="K17" s="15">
-        <f>K16</f>
-        <v>46726</v>
-      </c>
-      <c r="L17" s="15">
-        <f>L16</f>
-        <v>47132</v>
-      </c>
-      <c r="M17" s="7"/>
-      <c r="N17" s="7" t="s">
+      <c r="J18" s="15">
+        <f>J17</f>
+        <v>46999</v>
+      </c>
+      <c r="K18" s="15">
+        <f>K17</f>
+        <v>46754</v>
+      </c>
+      <c r="L18" s="15">
+        <f>L17</f>
+        <v>47195</v>
+      </c>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7" t="s">
+    <row r="19" spans="1:14" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="7"/>
+      <c r="B19" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7">
-        <f>ROUND(D17/4.33,1)</f>
-        <v>14.1</v>
-      </c>
-      <c r="E18" s="7">
-        <f>ROUND(E17/4.33,1)</f>
-        <v>27.5</v>
-      </c>
-      <c r="F18" s="7">
-        <f>ROUND(F17/4.33,1)</f>
-        <v>21.5</v>
-      </c>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
-      <c r="I18" s="7"/>
-      <c r="J18" s="7"/>
-      <c r="K18" s="7"/>
-      <c r="L18" s="7"/>
-      <c r="M18" s="7"/>
-      <c r="N18" s="7"/>
-    </row>
-    <row r="19" spans="1:14" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
-      <c r="J19" s="20"/>
-      <c r="K19" s="20"/>
-      <c r="L19" s="20"/>
-      <c r="M19" s="20"/>
-      <c r="N19" s="20"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7">
+        <f>ROUND(D18/4.33,1)</f>
+        <v>15</v>
+      </c>
+      <c r="E19" s="7">
+        <f>ROUND(E18/4.33,1)</f>
+        <v>29.6</v>
+      </c>
+      <c r="F19" s="7">
+        <f>ROUND(F18/4.33,1)</f>
+        <v>23.1</v>
+      </c>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="7"/>
+      <c r="M19" s="7"/>
+      <c r="N19" s="7"/>
     </row>
     <row r="20" spans="1:14" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="19" t="s">
-        <v>168</v>
-      </c>
+      <c r="B20" s="20"/>
       <c r="C20" s="20"/>
       <c r="D20" s="20"/>
       <c r="E20" s="20"/>
@@ -4934,9 +5233,9 @@
       <c r="M20" s="20"/>
       <c r="N20" s="20"/>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="19" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C21" s="20"/>
       <c r="D21" s="20"/>
@@ -4951,18 +5250,35 @@
       <c r="M21" s="20"/>
       <c r="N21" s="20"/>
     </row>
-    <row r="22" spans="1:14" ht="102" x14ac:dyDescent="0.25">
-      <c r="B22" s="4" t="s">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B22" s="19" t="s">
+        <v>169</v>
+      </c>
+      <c r="C22" s="20"/>
+      <c r="D22" s="20"/>
+      <c r="E22" s="20"/>
+      <c r="F22" s="20"/>
+      <c r="G22" s="20"/>
+      <c r="H22" s="20"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="20"/>
+      <c r="K22" s="20"/>
+      <c r="L22" s="20"/>
+      <c r="M22" s="20"/>
+      <c r="N22" s="20"/>
+    </row>
+    <row r="23" spans="1:14" ht="102" x14ac:dyDescent="0.25">
+      <c r="B23" s="4" t="s">
         <v>170</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="B21:N21"/>
+    <mergeCell ref="B22:N22"/>
     <mergeCell ref="B20:N20"/>
-    <mergeCell ref="B21:N21"/>
-    <mergeCell ref="B19:N19"/>
   </mergeCells>
-  <conditionalFormatting sqref="P7:CQ16">
+  <conditionalFormatting sqref="P7:CQ17">
     <cfRule type="expression" dxfId="10" priority="1">
       <formula>AND(P$6&gt;=$G7,P$6&lt;=$H7)</formula>
     </cfRule>
@@ -4973,7 +5289,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -5452,6 +5768,52 @@
         <v>177</v>
       </c>
       <c r="G23" s="16" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
+        <v>770</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>817</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>762</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>818</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="G24" s="16" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
+        <v>819</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>820</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>821</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>822</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>822</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="G25" s="16" t="s">
         <v>77</v>
       </c>
     </row>
@@ -5481,7 +5843,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -5551,27 +5913,27 @@
         <v>131</v>
       </c>
       <c r="E5" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$66,A5)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$75,A5)</f>
         <v>4</v>
       </c>
       <c r="F5" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A5,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A5,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>4</v>
       </c>
       <c r="G5" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A5,'User Stories'!$H$5:$H$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A5,'User Stories'!$H$5:$H$75)</f>
         <v>2</v>
       </c>
       <c r="H5" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A5,'User Stories'!$I$5:$I$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A5,'User Stories'!$I$5:$I$75)</f>
         <v>4</v>
       </c>
       <c r="I5" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A5,'User Stories'!$O$5:$O$66,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A5,'User Stories'!$O$5:$O$75,"Done")</f>
         <v>2</v>
       </c>
       <c r="J5" s="17">
-        <f t="shared" ref="J5:J18" si="0">IFERROR(I5/E5,0)</f>
+        <f t="shared" ref="J5:J19" si="0">IFERROR(I5/E5,0)</f>
         <v>0.5</v>
       </c>
     </row>
@@ -5589,23 +5951,23 @@
         <v>144</v>
       </c>
       <c r="E6" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$66,A6)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$75,A6)</f>
         <v>7</v>
       </c>
       <c r="F6" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A6,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A6,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>7</v>
       </c>
       <c r="G6" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A6,'User Stories'!$H$5:$H$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A6,'User Stories'!$H$5:$H$75)</f>
         <v>7.5</v>
       </c>
       <c r="H6" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A6,'User Stories'!$I$5:$I$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A6,'User Stories'!$I$5:$I$75)</f>
         <v>15</v>
       </c>
       <c r="I6" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A6,'User Stories'!$O$5:$O$66,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A6,'User Stories'!$O$5:$O$75,"Done")</f>
         <v>0</v>
       </c>
       <c r="J6" s="17">
@@ -5627,23 +5989,23 @@
         <v>136</v>
       </c>
       <c r="E7" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$66,A7)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$75,A7)</f>
         <v>5</v>
       </c>
       <c r="F7" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A7,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A7,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>5</v>
       </c>
       <c r="G7" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A7,'User Stories'!$H$5:$H$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A7,'User Stories'!$H$5:$H$75)</f>
         <v>4.5</v>
       </c>
       <c r="H7" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A7,'User Stories'!$I$5:$I$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A7,'User Stories'!$I$5:$I$75)</f>
         <v>9</v>
       </c>
       <c r="I7" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A7,'User Stories'!$O$5:$O$66,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A7,'User Stories'!$O$5:$O$75,"Done")</f>
         <v>0</v>
       </c>
       <c r="J7" s="17">
@@ -5665,23 +6027,23 @@
         <v>151</v>
       </c>
       <c r="E8" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$66,A8)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$75,A8)</f>
         <v>3</v>
       </c>
       <c r="F8" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A8,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A8,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>2</v>
       </c>
       <c r="G8" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A8,'User Stories'!$H$5:$H$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A8,'User Stories'!$H$5:$H$75)</f>
         <v>3.5</v>
       </c>
       <c r="H8" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A8,'User Stories'!$I$5:$I$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A8,'User Stories'!$I$5:$I$75)</f>
         <v>7</v>
       </c>
       <c r="I8" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A8,'User Stories'!$O$5:$O$66,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A8,'User Stories'!$O$5:$O$75,"Done")</f>
         <v>0</v>
       </c>
       <c r="J8" s="17">
@@ -5703,23 +6065,23 @@
         <v>155</v>
       </c>
       <c r="E9" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$66,A9)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$75,A9)</f>
         <v>4</v>
       </c>
       <c r="F9" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A9,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A9,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>3</v>
       </c>
       <c r="G9" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A9,'User Stories'!$H$5:$H$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A9,'User Stories'!$H$5:$H$75)</f>
         <v>5</v>
       </c>
       <c r="H9" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A9,'User Stories'!$I$5:$I$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A9,'User Stories'!$I$5:$I$75)</f>
         <v>10</v>
       </c>
       <c r="I9" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A9,'User Stories'!$O$5:$O$66,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A9,'User Stories'!$O$5:$O$75,"Done")</f>
         <v>0</v>
       </c>
       <c r="J9" s="17">
@@ -5741,23 +6103,23 @@
         <v>102</v>
       </c>
       <c r="E10" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$66,A10)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$75,A10)</f>
         <v>6</v>
       </c>
       <c r="F10" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A10,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A10,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>6</v>
       </c>
       <c r="G10" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A10,'User Stories'!$H$5:$H$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A10,'User Stories'!$H$5:$H$75)</f>
         <v>6</v>
       </c>
       <c r="H10" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A10,'User Stories'!$I$5:$I$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A10,'User Stories'!$I$5:$I$75)</f>
         <v>12</v>
       </c>
       <c r="I10" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A10,'User Stories'!$O$5:$O$66,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A10,'User Stories'!$O$5:$O$75,"Done")</f>
         <v>0</v>
       </c>
       <c r="J10" s="17">
@@ -5779,23 +6141,23 @@
         <v>102</v>
       </c>
       <c r="E11" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$66,A11)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$75,A11)</f>
         <v>4</v>
       </c>
       <c r="F11" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A11,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A11,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>3</v>
       </c>
       <c r="G11" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A11,'User Stories'!$H$5:$H$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A11,'User Stories'!$H$5:$H$75)</f>
         <v>4.5</v>
       </c>
       <c r="H11" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A11,'User Stories'!$I$5:$I$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A11,'User Stories'!$I$5:$I$75)</f>
         <v>9</v>
       </c>
       <c r="I11" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A11,'User Stories'!$O$5:$O$66,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A11,'User Stories'!$O$5:$O$75,"Done")</f>
         <v>0</v>
       </c>
       <c r="J11" s="17">
@@ -5817,23 +6179,23 @@
         <v>102</v>
       </c>
       <c r="E12" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$66,A12)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$75,A12)</f>
         <v>4</v>
       </c>
       <c r="F12" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A12,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A12,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>4</v>
       </c>
       <c r="G12" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A12,'User Stories'!$H$5:$H$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A12,'User Stories'!$H$5:$H$75)</f>
         <v>5.5</v>
       </c>
       <c r="H12" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A12,'User Stories'!$I$5:$I$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A12,'User Stories'!$I$5:$I$75)</f>
         <v>11</v>
       </c>
       <c r="I12" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A12,'User Stories'!$O$5:$O$66,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A12,'User Stories'!$O$5:$O$75,"Done")</f>
         <v>0</v>
       </c>
       <c r="J12" s="17">
@@ -5855,23 +6217,23 @@
         <v>280</v>
       </c>
       <c r="E13" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$66,A13)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$75,A13)</f>
         <v>4</v>
       </c>
       <c r="F13" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A13,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A13,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>2</v>
       </c>
       <c r="G13" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A13,'User Stories'!$H$5:$H$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A13,'User Stories'!$H$5:$H$75)</f>
         <v>3</v>
       </c>
       <c r="H13" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A13,'User Stories'!$I$5:$I$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A13,'User Stories'!$I$5:$I$75)</f>
         <v>6</v>
       </c>
       <c r="I13" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A13,'User Stories'!$O$5:$O$66,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A13,'User Stories'!$O$5:$O$75,"Done")</f>
         <v>0</v>
       </c>
       <c r="J13" s="17">
@@ -5893,23 +6255,23 @@
         <v>91</v>
       </c>
       <c r="E14" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$66,A14)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$75,A14)</f>
         <v>3</v>
       </c>
       <c r="F14" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A14,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A14,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>1</v>
       </c>
       <c r="G14" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A14,'User Stories'!$H$5:$H$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A14,'User Stories'!$H$5:$H$75)</f>
         <v>2</v>
       </c>
       <c r="H14" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A14,'User Stories'!$I$5:$I$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A14,'User Stories'!$I$5:$I$75)</f>
         <v>4</v>
       </c>
       <c r="I14" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A14,'User Stories'!$O$5:$O$66,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A14,'User Stories'!$O$5:$O$75,"Done")</f>
         <v>0</v>
       </c>
       <c r="J14" s="17">
@@ -5931,23 +6293,23 @@
         <v>140</v>
       </c>
       <c r="E15" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$66,A15)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$75,A15)</f>
         <v>5</v>
       </c>
       <c r="F15" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A15,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A15,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>5</v>
       </c>
       <c r="G15" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A15,'User Stories'!$H$5:$H$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A15,'User Stories'!$H$5:$H$75)</f>
         <v>6</v>
       </c>
       <c r="H15" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A15,'User Stories'!$I$5:$I$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A15,'User Stories'!$I$5:$I$75)</f>
         <v>12</v>
       </c>
       <c r="I15" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A15,'User Stories'!$O$5:$O$66,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A15,'User Stories'!$O$5:$O$75,"Done")</f>
         <v>0</v>
       </c>
       <c r="J15" s="17">
@@ -5969,23 +6331,23 @@
         <v>148</v>
       </c>
       <c r="E16" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$66,A16)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$75,A16)</f>
         <v>6</v>
       </c>
       <c r="F16" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A16,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A16,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>6</v>
       </c>
       <c r="G16" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A16,'User Stories'!$H$5:$H$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A16,'User Stories'!$H$5:$H$75)</f>
         <v>10</v>
       </c>
       <c r="H16" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A16,'User Stories'!$I$5:$I$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A16,'User Stories'!$I$5:$I$75)</f>
         <v>20</v>
       </c>
       <c r="I16" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A16,'User Stories'!$O$5:$O$66,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A16,'User Stories'!$O$5:$O$75,"Done")</f>
         <v>0</v>
       </c>
       <c r="J16" s="17">
@@ -6007,23 +6369,23 @@
         <v>710</v>
       </c>
       <c r="E17" s="9">
-        <f>COUNTIF('User Stories'!$B$5:$B$66,A17)</f>
+        <f>COUNTIF('User Stories'!$B$5:$B$75,A17)</f>
         <v>7</v>
       </c>
       <c r="F17" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A17,'User Stories'!$F$5:$F$66,"Must")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A17,'User Stories'!$F$5:$F$75,"Must")</f>
         <v>7</v>
       </c>
       <c r="G17" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A17,'User Stories'!$H$5:$H$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A17,'User Stories'!$H$5:$H$75)</f>
         <v>7</v>
       </c>
       <c r="H17" s="9">
-        <f>SUMIF('User Stories'!$B$5:$B$66,A17,'User Stories'!$I$5:$I$66)</f>
+        <f>SUMIF('User Stories'!$B$5:$B$75,A17,'User Stories'!$I$5:$I$75)</f>
         <v>14</v>
       </c>
       <c r="I17" s="9">
-        <f>COUNTIFS('User Stories'!$B$5:$B$66,A17,'User Stories'!$O$5:$O$66,"Done")</f>
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A17,'User Stories'!$O$5:$O$75,"Done")</f>
         <v>0</v>
       </c>
       <c r="J17" s="17">
@@ -6031,36 +6393,74 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7" t="s">
+    <row r="18" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>758</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>813</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>814</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>762</v>
+      </c>
+      <c r="E18" s="9">
+        <f>COUNTIF('User Stories'!$B$5:$B$75,A18)</f>
+        <v>9</v>
+      </c>
+      <c r="F18" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A18,'User Stories'!$F$5:$F$75,"Must")</f>
+        <v>7</v>
+      </c>
+      <c r="G18" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$75,A18,'User Stories'!$H$5:$H$75)</f>
+        <v>11</v>
+      </c>
+      <c r="H18" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$75,A18,'User Stories'!$I$5:$I$75)</f>
+        <v>22</v>
+      </c>
+      <c r="I18" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$75,A18,'User Stories'!$O$5:$O$75,"Done")</f>
+        <v>0</v>
+      </c>
+      <c r="J18" s="17">
+        <f t="shared" ref="J18" si="2">IFERROR(I18/E18,0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="7"/>
+      <c r="B19" s="7" t="s">
         <v>290</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7">
-        <f>SUM(E5:E17)</f>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7">
+        <f>SUM(E5:E18)</f>
+        <v>71</v>
+      </c>
+      <c r="F19" s="7">
+        <f>SUM(F5:F18)</f>
         <v>62</v>
       </c>
-      <c r="F18" s="7">
-        <f>SUM(F5:F17)</f>
-        <v>55</v>
-      </c>
-      <c r="G18" s="7">
-        <f>SUM(G5:G17)</f>
-        <v>66.5</v>
-      </c>
-      <c r="H18" s="7">
-        <f>SUM(H5:H17)</f>
-        <v>133</v>
-      </c>
-      <c r="I18" s="7">
-        <f>SUM(I5:I17)</f>
+      <c r="G19" s="7">
+        <f>SUM(G5:G18)</f>
+        <v>77.5</v>
+      </c>
+      <c r="H19" s="7">
+        <f>SUM(H5:H18)</f>
+        <v>155</v>
+      </c>
+      <c r="I19" s="7">
+        <f>SUM(I5:I18)</f>
         <v>2</v>
       </c>
-      <c r="J18" s="18">
+      <c r="J19" s="18">
         <f t="shared" si="0"/>
-        <v>3.2258064516129031E-2</v>
+        <v>2.8169014084507043E-2</v>
       </c>
     </row>
   </sheetData>
@@ -6070,7 +6470,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:O66"/>
+  <dimension ref="A1:O75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -9074,9 +9474,432 @@
         <v>319</v>
       </c>
     </row>
+    <row r="67" spans="1:15" ht="124.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="7" t="s">
+        <v>757</v>
+      </c>
+      <c r="B67" s="9" t="s">
+        <v>758</v>
+      </c>
+      <c r="C67" s="9" t="s">
+        <v>759</v>
+      </c>
+      <c r="D67" s="9" t="s">
+        <v>760</v>
+      </c>
+      <c r="E67" s="9" t="s">
+        <v>761</v>
+      </c>
+      <c r="F67" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="G67" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H67" s="9">
+        <v>2</v>
+      </c>
+      <c r="I67" s="9">
+        <v>4</v>
+      </c>
+      <c r="J67" s="9" t="s">
+        <v>762</v>
+      </c>
+      <c r="K67" s="9" t="s">
+        <v>705</v>
+      </c>
+      <c r="L67" s="9" t="s">
+        <v>763</v>
+      </c>
+      <c r="M67" s="9" t="s">
+        <v>764</v>
+      </c>
+      <c r="N67" s="9" t="s">
+        <v>765</v>
+      </c>
+      <c r="O67" s="16" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="68" spans="1:15" ht="124.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A68" s="7" t="s">
+        <v>766</v>
+      </c>
+      <c r="B68" s="9" t="s">
+        <v>758</v>
+      </c>
+      <c r="C68" s="9" t="s">
+        <v>767</v>
+      </c>
+      <c r="D68" s="9" t="s">
+        <v>768</v>
+      </c>
+      <c r="E68" s="9" t="s">
+        <v>769</v>
+      </c>
+      <c r="F68" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="G68" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H68" s="9">
+        <v>1</v>
+      </c>
+      <c r="I68" s="9">
+        <v>2</v>
+      </c>
+      <c r="J68" s="9" t="s">
+        <v>762</v>
+      </c>
+      <c r="K68" s="9" t="s">
+        <v>738</v>
+      </c>
+      <c r="L68" s="9" t="s">
+        <v>770</v>
+      </c>
+      <c r="M68" s="9" t="s">
+        <v>771</v>
+      </c>
+      <c r="N68" s="9" t="s">
+        <v>765</v>
+      </c>
+      <c r="O68" s="16" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15" ht="124.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A69" s="7" t="s">
+        <v>772</v>
+      </c>
+      <c r="B69" s="9" t="s">
+        <v>758</v>
+      </c>
+      <c r="C69" s="9" t="s">
+        <v>773</v>
+      </c>
+      <c r="D69" s="9" t="s">
+        <v>774</v>
+      </c>
+      <c r="E69" s="9" t="s">
+        <v>775</v>
+      </c>
+      <c r="F69" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="G69" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H69" s="9">
+        <v>1</v>
+      </c>
+      <c r="I69" s="9">
+        <v>2</v>
+      </c>
+      <c r="J69" s="9" t="s">
+        <v>762</v>
+      </c>
+      <c r="K69" s="9" t="s">
+        <v>757</v>
+      </c>
+      <c r="L69" s="9" t="s">
+        <v>776</v>
+      </c>
+      <c r="M69" s="9" t="s">
+        <v>777</v>
+      </c>
+      <c r="N69" s="9" t="s">
+        <v>765</v>
+      </c>
+      <c r="O69" s="16" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" ht="124.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A70" s="7" t="s">
+        <v>778</v>
+      </c>
+      <c r="B70" s="9" t="s">
+        <v>758</v>
+      </c>
+      <c r="C70" s="9" t="s">
+        <v>779</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>780</v>
+      </c>
+      <c r="E70" s="9" t="s">
+        <v>781</v>
+      </c>
+      <c r="F70" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="G70" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H70" s="9">
+        <v>2</v>
+      </c>
+      <c r="I70" s="9">
+        <v>4</v>
+      </c>
+      <c r="J70" s="9" t="s">
+        <v>762</v>
+      </c>
+      <c r="K70" s="9" t="s">
+        <v>782</v>
+      </c>
+      <c r="L70" s="9" t="s">
+        <v>770</v>
+      </c>
+      <c r="M70" s="9" t="s">
+        <v>783</v>
+      </c>
+      <c r="N70" s="9" t="s">
+        <v>765</v>
+      </c>
+      <c r="O70" s="16" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" ht="124.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A71" s="7" t="s">
+        <v>784</v>
+      </c>
+      <c r="B71" s="9" t="s">
+        <v>758</v>
+      </c>
+      <c r="C71" s="9" t="s">
+        <v>785</v>
+      </c>
+      <c r="D71" s="9" t="s">
+        <v>786</v>
+      </c>
+      <c r="E71" s="9" t="s">
+        <v>787</v>
+      </c>
+      <c r="F71" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="G71" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H71" s="9">
+        <v>1</v>
+      </c>
+      <c r="I71" s="9">
+        <v>2</v>
+      </c>
+      <c r="J71" s="9" t="s">
+        <v>762</v>
+      </c>
+      <c r="K71" s="9" t="s">
+        <v>778</v>
+      </c>
+      <c r="L71" s="9" t="s">
+        <v>788</v>
+      </c>
+      <c r="M71" s="9" t="s">
+        <v>789</v>
+      </c>
+      <c r="N71" s="9" t="s">
+        <v>765</v>
+      </c>
+      <c r="O71" s="16" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="72" spans="1:15" ht="124.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A72" s="7" t="s">
+        <v>790</v>
+      </c>
+      <c r="B72" s="9" t="s">
+        <v>758</v>
+      </c>
+      <c r="C72" s="9" t="s">
+        <v>791</v>
+      </c>
+      <c r="D72" s="9" t="s">
+        <v>792</v>
+      </c>
+      <c r="E72" s="9" t="s">
+        <v>793</v>
+      </c>
+      <c r="F72" s="9" t="s">
+        <v>415</v>
+      </c>
+      <c r="G72" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H72" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="I72" s="9">
+        <v>1</v>
+      </c>
+      <c r="J72" s="9" t="s">
+        <v>762</v>
+      </c>
+      <c r="K72" s="9" t="s">
+        <v>778</v>
+      </c>
+      <c r="L72" s="9" t="s">
+        <v>770</v>
+      </c>
+      <c r="M72" s="9" t="s">
+        <v>794</v>
+      </c>
+      <c r="N72" s="9" t="s">
+        <v>765</v>
+      </c>
+      <c r="O72" s="16" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="73" spans="1:15" ht="124.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="7" t="s">
+        <v>795</v>
+      </c>
+      <c r="B73" s="9" t="s">
+        <v>758</v>
+      </c>
+      <c r="C73" s="9" t="s">
+        <v>796</v>
+      </c>
+      <c r="D73" s="9" t="s">
+        <v>797</v>
+      </c>
+      <c r="E73" s="9" t="s">
+        <v>798</v>
+      </c>
+      <c r="F73" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="G73" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H73" s="9">
+        <v>2</v>
+      </c>
+      <c r="I73" s="9">
+        <v>4</v>
+      </c>
+      <c r="J73" s="9" t="s">
+        <v>762</v>
+      </c>
+      <c r="K73" s="9" t="s">
+        <v>799</v>
+      </c>
+      <c r="L73" s="9" t="s">
+        <v>770</v>
+      </c>
+      <c r="M73" s="9" t="s">
+        <v>800</v>
+      </c>
+      <c r="N73" s="9" t="s">
+        <v>765</v>
+      </c>
+      <c r="O73" s="16" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="74" spans="1:15" ht="124.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="7" t="s">
+        <v>801</v>
+      </c>
+      <c r="B74" s="9" t="s">
+        <v>758</v>
+      </c>
+      <c r="C74" s="9" t="s">
+        <v>802</v>
+      </c>
+      <c r="D74" s="9" t="s">
+        <v>803</v>
+      </c>
+      <c r="E74" s="9" t="s">
+        <v>804</v>
+      </c>
+      <c r="F74" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="G74" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H74" s="9">
+        <v>0.5</v>
+      </c>
+      <c r="I74" s="9">
+        <v>1</v>
+      </c>
+      <c r="J74" s="9" t="s">
+        <v>762</v>
+      </c>
+      <c r="K74" s="9" t="s">
+        <v>805</v>
+      </c>
+      <c r="L74" s="9" t="s">
+        <v>770</v>
+      </c>
+      <c r="M74" s="9" t="s">
+        <v>806</v>
+      </c>
+      <c r="N74" s="9" t="s">
+        <v>765</v>
+      </c>
+      <c r="O74" s="16" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15" ht="124.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A75" s="7" t="s">
+        <v>807</v>
+      </c>
+      <c r="B75" s="9" t="s">
+        <v>758</v>
+      </c>
+      <c r="C75" s="9" t="s">
+        <v>808</v>
+      </c>
+      <c r="D75" s="9" t="s">
+        <v>809</v>
+      </c>
+      <c r="E75" s="9" t="s">
+        <v>810</v>
+      </c>
+      <c r="F75" s="9" t="s">
+        <v>415</v>
+      </c>
+      <c r="G75" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H75" s="9">
+        <v>1</v>
+      </c>
+      <c r="I75" s="9">
+        <v>2</v>
+      </c>
+      <c r="J75" s="9" t="s">
+        <v>762</v>
+      </c>
+      <c r="K75" s="9" t="s">
+        <v>772</v>
+      </c>
+      <c r="L75" s="9" t="s">
+        <v>811</v>
+      </c>
+      <c r="M75" s="9" t="s">
+        <v>812</v>
+      </c>
+      <c r="N75" s="9" t="s">
+        <v>765</v>
+      </c>
+      <c r="O75" s="16" t="s">
+        <v>319</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:O48" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
-  <conditionalFormatting sqref="F5:F66">
+  <conditionalFormatting sqref="F5:F75">
     <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
       <formula>"Must"</formula>
     </cfRule>
@@ -9087,7 +9910,7 @@
       <formula>"Could"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O5:O66">
+  <conditionalFormatting sqref="O5:O75">
     <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
       <formula>"Done"</formula>
     </cfRule>
@@ -9099,7 +9922,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="O5:O66" xr:uid="{00000000-0002-0000-0500-000000000000}">
+    <dataValidation type="list" sqref="O5:O75" xr:uid="{00000000-0002-0000-0500-000000000000}">
       <formula1>"To do,In progress,Blocked,Done"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Codex v2.1: sync from Anima; requirements v2.2 and M10-M14 brief
Codex v2.1 (P-010, M10-M14, kill gate 2 after M14, D-40/D-41), requirements v2.2 and backlog mirrored from Drive, brief sections 9-10, changelog.
</commit_message>
<xml_diff>
--- a/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
+++ b/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
@@ -654,11 +654,10 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Working tracker for developers. The source of truth is Project Odyssey.docx v2.0, chapter 12; this workbook is generated from the same data. Updated 2026-10-01: M7-M9 added (D-34); statuses of built stories set to Done.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Working tracker for developers. The source of truth is Project Odyssey.docx v2.2, chapter 12; this workbook is generated from the same data. Updated 2026-10-01: M10-M14 added (D-40, D-41).</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="15.75" customHeight="1" s="20">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -701,7 +700,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15.75" customHeight="1" s="20">
       <c r="A11" s="5" t="inlineStr">
         <is>
@@ -796,7 +794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="20" min="1" max="1"/>
@@ -820,7 +818,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15.75" customHeight="1" s="20">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -835,7 +832,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="15.75" customHeight="1" s="20">
       <c r="A7" s="5" t="inlineStr">
         <is>
@@ -1072,17 +1068,17 @@
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Two pillars playable at region scale: Trade (barter and debts) and Religion (sacred fire and followers). The other four are shown as locked 'later Ages'.</t>
+          <t>Four pillars playable at region scale: Trade, Religion, Politics (D-40) and Technology (tech tree, research, workshops, espionage, the Ember Strand; D-41). Military and Ideology are shown as locked 'later Ages'.</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>PIL-02, PIL-04, ENV-10</t>
+          <t>PIL-02, PIL-03, PIL-04, PIL-05, PIL-08, PIL-09, ENV-10</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1095,7 @@
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Win: your clan leads the region (Dominion 60% in Trade or Religion, or 50% combined). Lose: your hero dies before the Mantle moment, or your clan disbands.</t>
+          <t>Win: Dominion 60% in Trade, Religion or Politics; or the Ember Strand held with a 60% Technology share; or the four pillars averaging 50% (values in Game Rules). Lose: your hero dies before the Mantle moment, or your clan disbands.</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
@@ -1248,72 +1244,77 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15.75" customHeight="1" s="20"/>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+    <row r="23" ht="38.25" customHeight="1" s="20">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>MVP-15</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Authoring</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>The Editor is the authoring tool for quests, story events, entities, mechanics, game rules, routines and the region with its clans and people; every result is a readable file (D-40, 2026-10-01).</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>EDT-01..EDT-06, STO-04, STO-05, SDC-07, ADR-020</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25" ht="51" customHeight="1" s="20">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Success and kill criteria (decided before building)</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="51" customHeight="1" s="20">
-      <c r="A25" s="6" t="inlineStr">
+    <row r="26" ht="63.75" customHeight="1" s="20">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>How measured</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>Gate</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="63.75" customHeight="1" s="20">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>Voluntary play time</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>5 of 8 playtesters play 30+ minutes without being asked to continue</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>Observation + local session log (US-092)</t>
-        </is>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>M6</t>
         </is>
       </c>
     </row>
     <row r="27" ht="38.25" customHeight="1" s="20">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Emergent story</t>
+          <t>Voluntary play time</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>3 of 8 can retell a story that came from the simulation, not from a script</t>
+          <t>5 of 8 playtesters play 30+ minutes without being asked to continue</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>Post-play interview</t>
+          <t>Observation + local session log (US-092)</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
@@ -1325,108 +1326,130 @@
     <row r="28" ht="63.75" customHeight="1" s="20">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Chronicle interest (early)</t>
+          <t>Emergent story</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>2 of 3 readers find a story in the console chronicle</t>
+          <t>3 of 8 can retell a story that came from the simulation, not from a script</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Show printed chronicle (M2: 3 readers, failed 2026-09-30; M2b retry: the owner reads and judges)</t>
+          <t>Post-play interview</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>M2, retried at M2b</t>
+          <t>M6</t>
         </is>
       </c>
     </row>
     <row r="29" ht="51" customHeight="1" s="20">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Frame rate</t>
+          <t>Chronicle interest (early)</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>60 FPS with 500 simulated agents in the region on the minimum PC (OPEN-19)</t>
+          <t>2 of 3 readers find a story in the console chronicle</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>FPS overlay (US-082)</t>
+          <t>Show printed chronicle (M2: 3 readers, failed 2026-09-30; M2b retry: the owner reads and judges)</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M2, retried at M2b</t>
         </is>
       </c>
     </row>
     <row r="30" ht="51" customHeight="1" s="20">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Determinism</t>
+          <t>Frame rate</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Same seed + inputs give the same world hash after 10,000 ticks</t>
+          <t>60 FPS with 500 simulated agents in the region on the minimum PC (OPEN-19)</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Automated test in CI</t>
+          <t>FPS overlay (US-082)</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>M2 onwards</t>
+          <t>M5</t>
         </is>
       </c>
     </row>
     <row r="31" ht="63.75" customHeight="1" s="20">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Stability</t>
+          <t>Determinism</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>No crash in a 2-hour play session or a 100-year soak test</t>
+          <t>Same seed + inputs give the same world hash after 10,000 ticks</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Soak test + crash log</t>
+          <t>Automated test in CI</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>M5, M6</t>
+          <t>M2 onwards</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
+          <t>Stability</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>No crash in a 2-hour play session or a 100-year soak test</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Soak test + crash log</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>M5, M6</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
           <t>Kill / pivot rule</t>
         </is>
       </c>
-      <c r="B32" s="9" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>If M2 or M6 fails: stop adding content; redesign the simulation or the loop first</t>
         </is>
       </c>
-      <c r="C32" s="9" t="inlineStr">
+      <c r="C33" s="9" t="inlineStr">
         <is>
           <t>Owner decision, recorded</t>
         </is>
       </c>
-      <c r="D32" s="9" t="inlineStr">
+      <c r="D33" s="9" t="inlineStr">
         <is>
           <t>M2, M6</t>
         </is>
@@ -1454,7 +1477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EY26"/>
+  <dimension ref="A1:IA31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -1529,6 +1552,86 @@
     <col width="13" customWidth="1" style="20" min="153" max="153"/>
     <col width="13" customWidth="1" style="20" min="154" max="154"/>
     <col width="13" customWidth="1" style="20" min="155" max="155"/>
+    <col width="13" customWidth="1" style="20" min="156" max="156"/>
+    <col width="13" customWidth="1" style="20" min="157" max="157"/>
+    <col width="13" customWidth="1" style="20" min="158" max="158"/>
+    <col width="13" customWidth="1" style="20" min="159" max="159"/>
+    <col width="13" customWidth="1" style="20" min="160" max="160"/>
+    <col width="13" customWidth="1" style="20" min="161" max="161"/>
+    <col width="13" customWidth="1" style="20" min="162" max="162"/>
+    <col width="13" customWidth="1" style="20" min="163" max="163"/>
+    <col width="13" customWidth="1" style="20" min="164" max="164"/>
+    <col width="13" customWidth="1" style="20" min="165" max="165"/>
+    <col width="13" customWidth="1" style="20" min="166" max="166"/>
+    <col width="13" customWidth="1" style="20" min="167" max="167"/>
+    <col width="13" customWidth="1" style="20" min="168" max="168"/>
+    <col width="13" customWidth="1" style="20" min="169" max="169"/>
+    <col width="13" customWidth="1" style="20" min="170" max="170"/>
+    <col width="13" customWidth="1" style="20" min="171" max="171"/>
+    <col width="13" customWidth="1" style="20" min="172" max="172"/>
+    <col width="13" customWidth="1" style="20" min="173" max="173"/>
+    <col width="13" customWidth="1" style="20" min="174" max="174"/>
+    <col width="13" customWidth="1" style="20" min="175" max="175"/>
+    <col width="13" customWidth="1" style="20" min="176" max="176"/>
+    <col width="13" customWidth="1" style="20" min="177" max="177"/>
+    <col width="13" customWidth="1" style="20" min="178" max="178"/>
+    <col width="13" customWidth="1" style="20" min="179" max="179"/>
+    <col width="13" customWidth="1" style="20" min="180" max="180"/>
+    <col width="13" customWidth="1" style="20" min="181" max="181"/>
+    <col width="13" customWidth="1" style="20" min="182" max="182"/>
+    <col width="13" customWidth="1" style="20" min="183" max="183"/>
+    <col width="13" customWidth="1" style="20" min="184" max="184"/>
+    <col width="13" customWidth="1" style="20" min="185" max="185"/>
+    <col width="13" customWidth="1" style="20" min="186" max="186"/>
+    <col width="13" customWidth="1" style="20" min="187" max="187"/>
+    <col width="13" customWidth="1" style="20" min="188" max="188"/>
+    <col width="13" customWidth="1" style="20" min="189" max="189"/>
+    <col width="13" customWidth="1" style="20" min="190" max="190"/>
+    <col width="13" customWidth="1" style="20" min="191" max="191"/>
+    <col width="13" customWidth="1" style="20" min="192" max="192"/>
+    <col width="13" customWidth="1" style="20" min="193" max="193"/>
+    <col width="13" customWidth="1" style="20" min="194" max="194"/>
+    <col width="13" customWidth="1" style="20" min="195" max="195"/>
+    <col width="13" customWidth="1" style="20" min="196" max="196"/>
+    <col width="13" customWidth="1" style="20" min="197" max="197"/>
+    <col width="13" customWidth="1" style="20" min="198" max="198"/>
+    <col width="13" customWidth="1" style="20" min="199" max="199"/>
+    <col width="13" customWidth="1" style="20" min="200" max="200"/>
+    <col width="13" customWidth="1" style="20" min="201" max="201"/>
+    <col width="13" customWidth="1" style="20" min="202" max="202"/>
+    <col width="13" customWidth="1" style="20" min="203" max="203"/>
+    <col width="13" customWidth="1" style="20" min="204" max="204"/>
+    <col width="13" customWidth="1" style="20" min="205" max="205"/>
+    <col width="13" customWidth="1" style="20" min="206" max="206"/>
+    <col width="13" customWidth="1" style="20" min="207" max="207"/>
+    <col width="13" customWidth="1" style="20" min="208" max="208"/>
+    <col width="13" customWidth="1" style="20" min="209" max="209"/>
+    <col width="13" customWidth="1" style="20" min="210" max="210"/>
+    <col width="13" customWidth="1" style="20" min="211" max="211"/>
+    <col width="13" customWidth="1" style="20" min="212" max="212"/>
+    <col width="13" customWidth="1" style="20" min="213" max="213"/>
+    <col width="13" customWidth="1" style="20" min="214" max="214"/>
+    <col width="13" customWidth="1" style="20" min="215" max="215"/>
+    <col width="13" customWidth="1" style="20" min="216" max="216"/>
+    <col width="13" customWidth="1" style="20" min="217" max="217"/>
+    <col width="13" customWidth="1" style="20" min="218" max="218"/>
+    <col width="13" customWidth="1" style="20" min="219" max="219"/>
+    <col width="13" customWidth="1" style="20" min="220" max="220"/>
+    <col width="13" customWidth="1" style="20" min="221" max="221"/>
+    <col width="13" customWidth="1" style="20" min="222" max="222"/>
+    <col width="13" customWidth="1" style="20" min="223" max="223"/>
+    <col width="13" customWidth="1" style="20" min="224" max="224"/>
+    <col width="13" customWidth="1" style="20" min="225" max="225"/>
+    <col width="13" customWidth="1" style="20" min="226" max="226"/>
+    <col width="13" customWidth="1" style="20" min="227" max="227"/>
+    <col width="13" customWidth="1" style="20" min="228" max="228"/>
+    <col width="13" customWidth="1" style="20" min="229" max="229"/>
+    <col width="13" customWidth="1" style="20" min="230" max="230"/>
+    <col width="13" customWidth="1" style="20" min="231" max="231"/>
+    <col width="13" customWidth="1" style="20" min="232" max="232"/>
+    <col width="13" customWidth="1" style="20" min="233" max="233"/>
+    <col width="13" customWidth="1" style="20" min="234" max="234"/>
+    <col width="13" customWidth="1" style="20" min="235" max="235"/>
   </cols>
   <sheetData>
     <row r="1" ht="20.25" customHeight="1" s="20">
@@ -1545,7 +1648,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -1556,7 +1658,6 @@
         <v>46300</v>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="38.25" customHeight="1" s="20">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -2048,6 +2149,246 @@
       <c r="EY6" s="12" t="n">
         <v>140</v>
       </c>
+      <c r="EZ6" s="12" t="n">
+        <v>141</v>
+      </c>
+      <c r="FA6" s="12" t="n">
+        <v>142</v>
+      </c>
+      <c r="FB6" s="12" t="n">
+        <v>143</v>
+      </c>
+      <c r="FC6" s="12" t="n">
+        <v>144</v>
+      </c>
+      <c r="FD6" s="12" t="n">
+        <v>145</v>
+      </c>
+      <c r="FE6" s="12" t="n">
+        <v>146</v>
+      </c>
+      <c r="FF6" s="12" t="n">
+        <v>147</v>
+      </c>
+      <c r="FG6" s="12" t="n">
+        <v>148</v>
+      </c>
+      <c r="FH6" s="12" t="n">
+        <v>149</v>
+      </c>
+      <c r="FI6" s="12" t="n">
+        <v>150</v>
+      </c>
+      <c r="FJ6" s="12" t="n">
+        <v>151</v>
+      </c>
+      <c r="FK6" s="12" t="n">
+        <v>152</v>
+      </c>
+      <c r="FL6" s="12" t="n">
+        <v>153</v>
+      </c>
+      <c r="FM6" s="12" t="n">
+        <v>154</v>
+      </c>
+      <c r="FN6" s="12" t="n">
+        <v>155</v>
+      </c>
+      <c r="FO6" s="12" t="n">
+        <v>156</v>
+      </c>
+      <c r="FP6" s="12" t="n">
+        <v>157</v>
+      </c>
+      <c r="FQ6" s="12" t="n">
+        <v>158</v>
+      </c>
+      <c r="FR6" s="12" t="n">
+        <v>159</v>
+      </c>
+      <c r="FS6" s="12" t="n">
+        <v>160</v>
+      </c>
+      <c r="FT6" s="12" t="n">
+        <v>161</v>
+      </c>
+      <c r="FU6" s="12" t="n">
+        <v>162</v>
+      </c>
+      <c r="FV6" s="12" t="n">
+        <v>163</v>
+      </c>
+      <c r="FW6" s="12" t="n">
+        <v>164</v>
+      </c>
+      <c r="FX6" s="12" t="n">
+        <v>165</v>
+      </c>
+      <c r="FY6" s="12" t="n">
+        <v>166</v>
+      </c>
+      <c r="FZ6" s="12" t="n">
+        <v>167</v>
+      </c>
+      <c r="GA6" s="12" t="n">
+        <v>168</v>
+      </c>
+      <c r="GB6" s="12" t="n">
+        <v>169</v>
+      </c>
+      <c r="GC6" s="12" t="n">
+        <v>170</v>
+      </c>
+      <c r="GD6" s="12" t="n">
+        <v>171</v>
+      </c>
+      <c r="GE6" s="12" t="n">
+        <v>172</v>
+      </c>
+      <c r="GF6" s="12" t="n">
+        <v>173</v>
+      </c>
+      <c r="GG6" s="12" t="n">
+        <v>174</v>
+      </c>
+      <c r="GH6" s="12" t="n">
+        <v>175</v>
+      </c>
+      <c r="GI6" s="12" t="n">
+        <v>176</v>
+      </c>
+      <c r="GJ6" s="12" t="n">
+        <v>177</v>
+      </c>
+      <c r="GK6" s="12" t="n">
+        <v>178</v>
+      </c>
+      <c r="GL6" s="12" t="n">
+        <v>179</v>
+      </c>
+      <c r="GM6" s="12" t="n">
+        <v>180</v>
+      </c>
+      <c r="GN6" s="12" t="n">
+        <v>181</v>
+      </c>
+      <c r="GO6" s="12" t="n">
+        <v>182</v>
+      </c>
+      <c r="GP6" s="12" t="n">
+        <v>183</v>
+      </c>
+      <c r="GQ6" s="12" t="n">
+        <v>184</v>
+      </c>
+      <c r="GR6" s="12" t="n">
+        <v>185</v>
+      </c>
+      <c r="GS6" s="12" t="n">
+        <v>186</v>
+      </c>
+      <c r="GT6" s="12" t="n">
+        <v>187</v>
+      </c>
+      <c r="GU6" s="12" t="n">
+        <v>188</v>
+      </c>
+      <c r="GV6" s="12" t="n">
+        <v>189</v>
+      </c>
+      <c r="GW6" s="12" t="n">
+        <v>190</v>
+      </c>
+      <c r="GX6" s="12" t="n">
+        <v>191</v>
+      </c>
+      <c r="GY6" s="12" t="n">
+        <v>192</v>
+      </c>
+      <c r="GZ6" s="12" t="n">
+        <v>193</v>
+      </c>
+      <c r="HA6" s="12" t="n">
+        <v>194</v>
+      </c>
+      <c r="HB6" s="12" t="n">
+        <v>195</v>
+      </c>
+      <c r="HC6" s="12" t="n">
+        <v>196</v>
+      </c>
+      <c r="HD6" s="12" t="n">
+        <v>197</v>
+      </c>
+      <c r="HE6" s="12" t="n">
+        <v>198</v>
+      </c>
+      <c r="HF6" s="12" t="n">
+        <v>199</v>
+      </c>
+      <c r="HG6" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="HH6" s="12" t="n">
+        <v>201</v>
+      </c>
+      <c r="HI6" s="12" t="n">
+        <v>202</v>
+      </c>
+      <c r="HJ6" s="12" t="n">
+        <v>203</v>
+      </c>
+      <c r="HK6" s="12" t="n">
+        <v>204</v>
+      </c>
+      <c r="HL6" s="12" t="n">
+        <v>205</v>
+      </c>
+      <c r="HM6" s="12" t="n">
+        <v>206</v>
+      </c>
+      <c r="HN6" s="12" t="n">
+        <v>207</v>
+      </c>
+      <c r="HO6" s="12" t="n">
+        <v>208</v>
+      </c>
+      <c r="HP6" s="12" t="n">
+        <v>209</v>
+      </c>
+      <c r="HQ6" s="12" t="n">
+        <v>210</v>
+      </c>
+      <c r="HR6" s="12" t="n">
+        <v>211</v>
+      </c>
+      <c r="HS6" s="12" t="n">
+        <v>212</v>
+      </c>
+      <c r="HT6" s="12" t="n">
+        <v>213</v>
+      </c>
+      <c r="HU6" s="12" t="n">
+        <v>214</v>
+      </c>
+      <c r="HV6" s="12" t="n">
+        <v>215</v>
+      </c>
+      <c r="HW6" s="12" t="n">
+        <v>216</v>
+      </c>
+      <c r="HX6" s="12" t="n">
+        <v>217</v>
+      </c>
+      <c r="HY6" s="12" t="n">
+        <v>218</v>
+      </c>
+      <c r="HZ6" s="12" t="n">
+        <v>219</v>
+      </c>
+      <c r="IA6" s="12" t="n">
+        <v>220</v>
+      </c>
     </row>
     <row r="7" ht="42" customHeight="1" s="20">
       <c r="A7" s="7" t="inlineStr">
@@ -2831,12 +3172,12 @@
     <row r="20" ht="25.5" customHeight="1" s="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Playtest and go/no-go (KILL GATE 2)</t>
+          <t>Quests and story authoring</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -2845,10 +3186,10 @@
         </is>
       </c>
       <c r="D20" s="13" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E20" s="13" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="F20" s="9">
         <f>ROUND((D20+E20)/2,0)</f>
@@ -2884,116 +3225,416 @@
       </c>
       <c r="N20" s="9" t="inlineStr">
         <is>
-          <t>8 outside playtesters play; success criteria measured; go/no-go decision recorded. Held after M9 (owner, 2026-10-01, D-34).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" s="20">
-      <c r="A21" s="7" t="n"/>
-      <c r="B21" s="7" t="inlineStr">
+          <t>The owner writes a quest in the Editor's graph (or offline in JSON), test-plays it with the debugger and saves it; a player gets it from an NPC, follows it in the journal, tracker and markers, and finishes it; the elder tutorial is a quest and crossroads events are edited as story events.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="25.5" customHeight="1" s="20">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Data editors</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="E21" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="F21" s="9">
+        <f>ROUND((D21+E21)/2,0)</f>
+        <v/>
+      </c>
+      <c r="G21" s="9">
+        <f>H20+1</f>
+        <v/>
+      </c>
+      <c r="H21" s="9">
+        <f>G21+F21-1</f>
+        <v/>
+      </c>
+      <c r="I21" s="14">
+        <f>$B$4+(G21-1)*7</f>
+        <v/>
+      </c>
+      <c r="J21" s="14">
+        <f>$B$4+H21*7-1</f>
+        <v/>
+      </c>
+      <c r="K21" s="14">
+        <f>$B$4+SUM($D$7:D21)*7-1</f>
+        <v/>
+      </c>
+      <c r="L21" s="14">
+        <f>$B$4+SUM($E$7:E21)*7-1</f>
+        <v/>
+      </c>
+      <c r="M21" s="9">
+        <f>SUMIFS('User Stories'!$H$5:$H$200,'User Stories'!$J$5:$J$200,A21,'User Stories'!$F$5:$F$200,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$200,'User Stories'!$J$5:$J$200,A21,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="N21" s="9" t="inlineStr">
+        <is>
+          <t>Every data file has a schema; the owner edits any entity, mechanic, story tuning value, game rule and daily routine in Editor forms with pickers and validation, and the running game reloads it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="25.5" customHeight="1" s="20">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>World editing</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="F22" s="9">
+        <f>ROUND((D22+E22)/2,0)</f>
+        <v/>
+      </c>
+      <c r="G22" s="9">
+        <f>H21+1</f>
+        <v/>
+      </c>
+      <c r="H22" s="9">
+        <f>G22+F22-1</f>
+        <v/>
+      </c>
+      <c r="I22" s="14">
+        <f>$B$4+(G22-1)*7</f>
+        <v/>
+      </c>
+      <c r="J22" s="14">
+        <f>$B$4+H22*7-1</f>
+        <v/>
+      </c>
+      <c r="K22" s="14">
+        <f>$B$4+SUM($D$7:D22)*7-1</f>
+        <v/>
+      </c>
+      <c r="L22" s="14">
+        <f>$B$4+SUM($E$7:E22)*7-1</f>
+        <v/>
+      </c>
+      <c r="M22" s="9">
+        <f>SUMIFS('User Stories'!$H$5:$H$200,'User Stories'!$J$5:$J$200,A22,'User Stories'!$F$5:$F$200,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$200,'User Stories'!$J$5:$J$200,A22,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="N22" s="9" t="inlineStr">
+        <is>
+          <t>The owner opens the procedural region in the Editor, tunes the generator with a live preview, paints terrain, water and mountains, places things, people and camps, and edits each clan's and person's relations, economy, routines and actions; edits are saved on top of the seed and a new game plays them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="25.5" customHeight="1" s="20">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D23" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="E23" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="F23" s="9">
+        <f>ROUND((D23+E23)/2,0)</f>
+        <v/>
+      </c>
+      <c r="G23" s="9">
+        <f>H22+1</f>
+        <v/>
+      </c>
+      <c r="H23" s="9">
+        <f>G23+F23-1</f>
+        <v/>
+      </c>
+      <c r="I23" s="14">
+        <f>$B$4+(G23-1)*7</f>
+        <v/>
+      </c>
+      <c r="J23" s="14">
+        <f>$B$4+H23*7-1</f>
+        <v/>
+      </c>
+      <c r="K23" s="14">
+        <f>$B$4+SUM($D$7:D23)*7-1</f>
+        <v/>
+      </c>
+      <c r="L23" s="14">
+        <f>$B$4+SUM($E$7:E23)*7-1</f>
+        <v/>
+      </c>
+      <c r="M23" s="9">
+        <f>SUMIFS('User Stories'!$H$5:$H$200,'User Stories'!$J$5:$J$200,A23,'User Stories'!$F$5:$F$200,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$200,'User Stories'!$J$5:$J$200,A23,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="N23" s="9" t="inlineStr">
+        <is>
+          <t>Clans form alliances and vassal oaths, hold elders' councils, bind themselves by marriage, challenge leaders and use trade and craft knowledge as levers; the player can win the region through Politics; every political rule is editable in the Editor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="25.5" customHeight="1" s="20">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>M14</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="F24" s="9">
+        <f>ROUND((D24+E24)/2,0)</f>
+        <v/>
+      </c>
+      <c r="G24" s="9">
+        <f>H23+1</f>
+        <v/>
+      </c>
+      <c r="H24" s="9">
+        <f>G24+F24-1</f>
+        <v/>
+      </c>
+      <c r="I24" s="14">
+        <f>$B$4+(G24-1)*7</f>
+        <v/>
+      </c>
+      <c r="J24" s="14">
+        <f>$B$4+H24*7-1</f>
+        <v/>
+      </c>
+      <c r="K24" s="14">
+        <f>$B$4+SUM($D$7:D24)*7-1</f>
+        <v/>
+      </c>
+      <c r="L24" s="14">
+        <f>$B$4+SUM($E$7:E24)*7-1</f>
+        <v/>
+      </c>
+      <c r="M24" s="9">
+        <f>SUMIFS('User Stories'!$H$5:$H$200,'User Stories'!$J$5:$J$200,A24,'User Stories'!$F$5:$F$200,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$200,'User Stories'!$J$5:$J$200,A24,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="N24" s="9" t="inlineStr">
+        <is>
+          <t>Clans research by doing in workshops with inventors, pass knowledge by teaching, steal and guard secrets, and unlock recipes, interactions and professions from an editable tech tree; the player can win by forging the Ember Strand while leading in known technologies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="25.5" customHeight="1" s="20">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Playtest and go/no-go (KILL GATE 2)</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="F25" s="9">
+        <f>ROUND((D25+E25)/2,0)</f>
+        <v/>
+      </c>
+      <c r="G25" s="9">
+        <f>H24+1</f>
+        <v/>
+      </c>
+      <c r="H25" s="9">
+        <f>G25+F25-1</f>
+        <v/>
+      </c>
+      <c r="I25" s="14">
+        <f>$B$4+(G25-1)*7</f>
+        <v/>
+      </c>
+      <c r="J25" s="14">
+        <f>$B$4+H25*7-1</f>
+        <v/>
+      </c>
+      <c r="K25" s="14">
+        <f>$B$4+SUM($D$7:D25)*7-1</f>
+        <v/>
+      </c>
+      <c r="L25" s="14">
+        <f>$B$4+SUM($E$7:E25)*7-1</f>
+        <v/>
+      </c>
+      <c r="M25" s="9">
+        <f>SUMIFS('User Stories'!$H$5:$H$200,'User Stories'!$J$5:$J$200,A25,'User Stories'!$F$5:$F$200,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$200,'User Stories'!$J$5:$J$200,A25,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="N25" s="9" t="inlineStr">
+        <is>
+          <t>8 outside playtesters play; success criteria measured; go/no-go decision recorded. Held after M14 (owner, 2026-10-01, D-41).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" s="20">
+      <c r="A26" s="7" t="n"/>
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>MVP total</t>
         </is>
       </c>
-      <c r="C21" s="7" t="n"/>
-      <c r="D21" s="7">
-        <f>SUM(D7:D20)</f>
-        <v/>
-      </c>
-      <c r="E21" s="7">
-        <f>SUM(E7:E20)</f>
-        <v/>
-      </c>
-      <c r="F21" s="7">
-        <f>SUM(F7:F20)</f>
-        <v/>
-      </c>
-      <c r="G21" s="7" t="n"/>
-      <c r="H21" s="7">
-        <f>H20</f>
-        <v/>
-      </c>
-      <c r="I21" s="15">
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="7">
+        <f>SUM(D7:D25)</f>
+        <v/>
+      </c>
+      <c r="E26" s="7">
+        <f>SUM(E7:E25)</f>
+        <v/>
+      </c>
+      <c r="F26" s="7">
+        <f>SUM(F7:F25)</f>
+        <v/>
+      </c>
+      <c r="G26" s="7" t="n"/>
+      <c r="H26" s="7">
+        <f>H25</f>
+        <v/>
+      </c>
+      <c r="I26" s="15">
         <f>I7</f>
         <v/>
       </c>
-      <c r="J21" s="15">
-        <f>J20</f>
-        <v/>
-      </c>
-      <c r="K21" s="15">
-        <f>K20</f>
-        <v/>
-      </c>
-      <c r="L21" s="15">
-        <f>L20</f>
-        <v/>
-      </c>
-      <c r="M21" s="7" t="n"/>
-      <c r="N21" s="7" t="inlineStr">
+      <c r="J26" s="15">
+        <f>J25</f>
+        <v/>
+      </c>
+      <c r="K26" s="15">
+        <f>K25</f>
+        <v/>
+      </c>
+      <c r="L26" s="15">
+        <f>L25</f>
+        <v/>
+      </c>
+      <c r="M26" s="7" t="n"/>
+      <c r="N26" s="7" t="inlineStr">
         <is>
           <t>Months (likely) = weeks / 4.33</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="27.95" customHeight="1" s="20">
-      <c r="A22" s="7" t="n"/>
-      <c r="B22" s="7" t="inlineStr">
+    <row r="27" ht="27.95" customHeight="1" s="20">
+      <c r="A27" s="7" t="n"/>
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>In months</t>
         </is>
       </c>
-      <c r="C22" s="7" t="n"/>
-      <c r="D22" s="7">
-        <f>ROUND(D21/4.33,1)</f>
-        <v/>
-      </c>
-      <c r="E22" s="7">
-        <f>ROUND(E21/4.33,1)</f>
-        <v/>
-      </c>
-      <c r="F22" s="7">
-        <f>ROUND(F21/4.33,1)</f>
-        <v/>
-      </c>
-      <c r="G22" s="7" t="n"/>
-      <c r="H22" s="7" t="n"/>
-      <c r="I22" s="7" t="n"/>
-      <c r="J22" s="7" t="n"/>
-      <c r="K22" s="7" t="n"/>
-      <c r="L22" s="7" t="n"/>
-      <c r="M22" s="7" t="n"/>
-      <c r="N22" s="7" t="n"/>
-    </row>
-    <row r="23" ht="27.95" customHeight="1" s="20"/>
-    <row r="24" ht="27.95" customHeight="1" s="20">
-      <c r="B24" s="19" t="inlineStr">
+      <c r="C27" s="7" t="n"/>
+      <c r="D27" s="7">
+        <f>ROUND(D26/4.33,1)</f>
+        <v/>
+      </c>
+      <c r="E27" s="7">
+        <f>ROUND(E26/4.33,1)</f>
+        <v/>
+      </c>
+      <c r="F27" s="7">
+        <f>ROUND(F26/4.33,1)</f>
+        <v/>
+      </c>
+      <c r="G27" s="7" t="n"/>
+      <c r="H27" s="7" t="n"/>
+      <c r="I27" s="7" t="n"/>
+      <c r="J27" s="7" t="n"/>
+      <c r="K27" s="7" t="n"/>
+      <c r="L27" s="7" t="n"/>
+      <c r="M27" s="7" t="n"/>
+      <c r="N27" s="7" t="n"/>
+    </row>
+    <row r="28" ht="27.95" customHeight="1" s="20"/>
+    <row r="29" ht="27.95" customHeight="1" s="20">
+      <c r="B29" s="19" t="inlineStr">
         <is>
           <t>Why the estimate grew: the learning path (requirements, section 8.3) estimated 9-13 months top-down. The bottom-up sum of the MVP stories is higher; this sheet uses the bottom-up figure.</t>
         </is>
       </c>
     </row>
-    <row r="25" s="20">
-      <c r="B25" s="19" t="inlineStr">
+    <row r="30" s="20">
+      <c r="B30" s="19" t="inlineStr">
         <is>
           <t>Buffer: the 'Should' stories are the cut list if time runs short. Cutting all of them saves about 5-11 weeks.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="102" customHeight="1" s="20">
-      <c r="B26" s="19" t="inlineStr">
-        <is>
-          <t>Kill gates: M2 (is the console chronicle interesting? failed 2026-09-30, passed at the M2b retry) and M6 (do playtesters stay?), held after M9 (D-34). Critical path: M0 &gt; M1 &gt; M1b &gt; M2 &gt; M2b &gt; M2c &gt; M2d &gt; M3 &gt; M4 &gt; M5 &gt; M7 &gt; M8 &gt; M9 &gt; M6. Dates of M2c onwards are not re-planned yet.</t>
+    <row r="31" ht="102" customHeight="1" s="20">
+      <c r="B31" s="19" t="inlineStr">
+        <is>
+          <t>Kill gates: M2 (is the console chronicle interesting? failed 2026-09-30, passed at the M2b retry) and M6 (do playtesters stay?), held after M14 (D-41). Critical path: M0 &gt; M1 &gt; M1b &gt; M2 &gt; M2b &gt; M2c &gt; M2d &gt; M3 &gt; M4 &gt; M5 &gt; M7 &gt; M8 &gt; M9 &gt; M10 &gt; M11 &gt; M12 &gt; M13 &gt; M14 &gt; M6. Dates of M2c onwards are not re-planned yet.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B25:N25"/>
-    <mergeCell ref="B24:N24"/>
-    <mergeCell ref="B26:N26"/>
+    <mergeCell ref="B31:N31"/>
+    <mergeCell ref="B30:N30"/>
+    <mergeCell ref="B29:N29"/>
   </mergeCells>
-  <conditionalFormatting sqref="P7:EY20">
+  <conditionalFormatting sqref="P7:IA25">
     <cfRule type="expression" priority="1" dxfId="10">
       <formula>AND(P$6&gt;=$G7,P$6&lt;=$H7)</formula>
     </cfRule>
@@ -3008,7 +3649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -3034,7 +3675,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -3598,7 +4238,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Technical chain: M0 &gt; M1 &gt; M1b &gt; M2 &gt; M2b &gt; M2c &gt; M2d &gt; M3 &gt; M4 &gt; M5 &gt; M7 &gt; M8 &gt; M9 &gt; M6 (each milestone needs the previous one)</t>
+          <t>Technical chain: M0 &gt; M1 &gt; M1b &gt; M2 &gt; M2b &gt; M2c &gt; M2d &gt; M3 &gt; M4 &gt; M5 &gt; M7 &gt; M8 &gt; M9 &gt; M10 &gt; M11 &gt; M12 &gt; M13 &gt; M14 &gt; M6 (each milestone needs the previous one)</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -3881,6 +4521,80 @@
         </is>
       </c>
       <c r="G26" s="16" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="25.5" customHeight="1" s="20">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>D-40</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (Round 14): M10 Quests (authored only, JSON + quest graph, flat with prerequisites, journal + tracker + markers, tutorial as a quest, story events), M11 Data editors (schema forms, Game Rules with system switches, daily routines), M12 World editing (generator settings with preview, overrides on the seed, per clan and person setup), M13 Politics (third pillar with victory); play-in-editor debugger; kill gate 2 after M13</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Design decision</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>US-180..US-216</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G27" s="16" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="25.5" customHeight="1" s="20">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>D-41</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Technology pillar (M14: tech tree as data, research by doing, workshops and inventors, espionage and theft; victory = Ember held + 60% Technology share or the four-pillar 50% average); Politics victory confirmed (60% / 50%); Game Rules default standard.json, levels may name their own; M10-M14: Dominus decides design questions (delegated) and tests run at exit reviews; kill gate 2 after M14</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Design decision</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>US-180..US-226</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G28" s="16" t="inlineStr">
         <is>
           <t>Decided</t>
         </is>
@@ -3916,7 +4630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -3944,7 +4658,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="25.5" customHeight="1" s="20">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -4779,37 +5492,267 @@
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="7" t="n"/>
-      <c r="B22" s="7" t="inlineStr">
+    <row r="22" ht="25.5" customHeight="1" s="20">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>E17</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Quests</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>The owner writes quests in the Editor and offline; players get, follow and finish them with a journal, a tracker and markers.</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="E22" s="9">
+        <f>COUNTIF('User Stories'!$B$5:$B$200,A22)</f>
+        <v/>
+      </c>
+      <c r="F22" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A22,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="G22" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A22,'User Stories'!$H$5:$H$200)</f>
+        <v/>
+      </c>
+      <c r="H22" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A22,'User Stories'!$I$5:$I$200)</f>
+        <v/>
+      </c>
+      <c r="I22" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A22,'User Stories'!$O$5:$O$200,"Done")</f>
+        <v/>
+      </c>
+      <c r="J22" s="17">
+        <f>IFERROR(I22/E22,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="25.5" customHeight="1" s="20">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>E18</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Data editors</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Every data file (entities, mechanics, story tuning, game rules, daily routines) is edited in the Editor through forms built from schemas.</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="E23" s="9">
+        <f>COUNTIF('User Stories'!$B$5:$B$200,A23)</f>
+        <v/>
+      </c>
+      <c r="F23" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A23,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="G23" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A23,'User Stories'!$H$5:$H$200)</f>
+        <v/>
+      </c>
+      <c r="H23" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A23,'User Stories'!$I$5:$I$200)</f>
+        <v/>
+      </c>
+      <c r="I23" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A23,'User Stories'!$O$5:$O$200,"Done")</f>
+        <v/>
+      </c>
+      <c r="J23" s="17">
+        <f>IFERROR(I23/E23,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="25.5" customHeight="1" s="20">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>E19</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>World editing</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>The owner shapes the procedural region and its clans, people, economy and relations in the Editor, on top of the seed.</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="E24" s="9">
+        <f>COUNTIF('User Stories'!$B$5:$B$200,A24)</f>
+        <v/>
+      </c>
+      <c r="F24" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A24,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="G24" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A24,'User Stories'!$H$5:$H$200)</f>
+        <v/>
+      </c>
+      <c r="H24" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A24,'User Stories'!$I$5:$I$200)</f>
+        <v/>
+      </c>
+      <c r="I24" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A24,'User Stories'!$O$5:$O$200,"Done")</f>
+        <v/>
+      </c>
+      <c r="J24" s="17">
+        <f>IFERROR(I24/E24,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="25.5" customHeight="1" s="20">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>E20</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Clans ally, swear and break oaths, marry, vote and challenge leaders; the player can win the region through Politics.</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="E25" s="9">
+        <f>COUNTIF('User Stories'!$B$5:$B$200,A25)</f>
+        <v/>
+      </c>
+      <c r="F25" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A25,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="G25" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A25,'User Stories'!$H$5:$H$200)</f>
+        <v/>
+      </c>
+      <c r="H25" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A25,'User Stories'!$I$5:$I$200)</f>
+        <v/>
+      </c>
+      <c r="I25" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A25,'User Stories'!$O$5:$O$200,"Done")</f>
+        <v/>
+      </c>
+      <c r="J25" s="17">
+        <f>IFERROR(I25/E25,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="25.5" customHeight="1" s="20">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>E21</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Clans discover, teach, guard and steal technologies; the player can win the region by forging the Ember Strand while leading in know-how.</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>M14</t>
+        </is>
+      </c>
+      <c r="E26" s="9">
+        <f>COUNTIF('User Stories'!$B$5:$B$200,A26)</f>
+        <v/>
+      </c>
+      <c r="F26" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A26,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="G26" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A26,'User Stories'!$H$5:$H$200)</f>
+        <v/>
+      </c>
+      <c r="H26" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A26,'User Stories'!$I$5:$I$200)</f>
+        <v/>
+      </c>
+      <c r="I26" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A26,'User Stories'!$O$5:$O$200,"Done")</f>
+        <v/>
+      </c>
+      <c r="J26" s="17">
+        <f>IFERROR(I26/E26,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="n"/>
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C22" s="7" t="n"/>
-      <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7">
-        <f>SUM(E5:E21)</f>
-        <v/>
-      </c>
-      <c r="F22" s="7">
-        <f>SUM(F5:F21)</f>
-        <v/>
-      </c>
-      <c r="G22" s="7">
-        <f>SUM(G5:G21)</f>
-        <v/>
-      </c>
-      <c r="H22" s="7">
-        <f>SUM(H5:H21)</f>
-        <v/>
-      </c>
-      <c r="I22" s="7">
-        <f>SUM(I5:I21)</f>
-        <v/>
-      </c>
-      <c r="J22" s="18">
-        <f>IFERROR(I22/E22,0)</f>
+      <c r="C27" s="7" t="n"/>
+      <c r="D27" s="7" t="n"/>
+      <c r="E27" s="7">
+        <f>SUM(E5:E26)</f>
+        <v/>
+      </c>
+      <c r="F27" s="7">
+        <f>SUM(F5:F26)</f>
+        <v/>
+      </c>
+      <c r="G27" s="7">
+        <f>SUM(G5:G26)</f>
+        <v/>
+      </c>
+      <c r="H27" s="7">
+        <f>SUM(H5:H26)</f>
+        <v/>
+      </c>
+      <c r="I27" s="7">
+        <f>SUM(I5:I26)</f>
+        <v/>
+      </c>
+      <c r="J27" s="18">
+        <f>IFERROR(I27/E27,0)</f>
         <v/>
       </c>
     </row>
@@ -4824,7 +5767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O97"/>
+  <dimension ref="A1:O134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="20" min="1" max="1"/>
@@ -4857,7 +5800,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="25.5" customHeight="1" s="20">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -11053,7 +11995,7 @@
       </c>
       <c r="O79" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11139,7 +12081,7 @@
       </c>
       <c r="O80" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11225,7 +12167,7 @@
       </c>
       <c r="O81" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11311,7 +12253,7 @@
       </c>
       <c r="O82" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11397,7 +12339,7 @@
       </c>
       <c r="O83" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11483,7 +12425,7 @@
       </c>
       <c r="O84" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -11569,7 +12511,7 @@
       </c>
       <c r="O85" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -12600,6 +13542,3188 @@
         </is>
       </c>
       <c r="O97" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="124.15" customHeight="1" s="20">
+      <c r="A98" s="7" t="inlineStr">
+        <is>
+          <t>US-180</t>
+        </is>
+      </c>
+      <c r="B98" s="9" t="inlineStr">
+        <is>
+          <t>E17</t>
+        </is>
+      </c>
+      <c r="C98" s="9" t="inlineStr">
+        <is>
+          <t>Quest data and runtime</t>
+        </is>
+      </c>
+      <c r="D98" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want quests as JSON files with steps, objectives, conditions, rewards and prerequisites, so that I can write quests offline and the game runs them.</t>
+        </is>
+      </c>
+      <c r="E98" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Load
+Given a quest file with two steps, a branch and a reward
+When the game starts
+Then the quest is available once its prerequisites hold
+Scenario: Progress
+Given an active quest
+When its step's objective is met
+Then the next step starts and the reward is given at the end
+Scenario: Error
+Given a quest whose step points to a missing step on line 14
+When the data loads
+Then the error reads 'quests/&lt;file&gt;.json:14: unknown step' and the rest loads</t>
+        </is>
+      </c>
+      <c r="F98" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G98" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H98" s="9">
+        <f>VLOOKUP(G98,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I98" s="9">
+        <f>VLOOKUP(G98,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J98" s="9" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="K98" s="9" t="inlineStr">
+        <is>
+          <t>US-150, US-164, D-40</t>
+        </is>
+      </c>
+      <c r="L98" s="9" t="inlineStr">
+        <is>
+          <t>STO-04, ADR-019</t>
+        </is>
+      </c>
+      <c r="M98" s="9" t="inlineStr">
+        <is>
+          <t>State machines over data; saving progress</t>
+        </is>
+      </c>
+      <c r="N98" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O98" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="124.15" customHeight="1" s="20">
+      <c r="A99" s="7" t="inlineStr">
+        <is>
+          <t>US-181</t>
+        </is>
+      </c>
+      <c r="B99" s="9" t="inlineStr">
+        <is>
+          <t>E17</t>
+        </is>
+      </c>
+      <c r="C99" s="9" t="inlineStr">
+        <is>
+          <t>Objectives from world events</t>
+        </is>
+      </c>
+      <c r="D99" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want my actions in the world to count toward quests, so that quests follow what I really do.</t>
+        </is>
+      </c>
+      <c r="E99" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Count
+Given an objective 'gather 5 berries'
+When the hero gathers 5 berries
+Then the objective is complete
+Scenario: Kinds
+Given objectives talk, go to, gather, give, craft, interact, defeat, wait and flag
+When each happens
+Then each is detected
+Scenario: Not mine
+Given an NPC gathering berries
+When it happens
+Then the hero's quest does not count it</t>
+        </is>
+      </c>
+      <c r="F99" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G99" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H99" s="9">
+        <f>VLOOKUP(G99,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I99" s="9">
+        <f>VLOOKUP(G99,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J99" s="9" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="K99" s="9" t="inlineStr">
+        <is>
+          <t>US-180</t>
+        </is>
+      </c>
+      <c r="L99" s="9" t="inlineStr">
+        <is>
+          <t>STO-04, INT-01</t>
+        </is>
+      </c>
+      <c r="M99" s="9" t="inlineStr">
+        <is>
+          <t>An event bus (observer pattern)</t>
+        </is>
+      </c>
+      <c r="N99" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O99" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="124.15" customHeight="1" s="20">
+      <c r="A100" s="7" t="inlineStr">
+        <is>
+          <t>US-182</t>
+        </is>
+      </c>
+      <c r="B100" s="9" t="inlineStr">
+        <is>
+          <t>E17</t>
+        </is>
+      </c>
+      <c r="C100" s="9" t="inlineStr">
+        <is>
+          <t>Getting and handing in quests</t>
+        </is>
+      </c>
+      <c r="D100" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want NPCs to offer quests in conversation and take them back when done, so that quests belong to people.</t>
+        </is>
+      </c>
+      <c r="E100" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Offer
+Given an NPC with an available quest
+When the hero is near
+Then a quest sign shows over the NPC and Talk offers the quest
+Scenario: Accept
+Given the offer in a .dlg choice with {quest start &lt;id&gt;}
+When the player picks it
+Then the quest is active
+Scenario: Hand in
+Given a finished quest and its giver
+When the player talks to the giver
+Then the turn-in line plays and the reward is given</t>
+        </is>
+      </c>
+      <c r="F100" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G100" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H100" s="9">
+        <f>VLOOKUP(G100,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I100" s="9">
+        <f>VLOOKUP(G100,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J100" s="9" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="K100" s="9" t="inlineStr">
+        <is>
+          <t>US-180, US-161</t>
+        </is>
+      </c>
+      <c r="L100" s="9" t="inlineStr">
+        <is>
+          <t>STO-04, SDC-03</t>
+        </is>
+      </c>
+      <c r="M100" s="9" t="inlineStr">
+        <is>
+          <t>Linking two data systems through ids</t>
+        </is>
+      </c>
+      <c r="N100" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O100" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="124.15" customHeight="1" s="20">
+      <c r="A101" s="7" t="inlineStr">
+        <is>
+          <t>US-183</t>
+        </is>
+      </c>
+      <c r="B101" s="9" t="inlineStr">
+        <is>
+          <t>E17</t>
+        </is>
+      </c>
+      <c r="C101" s="9" t="inlineStr">
+        <is>
+          <t>Journal, tracker and markers</t>
+        </is>
+      </c>
+      <c r="D101" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want a journal, an on-screen tracker and markers over targets, so that I always know what to do next.</t>
+        </is>
+      </c>
+      <c r="E101" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Journal
+Given two active, one done and one failed quest
+When the player opens the journal
+Then they are listed in their groups with each step's text and log
+Scenario: Tracker
+Given an active quest
+When its step changes
+Then the tracker shows the new step at once
+Scenario: Markers
+Given markers on in settings
+When a step targets a person or place
+Then a marker shows over it; with markers off, none shows</t>
+        </is>
+      </c>
+      <c r="F101" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G101" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H101" s="9">
+        <f>VLOOKUP(G101,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I101" s="9">
+        <f>VLOOKUP(G101,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J101" s="9" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="K101" s="9" t="inlineStr">
+        <is>
+          <t>US-180</t>
+        </is>
+      </c>
+      <c r="L101" s="9" t="inlineStr">
+        <is>
+          <t>STO-04</t>
+        </is>
+      </c>
+      <c r="M101" s="9" t="inlineStr">
+        <is>
+          <t>Immediate-mode UI lists</t>
+        </is>
+      </c>
+      <c r="N101" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O101" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="124.15" customHeight="1" s="20">
+      <c r="A102" s="7" t="inlineStr">
+        <is>
+          <t>US-184</t>
+        </is>
+      </c>
+      <c r="B102" s="9" t="inlineStr">
+        <is>
+          <t>E17</t>
+        </is>
+      </c>
+      <c r="C102" s="9" t="inlineStr">
+        <is>
+          <t>Quest graph editor</t>
+        </is>
+      </c>
+      <c r="D102" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to build quests as graphs in the Editor, so that I can see and change their steps, branches and prerequisites.</t>
+        </is>
+      </c>
+      <c r="E102" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Steps
+Given a quest open in the Editor
+When the owner adds a step and wires a branch
+Then the graph and the saved JSON show them
+Scenario: Blocks
+Given a step selected
+When the owner adds an objective, a condition and a reward
+Then pickers offer items, people, places, tags and quests
+Scenario: Prerequisites
+Given the quest list view
+When the owner links quest B after quest A
+Then B's prerequisites name A and the view draws the link</t>
+        </is>
+      </c>
+      <c r="F102" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G102" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H102" s="9">
+        <f>VLOOKUP(G102,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I102" s="9">
+        <f>VLOOKUP(G102,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J102" s="9" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="K102" s="9" t="inlineStr">
+        <is>
+          <t>US-180, US-170</t>
+        </is>
+      </c>
+      <c r="L102" s="9" t="inlineStr">
+        <is>
+          <t>STO-04, EDT-01</t>
+        </is>
+      </c>
+      <c r="M102" s="9" t="inlineStr">
+        <is>
+          <t>Reusing a generic widget for a new data type</t>
+        </is>
+      </c>
+      <c r="N102" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O102" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="124.15" customHeight="1" s="20">
+      <c r="A103" s="7" t="inlineStr">
+        <is>
+          <t>US-185</t>
+        </is>
+      </c>
+      <c r="B103" s="9" t="inlineStr">
+        <is>
+          <t>E17</t>
+        </is>
+      </c>
+      <c r="C103" s="9" t="inlineStr">
+        <is>
+          <t>The tutorial as a quest; story events</t>
+        </is>
+      </c>
+      <c r="D103" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want the elder tutorial rebuilt as the first quest and the crossroads events edited as story events, so that all story content is authored in one place.</t>
+        </is>
+      </c>
+      <c r="E103" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Tutorial
+Given a new game with the tutorial on
+When the player starts
+Then the elder quest guides gather, eat and tend the fire as before, with the hint after 2 minutes
+Scenario: Story events
+Given a crossroads event
+When the owner opens it in the Editor
+Then its trigger, text and options with effects are edited and saved
+Scenario: Same game
+Given the M5 and M6 tests
+When they run
+Then they pass</t>
+        </is>
+      </c>
+      <c r="F103" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G103" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H103" s="9">
+        <f>VLOOKUP(G103,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I103" s="9">
+        <f>VLOOKUP(G103,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J103" s="9" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="K103" s="9" t="inlineStr">
+        <is>
+          <t>US-184, US-090</t>
+        </is>
+      </c>
+      <c r="L103" s="9" t="inlineStr">
+        <is>
+          <t>STO-05, EDT-01</t>
+        </is>
+      </c>
+      <c r="M103" s="9" t="inlineStr">
+        <is>
+          <t>Migrating data without changing behaviour</t>
+        </is>
+      </c>
+      <c r="N103" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O103" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="124.15" customHeight="1" s="20">
+      <c r="A104" s="7" t="inlineStr">
+        <is>
+          <t>US-186</t>
+        </is>
+      </c>
+      <c r="B104" s="9" t="inlineStr">
+        <is>
+          <t>E17</t>
+        </is>
+      </c>
+      <c r="C104" s="9" t="inlineStr">
+        <is>
+          <t>Play-in-editor debugger</t>
+        </is>
+      </c>
+      <c r="D104" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to play from any spot in the Editor with a debug panel, so that I can test quests and content in minutes.</t>
+        </is>
+      </c>
+      <c r="E104" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Play here
+Given the Editor open
+When the owner chooses Play here
+Then the hero starts at the cursor and Esc returns to the Editor unchanged
+Scenario: Control
+Given the debug panel
+When the owner starts, completes or resets a quest, sets a flag, an item or an opinion, jumps time or teleports
+Then the game reflects it at once
+Scenario: Why not
+Given a quest step that does not complete
+When the owner selects it in the panel
+Then the failing condition and its current values are shown</t>
+        </is>
+      </c>
+      <c r="F104" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G104" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H104" s="9">
+        <f>VLOOKUP(G104,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I104" s="9">
+        <f>VLOOKUP(G104,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J104" s="9" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="K104" s="9" t="inlineStr">
+        <is>
+          <t>US-180</t>
+        </is>
+      </c>
+      <c r="L104" s="9" t="inlineStr">
+        <is>
+          <t>EDT-06</t>
+        </is>
+      </c>
+      <c r="M104" s="9" t="inlineStr">
+        <is>
+          <t>Debug-only code paths</t>
+        </is>
+      </c>
+      <c r="N104" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O104" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="124.15" customHeight="1" s="20">
+      <c r="A105" s="7" t="inlineStr">
+        <is>
+          <t>US-187</t>
+        </is>
+      </c>
+      <c r="B105" s="9" t="inlineStr">
+        <is>
+          <t>E17</t>
+        </is>
+      </c>
+      <c r="C105" s="9" t="inlineStr">
+        <is>
+          <t>Quest validation</t>
+        </is>
+      </c>
+      <c r="D105" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want broken quests found before players see them, so that no quest can get stuck.</t>
+        </is>
+      </c>
+      <c r="E105" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Unreachable
+Given a step no branch leads to
+When validation runs
+Then it is listed and clicking it selects it
+Scenario: Impossible
+Given an objective naming an unknown item, person or place
+When validation runs
+Then it is listed
+Scenario: Cycle
+Given quests that require each other
+When validation runs
+Then the prerequisite cycle is listed</t>
+        </is>
+      </c>
+      <c r="F105" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G105" s="9" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H105" s="9">
+        <f>VLOOKUP(G105,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I105" s="9">
+        <f>VLOOKUP(G105,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J105" s="9" t="inlineStr">
+        <is>
+          <t>M10</t>
+        </is>
+      </c>
+      <c r="K105" s="9" t="inlineStr">
+        <is>
+          <t>US-184</t>
+        </is>
+      </c>
+      <c r="L105" s="9" t="inlineStr">
+        <is>
+          <t>STO-04, EDT-01</t>
+        </is>
+      </c>
+      <c r="M105" s="9" t="inlineStr">
+        <is>
+          <t>Cycle detection in a graph</t>
+        </is>
+      </c>
+      <c r="N105" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O105" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="124.15" customHeight="1" s="20">
+      <c r="A106" s="7" t="inlineStr">
+        <is>
+          <t>US-190</t>
+        </is>
+      </c>
+      <c r="B106" s="9" t="inlineStr">
+        <is>
+          <t>E18</t>
+        </is>
+      </c>
+      <c r="C106" s="9" t="inlineStr">
+        <is>
+          <t>Schemas for every data file</t>
+        </is>
+      </c>
+      <c r="D106" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want every data file described by a schema with types, ranges, choices, links and help text, so that the Editor and the validator know what each field means.</t>
+        </is>
+      </c>
+      <c r="E106" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Coverage
+Given every file under assets/data/
+When the schema check runs in CI
+Then each file has a schema and passes it
+Scenario: Errors
+Given a value out of its range
+When the game loads it
+Then the error names file, line, field and the allowed range
+Scenario: Links
+Given a recipe naming an item no catalog has
+When the check runs
+Then the broken link is listed</t>
+        </is>
+      </c>
+      <c r="F106" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G106" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H106" s="9">
+        <f>VLOOKUP(G106,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I106" s="9">
+        <f>VLOOKUP(G106,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J106" s="9" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="K106" s="9" t="inlineStr">
+        <is>
+          <t>US-150</t>
+        </is>
+      </c>
+      <c r="L106" s="9" t="inlineStr">
+        <is>
+          <t>EDT-02, ADR-020</t>
+        </is>
+      </c>
+      <c r="M106" s="9" t="inlineStr">
+        <is>
+          <t>Describing data with data (a schema interpreter)</t>
+        </is>
+      </c>
+      <c r="N106" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O106" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="124.15" customHeight="1" s="20">
+      <c r="A107" s="7" t="inlineStr">
+        <is>
+          <t>US-191</t>
+        </is>
+      </c>
+      <c r="B107" s="9" t="inlineStr">
+        <is>
+          <t>E18</t>
+        </is>
+      </c>
+      <c r="C107" s="9" t="inlineStr">
+        <is>
+          <t>Schema-driven form editor</t>
+        </is>
+      </c>
+      <c r="D107" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want a Data tab where any file opens as forms built from its schema, so that I can edit everything without touching JSON.</t>
+        </is>
+      </c>
+      <c r="E107" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Open
+Given weapons.json
+When the owner opens it in the Data tab
+Then entries are listed with search, and a form shows the selected entry's fields with help text
+Scenario: Edit
+Given a damage value changed and Ctrl+S
+When the file is saved
+Then only that value changes in the file, note fields stay, and the running game uses it
+Scenario: Undo
+Given five form edits
+When Ctrl+Z five times
+Then the data is as before</t>
+        </is>
+      </c>
+      <c r="F107" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G107" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H107" s="9">
+        <f>VLOOKUP(G107,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I107" s="9">
+        <f>VLOOKUP(G107,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J107" s="9" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="K107" s="9" t="inlineStr">
+        <is>
+          <t>US-190, US-121</t>
+        </is>
+      </c>
+      <c r="L107" s="9" t="inlineStr">
+        <is>
+          <t>EDT-02</t>
+        </is>
+      </c>
+      <c r="M107" s="9" t="inlineStr">
+        <is>
+          <t>Building UI from a description at run time</t>
+        </is>
+      </c>
+      <c r="N107" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O107" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="124.15" customHeight="1" s="20">
+      <c r="A108" s="7" t="inlineStr">
+        <is>
+          <t>US-192</t>
+        </is>
+      </c>
+      <c r="B108" s="9" t="inlineStr">
+        <is>
+          <t>E18</t>
+        </is>
+      </c>
+      <c r="C108" s="9" t="inlineStr">
+        <is>
+          <t>Picture pickers and cutting frames</t>
+        </is>
+      </c>
+      <c r="D108" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to pick sprites, animations and effects by picture and cut new frames from my sheets in the Editor, so that new content gets its art without the command line.</t>
+        </is>
+      </c>
+      <c r="E108" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Pick
+Given a field holding an atlas frame
+When the owner opens its picker
+Then frames are shown as pictures and the choice is saved
+Scenario: Preview
+Given an effect or an animation
+When it is selected
+Then it plays in the form
+Scenario: Cut
+Given a sheet in assets/sprites/
+When the owner draws a rectangle and names it
+Then cuts.json gains the cut and the atlas is rebuilt</t>
+        </is>
+      </c>
+      <c r="F108" s="9" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="G108" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H108" s="9">
+        <f>VLOOKUP(G108,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I108" s="9">
+        <f>VLOOKUP(G108,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J108" s="9" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="K108" s="9" t="inlineStr">
+        <is>
+          <t>US-191, US-120</t>
+        </is>
+      </c>
+      <c r="L108" s="9" t="inlineStr">
+        <is>
+          <t>EDT-02, D-05</t>
+        </is>
+      </c>
+      <c r="M108" s="9" t="inlineStr">
+        <is>
+          <t>Image regions and previews</t>
+        </is>
+      </c>
+      <c r="N108" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O108" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="124.15" customHeight="1" s="20">
+      <c r="A109" s="7" t="inlineStr">
+        <is>
+          <t>US-193</t>
+        </is>
+      </c>
+      <c r="B109" s="9" t="inlineStr">
+        <is>
+          <t>E18</t>
+        </is>
+      </c>
+      <c r="C109" s="9" t="inlineStr">
+        <is>
+          <t>Entity editor</t>
+        </is>
+      </c>
+      <c r="D109" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to create, copy, rename and delete kinds of weapons, plants, animals, characters, objects and items, with their tags, states and interactions, so that new entities need no code.</t>
+        </is>
+      </c>
+      <c r="E109" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Create
+Given the plants catalog
+When the owner copies a bush, renames it and changes its tags
+Then the new plant appears in the Editor palette and offers its interactions
+Scenario: Rename
+Given an item used by recipes and quests
+When the owner renames it
+Then every reference is updated and listed
+Scenario: Delete
+Given a kind that is still used
+When the owner deletes it
+Then the uses are listed and the delete waits for confirmation</t>
+        </is>
+      </c>
+      <c r="F109" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G109" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H109" s="9">
+        <f>VLOOKUP(G109,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I109" s="9">
+        <f>VLOOKUP(G109,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J109" s="9" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="K109" s="9" t="inlineStr">
+        <is>
+          <t>US-191, US-172</t>
+        </is>
+      </c>
+      <c r="L109" s="9" t="inlineStr">
+        <is>
+          <t>EDT-02, INT-02</t>
+        </is>
+      </c>
+      <c r="M109" s="9" t="inlineStr">
+        <is>
+          <t>Keeping references consistent (rename refactoring)</t>
+        </is>
+      </c>
+      <c r="N109" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O109" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="124.15" customHeight="1" s="20">
+      <c r="A110" s="7" t="inlineStr">
+        <is>
+          <t>US-194</t>
+        </is>
+      </c>
+      <c r="B110" s="9" t="inlineStr">
+        <is>
+          <t>E18</t>
+        </is>
+      </c>
+      <c r="C110" s="9" t="inlineStr">
+        <is>
+          <t>Mechanics and story tuning with a quick check</t>
+        </is>
+      </c>
+      <c r="D110" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want needs, actions, life, social, story, calendar, professions, recipes and hero data in forms, and a quick headless run to see the effect, so that I can tune mechanics safely.</t>
+        </is>
+      </c>
+      <c r="E110" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Forms
+Given every mechanics and story file
+When the owner opens it
+Then it shows as forms
+Scenario: Quick check
+Given a changed hunger rate
+When the owner runs the 20-year check
+Then a summary shows population, deaths by cause and episodes, next to the last run
+Scenario: Determinism
+Given the same data and seed
+When the check runs twice
+Then the summaries are the same</t>
+        </is>
+      </c>
+      <c r="F110" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G110" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H110" s="9">
+        <f>VLOOKUP(G110,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I110" s="9">
+        <f>VLOOKUP(G110,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J110" s="9" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="K110" s="9" t="inlineStr">
+        <is>
+          <t>US-191</t>
+        </is>
+      </c>
+      <c r="L110" s="9" t="inlineStr">
+        <is>
+          <t>EDT-02, STO-02</t>
+        </is>
+      </c>
+      <c r="M110" s="9" t="inlineStr">
+        <is>
+          <t>Running the simulation headless from the game</t>
+        </is>
+      </c>
+      <c r="N110" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O110" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="124.15" customHeight="1" s="20">
+      <c r="A111" s="7" t="inlineStr">
+        <is>
+          <t>US-195</t>
+        </is>
+      </c>
+      <c r="B111" s="9" t="inlineStr">
+        <is>
+          <t>E18</t>
+        </is>
+      </c>
+      <c r="C111" s="9" t="inlineStr">
+        <is>
+          <t>Game Rules page</t>
+        </is>
+      </c>
+      <c r="D111" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want one page for New Game presets, comfort, victory thresholds and switches for whole systems, so that I can set up how a game plays.</t>
+        </is>
+      </c>
+      <c r="E111" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Switches
+Given weather, combat, rival clans, tutorial, markers, chronicle and politics switches
+When the owner turns weather off and starts a game
+Then no weather happens
+Scenario: Rules sets
+Given two rules files
+When a new game or a level picks one
+Then its values are used
+Scenario: Thresholds
+Given a victory threshold changed
+When a game reaches it
+Then victory follows the new value</t>
+        </is>
+      </c>
+      <c r="F111" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G111" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H111" s="9">
+        <f>VLOOKUP(G111,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I111" s="9">
+        <f>VLOOKUP(G111,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J111" s="9" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="K111" s="9" t="inlineStr">
+        <is>
+          <t>US-191</t>
+        </is>
+      </c>
+      <c r="L111" s="9" t="inlineStr">
+        <is>
+          <t>EDT-03, MVP-09</t>
+        </is>
+      </c>
+      <c r="M111" s="9" t="inlineStr">
+        <is>
+          <t>Feature flags read once at start</t>
+        </is>
+      </c>
+      <c r="N111" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O111" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="124.15" customHeight="1" s="20">
+      <c r="A112" s="7" t="inlineStr">
+        <is>
+          <t>US-196</t>
+        </is>
+      </c>
+      <c r="B112" s="9" t="inlineStr">
+        <is>
+          <t>E18</t>
+        </is>
+      </c>
+      <c r="C112" s="9" t="inlineStr">
+        <is>
+          <t>Daily routines as data</t>
+        </is>
+      </c>
+      <c r="D112" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want daily routines per role and per person (sleep, work, meals, gatherings at the fire), so that clan life has a rhythm I can shape.</t>
+        </is>
+      </c>
+      <c r="E112" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Routine
+Given the hunters' routine with work from 6 to 14
+When a day passes
+Then hunters choose work interactions in that block more often than at other times
+Scenario: Edit
+Given the Routines editor
+When the owner drags a block on the day timeline
+Then the routine file is saved and used
+Scenario: Needs win
+Given a starving hunter in a work block
+When time passes
+Then they eat first</t>
+        </is>
+      </c>
+      <c r="F112" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G112" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H112" s="9">
+        <f>VLOOKUP(G112,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I112" s="9">
+        <f>VLOOKUP(G112,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J112" s="9" t="inlineStr">
+        <is>
+          <t>M11</t>
+        </is>
+      </c>
+      <c r="K112" s="9" t="inlineStr">
+        <is>
+          <t>US-154, US-191</t>
+        </is>
+      </c>
+      <c r="L112" s="9" t="inlineStr">
+        <is>
+          <t>SDC-07, INT-05</t>
+        </is>
+      </c>
+      <c r="M112" s="9" t="inlineStr">
+        <is>
+          <t>Time blocks and weighting a utility AI</t>
+        </is>
+      </c>
+      <c r="N112" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O112" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="124.15" customHeight="1" s="20">
+      <c r="A113" s="7" t="inlineStr">
+        <is>
+          <t>US-200</t>
+        </is>
+      </c>
+      <c r="B113" s="9" t="inlineStr">
+        <is>
+          <t>E19</t>
+        </is>
+      </c>
+      <c r="C113" s="9" t="inlineStr">
+        <is>
+          <t>The region in the Editor</t>
+        </is>
+      </c>
+      <c r="D113" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to open the procedural region in the Editor with a zoomable map, so that I can work on the whole world.</t>
+        </is>
+      </c>
+      <c r="E113" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Open
+Given a seed
+When the owner opens the region
+Then it shows at any zoom from the whole 256 x 256 map to single tiles, at a smooth frame rate
+Scenario: Layers
+Given the layer switches
+When the owner hides plants and people
+Then only terrain shows
+Scenario: Same world
+Given the region opened in the Editor
+When it is compared to the game's
+Then they are identical</t>
+        </is>
+      </c>
+      <c r="F113" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G113" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H113" s="9">
+        <f>VLOOKUP(G113,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I113" s="9">
+        <f>VLOOKUP(G113,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J113" s="9" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="K113" s="9" t="inlineStr">
+        <is>
+          <t>US-040, US-123</t>
+        </is>
+      </c>
+      <c r="L113" s="9" t="inlineStr">
+        <is>
+          <t>EDT-04</t>
+        </is>
+      </c>
+      <c r="M113" s="9" t="inlineStr">
+        <is>
+          <t>Streaming chunks and level of detail</t>
+        </is>
+      </c>
+      <c r="N113" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O113" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="124.15" customHeight="1" s="20">
+      <c r="A114" s="7" t="inlineStr">
+        <is>
+          <t>US-201</t>
+        </is>
+      </c>
+      <c r="B114" s="9" t="inlineStr">
+        <is>
+          <t>E19</t>
+        </is>
+      </c>
+      <c r="C114" s="9" t="inlineStr">
+        <is>
+          <t>Generator settings with live preview</t>
+        </is>
+      </c>
+      <c r="D114" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want every generator setting in forms with a preview map, so that I can shape a region before committing to it.</t>
+        </is>
+      </c>
+      <c r="E114" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Preview
+Given the biome mix changed
+When the owner presses Preview
+Then a new map shows within a few seconds beside the old one
+Scenario: Apply
+Given a preview the owner likes
+When Apply
+Then the region and region.json use the new settings
+Scenario: Keep edits
+Given hand edits on the region
+When the settings change
+Then the edits stay and conflicts are listed</t>
+        </is>
+      </c>
+      <c r="F114" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G114" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H114" s="9">
+        <f>VLOOKUP(G114,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I114" s="9">
+        <f>VLOOKUP(G114,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J114" s="9" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="K114" s="9" t="inlineStr">
+        <is>
+          <t>US-200, US-191</t>
+        </is>
+      </c>
+      <c r="L114" s="9" t="inlineStr">
+        <is>
+          <t>EDT-04</t>
+        </is>
+      </c>
+      <c r="M114" s="9" t="inlineStr">
+        <is>
+          <t>Pure functions of a seed</t>
+        </is>
+      </c>
+      <c r="N114" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O114" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="124.15" customHeight="1" s="20">
+      <c r="A115" s="7" t="inlineStr">
+        <is>
+          <t>US-202</t>
+        </is>
+      </c>
+      <c r="B115" s="9" t="inlineStr">
+        <is>
+          <t>E19</t>
+        </is>
+      </c>
+      <c r="C115" s="9" t="inlineStr">
+        <is>
+          <t>Hand edits on top of the seed</t>
+        </is>
+      </c>
+      <c r="D115" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to paint terrain and biomes on the region and keep them on top of the seed, so that the world is generated and hand-made at once.</t>
+        </is>
+      </c>
+      <c r="E115" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Paint
+Given the brush on the region
+When the owner paints a meadow into a forest
+Then the change shows and is saved as an override of those chunks
+Scenario: Small saves
+Given 100 painted tiles
+When the region is saved
+Then the file holds the seed plus the changed tiles, not the whole map
+Scenario: Undo
+Given region edits
+When Ctrl+Z
+Then they are undone as in the level editor</t>
+        </is>
+      </c>
+      <c r="F115" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G115" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H115" s="9">
+        <f>VLOOKUP(G115,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I115" s="9">
+        <f>VLOOKUP(G115,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J115" s="9" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="K115" s="9" t="inlineStr">
+        <is>
+          <t>US-200</t>
+        </is>
+      </c>
+      <c r="L115" s="9" t="inlineStr">
+        <is>
+          <t>EDT-04, ADR-010</t>
+        </is>
+      </c>
+      <c r="M115" s="9" t="inlineStr">
+        <is>
+          <t>Storing differences (overlays) instead of copies</t>
+        </is>
+      </c>
+      <c r="N115" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O115" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="124.15" customHeight="1" s="20">
+      <c r="A116" s="7" t="inlineStr">
+        <is>
+          <t>US-203</t>
+        </is>
+      </c>
+      <c r="B116" s="9" t="inlineStr">
+        <is>
+          <t>E19</t>
+        </is>
+      </c>
+      <c r="C116" s="9" t="inlineStr">
+        <is>
+          <t>Water and mountains</t>
+        </is>
+      </c>
+      <c r="D116" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to draw and remove rivers, lakes, cliffs and caves, so that I can shape the land.</t>
+        </is>
+      </c>
+      <c r="E116" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: River
+Given the river tool
+When the owner draws a river
+Then it flows from start to end and blocks walking except at fords
+Scenario: Cave
+Given a cliff
+When the owner places a cave mouth
+Then the cave can be entered in the game
+Scenario: Remove
+Given a generated lake
+When the owner removes it
+Then land replaces it and the change is an override</t>
+        </is>
+      </c>
+      <c r="F116" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G116" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H116" s="9">
+        <f>VLOOKUP(G116,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I116" s="9">
+        <f>VLOOKUP(G116,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J116" s="9" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="K116" s="9" t="inlineStr">
+        <is>
+          <t>US-202</t>
+        </is>
+      </c>
+      <c r="L116" s="9" t="inlineStr">
+        <is>
+          <t>EDT-04</t>
+        </is>
+      </c>
+      <c r="M116" s="9" t="inlineStr">
+        <is>
+          <t>Path tools and connected areas</t>
+        </is>
+      </c>
+      <c r="N116" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O116" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="124.15" customHeight="1" s="20">
+      <c r="A117" s="7" t="inlineStr">
+        <is>
+          <t>US-204</t>
+        </is>
+      </c>
+      <c r="B117" s="9" t="inlineStr">
+        <is>
+          <t>E19</t>
+        </is>
+      </c>
+      <c r="C117" s="9" t="inlineStr">
+        <is>
+          <t>Things, people and places in the region</t>
+        </is>
+      </c>
+      <c r="D117" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to place plants, animals, objects, people and named places in the region, so that quests and stories have their spots.</t>
+        </is>
+      </c>
+      <c r="E117" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Place
+Given the palettes
+When the owner places a fire pit and an NPC
+Then they are saved as region overrides and appear in the game
+Scenario: Places
+Given a named place 'Red Cliff'
+When a quest step targets it
+Then the quest marker points to it
+Scenario: Pickers
+Given a quest or dialogue field
+When the owner picks a person or place
+Then region people and places are offered</t>
+        </is>
+      </c>
+      <c r="F117" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G117" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H117" s="9">
+        <f>VLOOKUP(G117,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I117" s="9">
+        <f>VLOOKUP(G117,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J117" s="9" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="K117" s="9" t="inlineStr">
+        <is>
+          <t>US-202, US-155</t>
+        </is>
+      </c>
+      <c r="L117" s="9" t="inlineStr">
+        <is>
+          <t>EDT-04, STO-04</t>
+        </is>
+      </c>
+      <c r="M117" s="9" t="inlineStr">
+        <is>
+          <t>Ids that survive regeneration</t>
+        </is>
+      </c>
+      <c r="N117" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O117" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="124.15" customHeight="1" s="20">
+      <c r="A118" s="7" t="inlineStr">
+        <is>
+          <t>US-205</t>
+        </is>
+      </c>
+      <c r="B118" s="9" t="inlineStr">
+        <is>
+          <t>E19</t>
+        </is>
+      </c>
+      <c r="C118" s="9" t="inlineStr">
+        <is>
+          <t>Camps and resources</t>
+        </is>
+      </c>
+      <c r="D118" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to move the player and rival camps and set resource spots and amounts, so that I control the region's balance.</t>
+        </is>
+      </c>
+      <c r="E118" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Camps
+Given a rival camp
+When the owner moves it
+Then the rival clan lives there in the game
+Scenario: Resources
+Given a flint spot
+When the owner sets it to 50
+Then 50 flint can be taken there
+Scenario: Rules
+Given a camp placed in water
+When the owner tries
+Then it is refused with the reason</t>
+        </is>
+      </c>
+      <c r="F118" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G118" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H118" s="9">
+        <f>VLOOKUP(G118,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I118" s="9">
+        <f>VLOOKUP(G118,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J118" s="9" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="K118" s="9" t="inlineStr">
+        <is>
+          <t>US-202, US-041</t>
+        </is>
+      </c>
+      <c r="L118" s="9" t="inlineStr">
+        <is>
+          <t>EDT-04, MVP-10</t>
+        </is>
+      </c>
+      <c r="M118" s="9" t="inlineStr">
+        <is>
+          <t>Validating placements against rules</t>
+        </is>
+      </c>
+      <c r="N118" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O118" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="124.15" customHeight="1" s="20">
+      <c r="A119" s="7" t="inlineStr">
+        <is>
+          <t>US-206</t>
+        </is>
+      </c>
+      <c r="B119" s="9" t="inlineStr">
+        <is>
+          <t>E19</t>
+        </is>
+      </c>
+      <c r="C119" s="9" t="inlineStr">
+        <is>
+          <t>Clans and people inspector</t>
+        </is>
+      </c>
+      <c r="D119" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to edit each clan and person in the world: members, kinship, leader, opinions and grudges, rival stance, owned items, stores, debts, trade partners, routine and allowed actions, so that I set up the social, economic and political world.</t>
+        </is>
+      </c>
+      <c r="E119" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Social
+Given two people selected
+When the owner sets their opinion to -50 and adds a grudge with a reason
+Then the game starts with that grudge and the chronicle can tell it
+Scenario: Economy
+Given a clan selected
+When the owner fills its store and adds a debt to a rival
+Then the game starts with that store and debt
+Scenario: Overrides
+Given a person selected
+When the owner removes Barter from their actions and changes their HP
+Then only that person changes</t>
+        </is>
+      </c>
+      <c r="F119" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G119" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H119" s="9">
+        <f>VLOOKUP(G119,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I119" s="9">
+        <f>VLOOKUP(G119,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J119" s="9" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="K119" s="9" t="inlineStr">
+        <is>
+          <t>US-204, US-196, US-173</t>
+        </is>
+      </c>
+      <c r="L119" s="9" t="inlineStr">
+        <is>
+          <t>EDT-05, SDC-07, PIL-08</t>
+        </is>
+      </c>
+      <c r="M119" s="9" t="inlineStr">
+        <is>
+          <t>Editing a graph of relations safely</t>
+        </is>
+      </c>
+      <c r="N119" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O119" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="124.15" customHeight="1" s="20">
+      <c r="A120" s="7" t="inlineStr">
+        <is>
+          <t>US-207</t>
+        </is>
+      </c>
+      <c r="B120" s="9" t="inlineStr">
+        <is>
+          <t>E19</t>
+        </is>
+      </c>
+      <c r="C120" s="9" t="inlineStr">
+        <is>
+          <t>Play the edited region</t>
+        </is>
+      </c>
+      <c r="D120" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to start a new game on my edited region or play it from the Editor, so that my world is the game.</t>
+        </is>
+      </c>
+      <c r="E120" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: New game
+Given an edited region saved as a world file
+When the player starts a new game from it
+Then every edit is there
+Scenario: Play here
+Given the region in the Editor
+When the owner chooses Play here
+Then the game starts on the edited region at the cursor
+Scenario: Old saves
+Given a save from before region editing
+When it loads
+Then it still works</t>
+        </is>
+      </c>
+      <c r="F120" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G120" s="9" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H120" s="9">
+        <f>VLOOKUP(G120,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I120" s="9">
+        <f>VLOOKUP(G120,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J120" s="9" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="K120" s="9" t="inlineStr">
+        <is>
+          <t>US-206, US-186</t>
+        </is>
+      </c>
+      <c r="L120" s="9" t="inlineStr">
+        <is>
+          <t>EDT-04, EDT-06</t>
+        </is>
+      </c>
+      <c r="M120" s="9" t="inlineStr">
+        <is>
+          <t>Versioned save formats</t>
+        </is>
+      </c>
+      <c r="N120" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O120" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="124.15" customHeight="1" s="20">
+      <c r="A121" s="7" t="inlineStr">
+        <is>
+          <t>US-210</t>
+        </is>
+      </c>
+      <c r="B121" s="9" t="inlineStr">
+        <is>
+          <t>E20</t>
+        </is>
+      </c>
+      <c r="C121" s="9" t="inlineStr">
+        <is>
+          <t>The political model</t>
+        </is>
+      </c>
+      <c r="D121" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want clans as political actors with relations, alliances, vassal ties and a Politics share of the region, all as editable data, so that politics is part of the simulation.</t>
+        </is>
+      </c>
+      <c r="E121" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Relations
+Given three clans
+When the simulation runs
+Then each pair has a stance from -100 to 100 that moves with events, with reasons
+Scenario: Share
+Given one rival a vassal of the player's clan
+When the dominion screen opens
+Then Politics shows that clan's share of the region's people
+Scenario: Data
+Given politics.json
+When the owner opens it in the Data tab
+Then every political rule is a form</t>
+        </is>
+      </c>
+      <c r="F121" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G121" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H121" s="9">
+        <f>VLOOKUP(G121,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I121" s="9">
+        <f>VLOOKUP(G121,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J121" s="9" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="K121" s="9" t="inlineStr">
+        <is>
+          <t>US-206, US-195</t>
+        </is>
+      </c>
+      <c r="L121" s="9" t="inlineStr">
+        <is>
+          <t>PIL-03, PIL-08</t>
+        </is>
+      </c>
+      <c r="M121" s="9" t="inlineStr">
+        <is>
+          <t>Modelling relations between groups</t>
+        </is>
+      </c>
+      <c r="N121" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O121" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="124.15" customHeight="1" s="20">
+      <c r="A122" s="7" t="inlineStr">
+        <is>
+          <t>US-211</t>
+        </is>
+      </c>
+      <c r="B122" s="9" t="inlineStr">
+        <is>
+          <t>E20</t>
+        </is>
+      </c>
+      <c r="C122" s="9" t="inlineStr">
+        <is>
+          <t>Alliances and vassal oaths</t>
+        </is>
+      </c>
+      <c r="D122" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want to ally with clans, take tribute and make them swear vassal oaths, which can break, so that I can bind the region to my clan.</t>
+        </is>
+      </c>
+      <c r="E122" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Alliance
+Given a rival with a good stance
+When the hero proposes an alliance
+Then it is accepted or refused with a reason
+Scenario: Oath
+Given an allied clan that is weaker and indebted
+When the hero asks for a vassal oath
+Then it swears and pays tribute each season
+Scenario: Break
+Given a vassal whose stance falls below its limit
+When a season passes
+Then it may break the oath, and the chronicle says why</t>
+        </is>
+      </c>
+      <c r="F122" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G122" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H122" s="9">
+        <f>VLOOKUP(G122,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I122" s="9">
+        <f>VLOOKUP(G122,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J122" s="9" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="K122" s="9" t="inlineStr">
+        <is>
+          <t>US-210</t>
+        </is>
+      </c>
+      <c r="L122" s="9" t="inlineStr">
+        <is>
+          <t>PIL-03, PIL-08</t>
+        </is>
+      </c>
+      <c r="M122" s="9" t="inlineStr">
+        <is>
+          <t>Contracts as data with conditions</t>
+        </is>
+      </c>
+      <c r="N122" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O122" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="124.15" customHeight="1" s="20">
+      <c r="A123" s="7" t="inlineStr">
+        <is>
+          <t>US-212</t>
+        </is>
+      </c>
+      <c r="B123" s="9" t="inlineStr">
+        <is>
+          <t>E20</t>
+        </is>
+      </c>
+      <c r="C123" s="9" t="inlineStr">
+        <is>
+          <t>Elders' council</t>
+        </is>
+      </c>
+      <c r="D123" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want clan decisions voted by the elders and to sway them, so that leading a clan means persuading people.</t>
+        </is>
+      </c>
+      <c r="E123" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Vote
+Given a decision to move camp
+When the council meets
+Then each elder votes by needs, traits and opinion, and the result is shown
+Scenario: Sway
+Given the hero talks to an elder before the vote
+When a persuasion choice succeeds
+Then that elder's vote changes
+Scenario: Record
+Given a council decision
+When it is taken
+Then the chronicle records it with the votes</t>
+        </is>
+      </c>
+      <c r="F123" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G123" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H123" s="9">
+        <f>VLOOKUP(G123,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I123" s="9">
+        <f>VLOOKUP(G123,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J123" s="9" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="K123" s="9" t="inlineStr">
+        <is>
+          <t>US-210</t>
+        </is>
+      </c>
+      <c r="L123" s="9" t="inlineStr">
+        <is>
+          <t>PIL-08, SDC-02</t>
+        </is>
+      </c>
+      <c r="M123" s="9" t="inlineStr">
+        <is>
+          <t>Simple voting rules and weights</t>
+        </is>
+      </c>
+      <c r="N123" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O123" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="124.15" customHeight="1" s="20">
+      <c r="A124" s="7" t="inlineStr">
+        <is>
+          <t>US-213</t>
+        </is>
+      </c>
+      <c r="B124" s="9" t="inlineStr">
+        <is>
+          <t>E20</t>
+        </is>
+      </c>
+      <c r="C124" s="9" t="inlineStr">
+        <is>
+          <t>Marriage ties</t>
+        </is>
+      </c>
+      <c r="D124" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want marriages between clans to bind them, so that love and politics meet.</t>
+        </is>
+      </c>
+      <c r="E124" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Tie
+Given a courtship between two clans' members
+When they marry
+Then the clans' stance rises and a marriage tie is recorded
+Scenario: Alliance
+Given a marriage tie
+When an alliance is proposed
+Then acceptance is more likely
+Scenario: Parting
+Given a married couple parts
+When it happens
+Then the tie weakens and the stance falls</t>
+        </is>
+      </c>
+      <c r="F124" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G124" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H124" s="9">
+        <f>VLOOKUP(G124,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I124" s="9">
+        <f>VLOOKUP(G124,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J124" s="9" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="K124" s="9" t="inlineStr">
+        <is>
+          <t>US-210, US-113</t>
+        </is>
+      </c>
+      <c r="L124" s="9" t="inlineStr">
+        <is>
+          <t>PIL-08, SDC-02</t>
+        </is>
+      </c>
+      <c r="M124" s="9" t="inlineStr">
+        <is>
+          <t>Events that affect two systems</t>
+        </is>
+      </c>
+      <c r="N124" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O124" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="124.15" customHeight="1" s="20">
+      <c r="A125" s="7" t="inlineStr">
+        <is>
+          <t>US-214</t>
+        </is>
+      </c>
+      <c r="B125" s="9" t="inlineStr">
+        <is>
+          <t>E20</t>
+        </is>
+      </c>
+      <c r="C125" s="9" t="inlineStr">
+        <is>
+          <t>Leadership challenges</t>
+        </is>
+      </c>
+      <c r="D125" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want leaders to be challenged when their people turn against them, and to challenge or back a leader myself, so that power can change hands.</t>
+        </is>
+      </c>
+      <c r="E125" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Challenge
+Given a leader whose clan opinion is below the limit
+When time passes
+Then a challenger rises and the council or a contest decides
+Scenario: Hero
+Given the hero with enough support
+When the hero challenges the leader
+Then the outcome follows the rules and the chronicle tells it
+Scenario: Succession
+Given a leader dies
+When it happens
+Then succession is contested between candidates with reasons</t>
+        </is>
+      </c>
+      <c r="F125" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G125" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H125" s="9">
+        <f>VLOOKUP(G125,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I125" s="9">
+        <f>VLOOKUP(G125,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J125" s="9" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="K125" s="9" t="inlineStr">
+        <is>
+          <t>US-212</t>
+        </is>
+      </c>
+      <c r="L125" s="9" t="inlineStr">
+        <is>
+          <t>PIL-08</t>
+        </is>
+      </c>
+      <c r="M125" s="9" t="inlineStr">
+        <is>
+          <t>State transitions with guards</t>
+        </is>
+      </c>
+      <c r="N125" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O125" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="124.15" customHeight="1" s="20">
+      <c r="A126" s="7" t="inlineStr">
+        <is>
+          <t>US-215</t>
+        </is>
+      </c>
+      <c r="B126" s="9" t="inlineStr">
+        <is>
+          <t>E20</t>
+        </is>
+      </c>
+      <c r="C126" s="9" t="inlineStr">
+        <is>
+          <t>Economic and technological levers</t>
+        </is>
+      </c>
+      <c r="D126" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want trade pacts, tribute in goods, embargoes and sharing crafts with allies as political tools, so that wealth and know-how buy influence.</t>
+        </is>
+      </c>
+      <c r="E126" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Pact
+Given two allied clans
+When a trade pact is made
+Then barter between them is cheaper and stance rises
+Scenario: Embargo
+Given a rival under embargo
+When it tries to trade with the hero's allies
+Then it is refused and stance falls
+Scenario: Know-how
+Given the hero teaches an ally a recipe
+When it happens
+Then the ally can craft it and its stance and dependence rise</t>
+        </is>
+      </c>
+      <c r="F126" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G126" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H126" s="9">
+        <f>VLOOKUP(G126,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I126" s="9">
+        <f>VLOOKUP(G126,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J126" s="9" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="K126" s="9" t="inlineStr">
+        <is>
+          <t>US-211, US-062</t>
+        </is>
+      </c>
+      <c r="L126" s="9" t="inlineStr">
+        <is>
+          <t>PIL-08, PIL-02</t>
+        </is>
+      </c>
+      <c r="M126" s="9" t="inlineStr">
+        <is>
+          <t>Interfaces between subsystems</t>
+        </is>
+      </c>
+      <c r="N126" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O126" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="124.15" customHeight="1" s="20">
+      <c r="A127" s="7" t="inlineStr">
+        <is>
+          <t>US-216</t>
+        </is>
+      </c>
+      <c r="B127" s="9" t="inlineStr">
+        <is>
+          <t>E20</t>
+        </is>
+      </c>
+      <c r="C127" s="9" t="inlineStr">
+        <is>
+          <t>Political victory and diplomacy</t>
+        </is>
+      </c>
+      <c r="D127" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want to win the region through Politics and to do diplomacy in conversation, so that Politics is a full path to victory.</t>
+        </is>
+      </c>
+      <c r="E127" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Victory
+Given vassals holding 60% of the region's people (Game Rules value)
+When the share is reached
+Then the game ends in a Political victory with the chronicle
+Scenario: Combined
+Given Trade, Religion and Politics shares
+When they reach the combined threshold
+Then victory follows the Game Rules
+Scenario: Diplomacy
+Given a clan leader
+When the hero talks to them
+Then alliance, oath, pact and embargo choices are offered in the conversation</t>
+        </is>
+      </c>
+      <c r="F127" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G127" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H127" s="9">
+        <f>VLOOKUP(G127,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I127" s="9">
+        <f>VLOOKUP(G127,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J127" s="9" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="K127" s="9" t="inlineStr">
+        <is>
+          <t>US-211, US-195, US-161</t>
+        </is>
+      </c>
+      <c r="L127" s="9" t="inlineStr">
+        <is>
+          <t>PIL-03, PIL-08, MVP-08, MVP-09</t>
+        </is>
+      </c>
+      <c r="M127" s="9" t="inlineStr">
+        <is>
+          <t>Combining scores from several systems</t>
+        </is>
+      </c>
+      <c r="N127" s="9" t="inlineStr">
+        <is>
+          <t>Authoring tools and Politics (owner, 2026-10-01, D-40)</t>
+        </is>
+      </c>
+      <c r="O127" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="124.15" customHeight="1" s="20">
+      <c r="A128" s="7" t="inlineStr">
+        <is>
+          <t>US-220</t>
+        </is>
+      </c>
+      <c r="B128" s="9" t="inlineStr">
+        <is>
+          <t>E21</t>
+        </is>
+      </c>
+      <c r="C128" s="9" t="inlineStr">
+        <is>
+          <t>The tech tree as data</t>
+        </is>
+      </c>
+      <c r="D128" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want Age 1 technologies with prerequisites, discovery rules and unlocks in a data file shown as a tree in the Editor, so that I can design how know-how grows.</t>
+        </is>
+      </c>
+      <c r="E128" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Load
+Given technologies.json with fire mastery, hafted spears, sewing and ochre
+When the game starts
+Then each technology's prerequisites and unlocks (recipes, interactions, professions, objects) are known
+Scenario: Editor
+Given the tech tree view
+When the owner adds a technology and links it after another
+Then the tree and the saved file show it
+Scenario: Cycle
+Given two technologies that require each other
+When validation runs
+Then the cycle is listed</t>
+        </is>
+      </c>
+      <c r="F128" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G128" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H128" s="9">
+        <f>VLOOKUP(G128,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I128" s="9">
+        <f>VLOOKUP(G128,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J128" s="9" t="inlineStr">
+        <is>
+          <t>M14</t>
+        </is>
+      </c>
+      <c r="K128" s="9" t="inlineStr">
+        <is>
+          <t>US-191, US-170, D-41</t>
+        </is>
+      </c>
+      <c r="L128" s="9" t="inlineStr">
+        <is>
+          <t>PIL-05, PIL-09, EDT-02</t>
+        </is>
+      </c>
+      <c r="M128" s="9" t="inlineStr">
+        <is>
+          <t>Directed acyclic graphs and topological order</t>
+        </is>
+      </c>
+      <c r="N128" s="9" t="inlineStr">
+        <is>
+          <t>Technology pillar (owner, 2026-10-01, D-41)</t>
+        </is>
+      </c>
+      <c r="O128" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="124.15" customHeight="1" s="20">
+      <c r="A129" s="7" t="inlineStr">
+        <is>
+          <t>US-221</t>
+        </is>
+      </c>
+      <c r="B129" s="9" t="inlineStr">
+        <is>
+          <t>E21</t>
+        </is>
+      </c>
+      <c r="C129" s="9" t="inlineStr">
+        <is>
+          <t>Research by doing</t>
+        </is>
+      </c>
+      <c r="D129" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want my clan to discover technologies by using skills and materials, so that progress grows out of daily life.</t>
+        </is>
+      </c>
+      <c r="E129" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Discover
+Given a clan that knaps flint every day
+When enough research has built up
+Then the next flint technology is discovered and its recipes unlock
+Scenario: Chronicle
+Given a discovery
+When it happens
+Then the chronicle says who discovered it and how
+Scenario: Locked
+Given a technology whose prerequisite is unknown
+When the work happens
+Then it is not discovered</t>
+        </is>
+      </c>
+      <c r="F129" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G129" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H129" s="9">
+        <f>VLOOKUP(G129,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I129" s="9">
+        <f>VLOOKUP(G129,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J129" s="9" t="inlineStr">
+        <is>
+          <t>M14</t>
+        </is>
+      </c>
+      <c r="K129" s="9" t="inlineStr">
+        <is>
+          <t>US-220</t>
+        </is>
+      </c>
+      <c r="L129" s="9" t="inlineStr">
+        <is>
+          <t>PIL-09</t>
+        </is>
+      </c>
+      <c r="M129" s="9" t="inlineStr">
+        <is>
+          <t>Accumulators and thresholds</t>
+        </is>
+      </c>
+      <c r="N129" s="9" t="inlineStr">
+        <is>
+          <t>Technology pillar (owner, 2026-10-01, D-41)</t>
+        </is>
+      </c>
+      <c r="O129" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="124.15" customHeight="1" s="20">
+      <c r="A130" s="7" t="inlineStr">
+        <is>
+          <t>US-222</t>
+        </is>
+      </c>
+      <c r="B130" s="9" t="inlineStr">
+        <is>
+          <t>E21</t>
+        </is>
+      </c>
+      <c r="C130" s="9" t="inlineStr">
+        <is>
+          <t>Workshops, inventors and teaching</t>
+        </is>
+      </c>
+      <c r="D130" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want workshops and inventive people to speed research and teaching to spread knowledge, so that who works where matters.</t>
+        </is>
+      </c>
+      <c r="E130" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Workshop
+Given knapping at a knapping stone versus in the open
+When a day passes
+Then the workshop gives more research, by the data's factor
+Scenario: Inventor
+Given an NPC with the inventive trait
+When they work
+Then they add research faster and can discover alone
+Scenario: Teach
+Given a known technology
+When a member teaches another clan's member (an ally)
+Then that clan knows it after the teaching time</t>
+        </is>
+      </c>
+      <c r="F130" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G130" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H130" s="9">
+        <f>VLOOKUP(G130,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I130" s="9">
+        <f>VLOOKUP(G130,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J130" s="9" t="inlineStr">
+        <is>
+          <t>M14</t>
+        </is>
+      </c>
+      <c r="K130" s="9" t="inlineStr">
+        <is>
+          <t>US-221, US-155</t>
+        </is>
+      </c>
+      <c r="L130" s="9" t="inlineStr">
+        <is>
+          <t>PIL-09, US-215</t>
+        </is>
+      </c>
+      <c r="M130" s="9" t="inlineStr">
+        <is>
+          <t>Modifiers that stack in a defined order</t>
+        </is>
+      </c>
+      <c r="N130" s="9" t="inlineStr">
+        <is>
+          <t>Technology pillar (owner, 2026-10-01, D-41)</t>
+        </is>
+      </c>
+      <c r="O130" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="124.15" customHeight="1" s="20">
+      <c r="A131" s="7" t="inlineStr">
+        <is>
+          <t>US-223</t>
+        </is>
+      </c>
+      <c r="B131" s="9" t="inlineStr">
+        <is>
+          <t>E21</t>
+        </is>
+      </c>
+      <c r="C131" s="9" t="inlineStr">
+        <is>
+          <t>Espionage, theft and secrets</t>
+        </is>
+      </c>
+      <c r="D131" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want rivals to steal or copy know-how and to guard my own, so that knowledge is power to protect.</t>
+        </is>
+      </c>
+      <c r="E131" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Steal
+Given a rival watching our workshop or trading with us
+When time passes
+Then it may learn one of our technologies, and stance falls if caught
+Scenario: Guard
+Given a technology marked secret
+When a rival tries to learn it
+Then the chance is lower and secret-keepers can catch the spy
+Scenario: Repeat
+Given the same seed and inputs
+When two runs
+Then the same thefts happen</t>
+        </is>
+      </c>
+      <c r="F131" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G131" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H131" s="9">
+        <f>VLOOKUP(G131,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I131" s="9">
+        <f>VLOOKUP(G131,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J131" s="9" t="inlineStr">
+        <is>
+          <t>M14</t>
+        </is>
+      </c>
+      <c r="K131" s="9" t="inlineStr">
+        <is>
+          <t>US-222, US-210</t>
+        </is>
+      </c>
+      <c r="L131" s="9" t="inlineStr">
+        <is>
+          <t>PIL-09, PIL-08</t>
+        </is>
+      </c>
+      <c r="M131" s="9" t="inlineStr">
+        <is>
+          <t>Probabilities from a seeded stream</t>
+        </is>
+      </c>
+      <c r="N131" s="9" t="inlineStr">
+        <is>
+          <t>Technology pillar (owner, 2026-10-01, D-41)</t>
+        </is>
+      </c>
+      <c r="O131" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="124.15" customHeight="1" s="20">
+      <c r="A132" s="7" t="inlineStr">
+        <is>
+          <t>US-224</t>
+        </is>
+      </c>
+      <c r="B132" s="9" t="inlineStr">
+        <is>
+          <t>E21</t>
+        </is>
+      </c>
+      <c r="C132" s="9" t="inlineStr">
+        <is>
+          <t>Rival research and the Technology share</t>
+        </is>
+      </c>
+      <c r="D132" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want rival clans to research too and to see who leads in know-how, so that Technology is a race.</t>
+        </is>
+      </c>
+      <c r="E132" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Rivals
+Given two rival clans
+When a year passes
+Then each has discovered technologies by its own priorities
+Scenario: Share
+Given the dominion screen
+When the player opens it
+Then Technology shows each clan's share of the Age 1 technologies known
+Scenario: Data
+Given rival priorities
+When the owner edits them in forms
+Then rivals follow the new priorities</t>
+        </is>
+      </c>
+      <c r="F132" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G132" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H132" s="9">
+        <f>VLOOKUP(G132,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I132" s="9">
+        <f>VLOOKUP(G132,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J132" s="9" t="inlineStr">
+        <is>
+          <t>M14</t>
+        </is>
+      </c>
+      <c r="K132" s="9" t="inlineStr">
+        <is>
+          <t>US-221</t>
+        </is>
+      </c>
+      <c r="L132" s="9" t="inlineStr">
+        <is>
+          <t>PIL-09, ENV-10</t>
+        </is>
+      </c>
+      <c r="M132" s="9" t="inlineStr">
+        <is>
+          <t>Comparing scores across actors</t>
+        </is>
+      </c>
+      <c r="N132" s="9" t="inlineStr">
+        <is>
+          <t>Technology pillar (owner, 2026-10-01, D-41)</t>
+        </is>
+      </c>
+      <c r="O132" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="124.15" customHeight="1" s="20">
+      <c r="A133" s="7" t="inlineStr">
+        <is>
+          <t>US-225</t>
+        </is>
+      </c>
+      <c r="B133" s="9" t="inlineStr">
+        <is>
+          <t>E21</t>
+        </is>
+      </c>
+      <c r="C133" s="9" t="inlineStr">
+        <is>
+          <t>The Ember Strand and Technology victory</t>
+        </is>
+      </c>
+      <c r="D133" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want to forge the Ember Strand at the end of a long chain of discoveries and win when I hold it and lead in know-how, so that Technology is a full path to victory.</t>
+        </is>
+      </c>
+      <c r="E133" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Chain
+Given the Ember chain in technologies.json and recipes.json
+When the clan discovers every step and gathers the materials
+Then the Ember Strand can be forged at the sacred fire
+Scenario: Victory
+Given the Ember Strand held and a Technology share at or above the Game Rules value (60%)
+When both are true
+Then the game ends in a Technology victory with the chronicle
+Scenario: Rival forges
+Given a rival forges Ember first
+When it happens
+Then the chronicle tells it and the player can still win another way or take it</t>
+        </is>
+      </c>
+      <c r="F133" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G133" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H133" s="9">
+        <f>VLOOKUP(G133,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I133" s="9">
+        <f>VLOOKUP(G133,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J133" s="9" t="inlineStr">
+        <is>
+          <t>M14</t>
+        </is>
+      </c>
+      <c r="K133" s="9" t="inlineStr">
+        <is>
+          <t>US-224, US-195, US-062</t>
+        </is>
+      </c>
+      <c r="L133" s="9" t="inlineStr">
+        <is>
+          <t>PIL-05, PIL-09, MVP-08, MVP-09</t>
+        </is>
+      </c>
+      <c r="M133" s="9" t="inlineStr">
+        <is>
+          <t>Long multi-step goals as data</t>
+        </is>
+      </c>
+      <c r="N133" s="9" t="inlineStr">
+        <is>
+          <t>Technology pillar (owner, 2026-10-01, D-41)</t>
+        </is>
+      </c>
+      <c r="O133" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="124.15" customHeight="1" s="20">
+      <c r="A134" s="7" t="inlineStr">
+        <is>
+          <t>US-226</t>
+        </is>
+      </c>
+      <c r="B134" s="9" t="inlineStr">
+        <is>
+          <t>E21</t>
+        </is>
+      </c>
+      <c r="C134" s="9" t="inlineStr">
+        <is>
+          <t>The technology screen</t>
+        </is>
+      </c>
+      <c r="D134" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want a screen with what my clan knows, what is next and what each discovery unlocks, so that I can plan research.</t>
+        </is>
+      </c>
+      <c r="E134" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Tree
+Given a clan with some technologies
+When the player opens the screen
+Then known, reachable and locked technologies are shown as a tree
+Scenario: Detail
+Given a technology selected
+When it is shown
+Then its discovery rule, progress and unlocks are listed
+Scenario: Secrets
+Given a technology marked secret
+When it is shown
+Then who else is known to have it is listed</t>
+        </is>
+      </c>
+      <c r="F134" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G134" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H134" s="9">
+        <f>VLOOKUP(G134,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I134" s="9">
+        <f>VLOOKUP(G134,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J134" s="9" t="inlineStr">
+        <is>
+          <t>M14</t>
+        </is>
+      </c>
+      <c r="K134" s="9" t="inlineStr">
+        <is>
+          <t>US-220</t>
+        </is>
+      </c>
+      <c r="L134" s="9" t="inlineStr">
+        <is>
+          <t>PIL-09, PIL-07</t>
+        </is>
+      </c>
+      <c r="M134" s="9" t="inlineStr">
+        <is>
+          <t>Laying out a tree for reading</t>
+        </is>
+      </c>
+      <c r="N134" s="9" t="inlineStr">
+        <is>
+          <t>Technology pillar (owner, 2026-10-01, D-41)</t>
+        </is>
+      </c>
+      <c r="O134" s="16" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
@@ -12704,7 +16828,7 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Ages 2-10, Mythic Strands, Phase 2 space</t>
+          <t>Ages 2-10, Mythic Strands 2-10, Phase 2 space</t>
         </is>
       </c>
       <c r="B6" s="9" t="inlineStr">
@@ -12738,17 +16862,17 @@
     <row r="8" ht="25.5" customHeight="1" s="20">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Military, Politics, Technology, Ideology pillars</t>
+          <t>Military, Ideology pillars</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Two pillars are enough to test 'many paths to dominance'; combat is the most expensive system.</t>
+          <t>Four pillars (Trade, Religion, Politics, Technology) are enough to test 'many paths to dominance'; combat as a pillar is the most expensive system. Politics (D-40) and Technology (D-41) returned to the MVP on 2026-10-01.</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Next (Politics), Later (others)</t>
+          <t>Later</t>
         </is>
       </c>
     </row>
@@ -12885,7 +17009,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -12921,7 +17044,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Codex v2.2: sync from Anima; requirements v2.4 and M8b-M8e brief
Codex v2.2 (P-011, M8b-M8e between M8 and M9, Charter rule 11, D-06/D-42/D-43), requirements v2.4 and backlog mirrored from Drive, the M8b-M8e brief, changelog.
</commit_message>
<xml_diff>
--- a/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
+++ b/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
@@ -654,7 +654,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Working tracker for developers. The source of truth is Project Odyssey.docx v2.2, chapter 12; this workbook is generated from the same data. Updated 2026-10-01: M10-M14 added (D-40, D-41).</t>
+          <t>Working tracker for developers. The source of truth is Project Odyssey.docx v2.4, chapter 12; this workbook is generated from the same data. Updated 2026-10-01: M8d split into M8d and M8e (D-43); D-06 decided.</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="20" min="1" max="1"/>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Layered 32 x 48 sprites with 3 outfits per body; programmer or placeholder art allowed; minimal sound effects.</t>
+          <t>Layered 32 x 48 sprites with 3 outfits per body; programmer or placeholder art allowed; minimal sound effects. From M8b: 960x540 on the SDL_GPU renderer with global lighting and shadows (D-42).</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
@@ -1271,72 +1271,77 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25" ht="51" customHeight="1" s="20">
-      <c r="A25" s="5" t="inlineStr">
+    <row r="24" ht="38.25" customHeight="1" s="20">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>MVP-16</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Buildings and light</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>960x540 on the GPU renderer; day, night, seasons and weather lighting; fire light; shadows from the sun, the moon and nearby fires; buildings from blueprints and pieces, built by the hero and the clans, with wear, repair, fire, interiors and Editor prefabs (D-42).</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>ENV-18..ENV-21, ARC-11, INT-07, INT-08, EDT-07, ADR-021</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="51" customHeight="1" s="20"/>
+    <row r="26" ht="63.75" customHeight="1" s="20">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Success and kill criteria (decided before building)</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="63.75" customHeight="1" s="20">
-      <c r="A26" s="6" t="inlineStr">
+    <row r="27" ht="38.25" customHeight="1" s="20">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>How measured</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>Gate</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="38.25" customHeight="1" s="20">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>Voluntary play time</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>5 of 8 playtesters play 30+ minutes without being asked to continue</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
-        <is>
-          <t>Observation + local session log (US-092)</t>
-        </is>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>M6</t>
         </is>
       </c>
     </row>
     <row r="28" ht="63.75" customHeight="1" s="20">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Emergent story</t>
+          <t>Voluntary play time</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>3 of 8 can retell a story that came from the simulation, not from a script</t>
+          <t>5 of 8 playtesters play 30+ minutes without being asked to continue</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Post-play interview</t>
+          <t>Observation + local session log (US-092)</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
@@ -1348,108 +1353,130 @@
     <row r="29" ht="51" customHeight="1" s="20">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Chronicle interest (early)</t>
+          <t>Emergent story</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>2 of 3 readers find a story in the console chronicle</t>
+          <t>3 of 8 can retell a story that came from the simulation, not from a script</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Show printed chronicle (M2: 3 readers, failed 2026-09-30; M2b retry: the owner reads and judges)</t>
+          <t>Post-play interview</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>M2, retried at M2b</t>
+          <t>M6</t>
         </is>
       </c>
     </row>
     <row r="30" ht="51" customHeight="1" s="20">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Frame rate</t>
+          <t>Chronicle interest (early)</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>60 FPS with 500 simulated agents in the region on the minimum PC (OPEN-19)</t>
+          <t>2 of 3 readers find a story in the console chronicle</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>FPS overlay (US-082)</t>
+          <t>Show printed chronicle (M2: 3 readers, failed 2026-09-30; M2b retry: the owner reads and judges)</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M2, retried at M2b</t>
         </is>
       </c>
     </row>
     <row r="31" ht="63.75" customHeight="1" s="20">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Determinism</t>
+          <t>Frame rate</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>Same seed + inputs give the same world hash after 10,000 ticks</t>
+          <t>60 FPS with 500 simulated agents in the region on the minimum PC (OPEN-19)</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>Automated test in CI</t>
+          <t>FPS overlay (US-082)</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>M2 onwards</t>
+          <t>M5</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Stability</t>
+          <t>Determinism</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>No crash in a 2-hour play session or a 100-year soak test</t>
+          <t>Same seed + inputs give the same world hash after 10,000 ticks</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Soak test + crash log</t>
+          <t>Automated test in CI</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>M5, M6</t>
+          <t>M2 onwards</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
+          <t>Stability</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>No crash in a 2-hour play session or a 100-year soak test</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>Soak test + crash log</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>M5, M6</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
           <t>Kill / pivot rule</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>If M2 or M6 fails: stop adding content; redesign the simulation or the loop first</t>
         </is>
       </c>
-      <c r="C33" s="9" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>Owner decision, recorded</t>
         </is>
       </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>M2, M6</t>
         </is>
@@ -1477,7 +1504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:IA31"/>
+  <dimension ref="A1:JO36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -1632,6 +1659,46 @@
     <col width="13" customWidth="1" style="20" min="233" max="233"/>
     <col width="13" customWidth="1" style="20" min="234" max="234"/>
     <col width="13" customWidth="1" style="20" min="235" max="235"/>
+    <col width="13" customWidth="1" style="20" min="236" max="236"/>
+    <col width="13" customWidth="1" style="20" min="237" max="237"/>
+    <col width="13" customWidth="1" style="20" min="238" max="238"/>
+    <col width="13" customWidth="1" style="20" min="239" max="239"/>
+    <col width="13" customWidth="1" style="20" min="240" max="240"/>
+    <col width="13" customWidth="1" style="20" min="241" max="241"/>
+    <col width="13" customWidth="1" style="20" min="242" max="242"/>
+    <col width="13" customWidth="1" style="20" min="243" max="243"/>
+    <col width="13" customWidth="1" style="20" min="244" max="244"/>
+    <col width="13" customWidth="1" style="20" min="245" max="245"/>
+    <col width="13" customWidth="1" style="20" min="246" max="246"/>
+    <col width="13" customWidth="1" style="20" min="247" max="247"/>
+    <col width="13" customWidth="1" style="20" min="248" max="248"/>
+    <col width="13" customWidth="1" style="20" min="249" max="249"/>
+    <col width="13" customWidth="1" style="20" min="250" max="250"/>
+    <col width="13" customWidth="1" style="20" min="251" max="251"/>
+    <col width="13" customWidth="1" style="20" min="252" max="252"/>
+    <col width="13" customWidth="1" style="20" min="253" max="253"/>
+    <col width="13" customWidth="1" style="20" min="254" max="254"/>
+    <col width="13" customWidth="1" style="20" min="255" max="255"/>
+    <col width="13" customWidth="1" style="20" min="256" max="256"/>
+    <col width="13" customWidth="1" style="20" min="257" max="257"/>
+    <col width="13" customWidth="1" style="20" min="258" max="258"/>
+    <col width="13" customWidth="1" style="20" min="259" max="259"/>
+    <col width="13" customWidth="1" style="20" min="260" max="260"/>
+    <col width="13" customWidth="1" style="20" min="261" max="261"/>
+    <col width="13" customWidth="1" style="20" min="262" max="262"/>
+    <col width="13" customWidth="1" style="20" min="263" max="263"/>
+    <col width="13" customWidth="1" style="20" min="264" max="264"/>
+    <col width="13" customWidth="1" style="20" min="265" max="265"/>
+    <col width="13" customWidth="1" style="20" min="266" max="266"/>
+    <col width="13" customWidth="1" style="20" min="267" max="267"/>
+    <col width="13" customWidth="1" style="20" min="268" max="268"/>
+    <col width="13" customWidth="1" style="20" min="269" max="269"/>
+    <col width="13" customWidth="1" style="20" min="270" max="270"/>
+    <col width="13" customWidth="1" style="20" min="271" max="271"/>
+    <col width="13" customWidth="1" style="20" min="272" max="272"/>
+    <col width="13" customWidth="1" style="20" min="273" max="273"/>
+    <col width="13" customWidth="1" style="20" min="274" max="274"/>
+    <col width="13" customWidth="1" style="20" min="275" max="275"/>
   </cols>
   <sheetData>
     <row r="1" ht="20.25" customHeight="1" s="20">
@@ -2389,6 +2456,126 @@
       <c r="IA6" s="12" t="n">
         <v>220</v>
       </c>
+      <c r="IB6" s="12" t="n">
+        <v>221</v>
+      </c>
+      <c r="IC6" s="12" t="n">
+        <v>222</v>
+      </c>
+      <c r="ID6" s="12" t="n">
+        <v>223</v>
+      </c>
+      <c r="IE6" s="12" t="n">
+        <v>224</v>
+      </c>
+      <c r="IF6" s="12" t="n">
+        <v>225</v>
+      </c>
+      <c r="IG6" s="12" t="n">
+        <v>226</v>
+      </c>
+      <c r="IH6" s="12" t="n">
+        <v>227</v>
+      </c>
+      <c r="II6" s="12" t="n">
+        <v>228</v>
+      </c>
+      <c r="IJ6" s="12" t="n">
+        <v>229</v>
+      </c>
+      <c r="IK6" s="12" t="n">
+        <v>230</v>
+      </c>
+      <c r="IL6" s="12" t="n">
+        <v>231</v>
+      </c>
+      <c r="IM6" s="12" t="n">
+        <v>232</v>
+      </c>
+      <c r="IN6" s="12" t="n">
+        <v>233</v>
+      </c>
+      <c r="IO6" s="12" t="n">
+        <v>234</v>
+      </c>
+      <c r="IP6" s="12" t="n">
+        <v>235</v>
+      </c>
+      <c r="IQ6" s="12" t="n">
+        <v>236</v>
+      </c>
+      <c r="IR6" s="12" t="n">
+        <v>237</v>
+      </c>
+      <c r="IS6" s="12" t="n">
+        <v>238</v>
+      </c>
+      <c r="IT6" s="12" t="n">
+        <v>239</v>
+      </c>
+      <c r="IU6" s="12" t="n">
+        <v>240</v>
+      </c>
+      <c r="IV6" s="12" t="n">
+        <v>241</v>
+      </c>
+      <c r="IW6" s="12" t="n">
+        <v>242</v>
+      </c>
+      <c r="IX6" s="12" t="n">
+        <v>243</v>
+      </c>
+      <c r="IY6" s="12" t="n">
+        <v>244</v>
+      </c>
+      <c r="IZ6" s="12" t="n">
+        <v>245</v>
+      </c>
+      <c r="JA6" s="12" t="n">
+        <v>246</v>
+      </c>
+      <c r="JB6" s="12" t="n">
+        <v>247</v>
+      </c>
+      <c r="JC6" s="12" t="n">
+        <v>248</v>
+      </c>
+      <c r="JD6" s="12" t="n">
+        <v>249</v>
+      </c>
+      <c r="JE6" s="12" t="n">
+        <v>250</v>
+      </c>
+      <c r="JF6" s="12" t="n">
+        <v>251</v>
+      </c>
+      <c r="JG6" s="12" t="n">
+        <v>252</v>
+      </c>
+      <c r="JH6" s="12" t="n">
+        <v>253</v>
+      </c>
+      <c r="JI6" s="12" t="n">
+        <v>254</v>
+      </c>
+      <c r="JJ6" s="12" t="n">
+        <v>255</v>
+      </c>
+      <c r="JK6" s="12" t="n">
+        <v>256</v>
+      </c>
+      <c r="JL6" s="12" t="n">
+        <v>257</v>
+      </c>
+      <c r="JM6" s="12" t="n">
+        <v>258</v>
+      </c>
+      <c r="JN6" s="12" t="n">
+        <v>259</v>
+      </c>
+      <c r="JO6" s="12" t="n">
+        <v>260</v>
+      </c>
     </row>
     <row r="7" ht="42" customHeight="1" s="20">
       <c r="A7" s="7" t="inlineStr">
@@ -3112,12 +3299,12 @@
     <row r="19" ht="25.5" customHeight="1" s="20">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>M9</t>
+          <t>M8b</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Interaction and dialogue editor</t>
+          <t>Resolution and GPU renderer</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -3126,10 +3313,10 @@
         </is>
       </c>
       <c r="D19" s="13" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E19" s="13" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F19" s="9">
         <f>ROUND((D19+E19)/2,0)</f>
@@ -3165,19 +3352,19 @@
       </c>
       <c r="N19" s="9" t="inlineStr">
         <is>
-          <t>The owner opens any dialogue or interaction in the Editor as a graph, edits it, test-plays it and saves it, and the file still reads well in a text editor.</t>
+          <t>The game renders at 960x540 through Luna's SDL_GPU renderer (with the old renderer as fallback) and looks the same at 2x camera zoom; windowed sizes, borderless and exclusive full screen work; every screen and editor panel is laid out for the new size; the frame budget holds.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="25.5" customHeight="1" s="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M8c</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Quests and story authoring</t>
+          <t>Lighting and shadows</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -3189,7 +3376,7 @@
         <v>9</v>
       </c>
       <c r="E20" s="13" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F20" s="9">
         <f>ROUND((D20+E20)/2,0)</f>
@@ -3225,19 +3412,19 @@
       </c>
       <c r="N20" s="9" t="inlineStr">
         <is>
-          <t>The owner writes a quest in the Editor's graph (or offline in JSON), test-plays it with the debugger and saves it; a player gets it from an NPC, follows it in the journal, tracker and markers, and finishes it; the elder tutorial is a quest and crossroads events are edited as story events.</t>
+          <t>The world is lit by the sun and moon through the day and the seasons, by fires, torches and effects at night, and dimmed by weather; sprites are shaded with generated normal maps; characters, plants and buildings cast shadows from the sun, the moon and nearby fires; the Editor previews any time of day.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="25.5" customHeight="1" s="20">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M8d</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Data editors</t>
+          <t>Buildings</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -3246,10 +3433,10 @@
         </is>
       </c>
       <c r="D21" s="13" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E21" s="13" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F21" s="9">
         <f>ROUND((D21+E21)/2,0)</f>
@@ -3285,19 +3472,19 @@
       </c>
       <c r="N21" s="9" t="inlineStr">
         <is>
-          <t>Every data file has a schema; the owner edits any entity, mechanic, story tuning value, game rule and daily routine in Editor forms with pickers and validation, and the running game reloads it.</t>
+          <t>The hero builds from blueprints and piece by piece on a building grid, and rooms form; the owner composes prefabs from pieces in the Editor and places them in levels; prefabs marked buildable are offered as blueprints.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="25.5" customHeight="1" s="20">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>M12</t>
+          <t>M8e</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>World editing</t>
+          <t>Building life</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -3306,10 +3493,10 @@
         </is>
       </c>
       <c r="D22" s="13" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E22" s="13" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="F22" s="9">
         <f>ROUND((D22+E22)/2,0)</f>
@@ -3345,19 +3532,19 @@
       </c>
       <c r="N22" s="9" t="inlineStr">
         <is>
-          <t>The owner opens the procedural region in the Editor, tunes the generator with a live preview, paints terrain, water and mountains, places things, people and camps, and edits each clan's and person's relations, economy, routines and actions; edits are saved on top of the seed and a new game plays them.</t>
+          <t>Clan members help build and rival clans build; each building fades its roof or opens an interior map as set in the Editor; buildings wear, are repaired, take damage, burn and fall; they shelter, warm and store for the clan and are saved.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="25.5" customHeight="1" s="20">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>M13</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Politics</t>
+          <t>Interaction and dialogue editor</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -3366,10 +3553,10 @@
         </is>
       </c>
       <c r="D23" s="13" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E23" s="13" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F23" s="9">
         <f>ROUND((D23+E23)/2,0)</f>
@@ -3405,19 +3592,19 @@
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Clans form alliances and vassal oaths, hold elders' councils, bind themselves by marriage, challenge leaders and use trade and craft knowledge as levers; the player can win the region through Politics; every political rule is editable in the Editor.</t>
+          <t>The owner opens any dialogue or interaction in the Editor as a graph, edits it, test-plays it and saves it, and the file still reads well in a text editor.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="25.5" customHeight="1" s="20">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>M14</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Quests and story authoring</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
@@ -3465,19 +3652,19 @@
       </c>
       <c r="N24" s="9" t="inlineStr">
         <is>
-          <t>Clans research by doing in workshops with inventors, pass knowledge by teaching, steal and guard secrets, and unlock recipes, interactions and professions from an editable tech tree; the player can win by forging the Ember Strand while leading in known technologies.</t>
+          <t>The owner writes a quest in the Editor's graph (or offline in JSON), test-plays it with the debugger and saves it; a player gets it from an NPC, follows it in the journal, tracker and markers, and finishes it; the elder tutorial is a quest and crossroads events are edited as story events.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="25.5" customHeight="1" s="20">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>M11</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>Playtest and go/no-go (KILL GATE 2)</t>
+          <t>Data editors</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -3486,10 +3673,10 @@
         </is>
       </c>
       <c r="D25" s="13" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E25" s="13" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="F25" s="9">
         <f>ROUND((D25+E25)/2,0)</f>
@@ -3525,116 +3712,357 @@
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
+          <t>Every data file has a schema; the owner edits any entity, mechanic, story tuning value, game rule and daily routine in Editor forms with pickers and validation, and the running game reloads it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="25.5" customHeight="1" s="20">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>M12</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>World editing</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D26" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="E26" s="13" t="n">
+        <v>21</v>
+      </c>
+      <c r="F26" s="9">
+        <f>ROUND((D26+E26)/2,0)</f>
+        <v/>
+      </c>
+      <c r="G26" s="9">
+        <f>H25+1</f>
+        <v/>
+      </c>
+      <c r="H26" s="9">
+        <f>G26+F26-1</f>
+        <v/>
+      </c>
+      <c r="I26" s="14">
+        <f>$B$4+(G26-1)*7</f>
+        <v/>
+      </c>
+      <c r="J26" s="14">
+        <f>$B$4+H26*7-1</f>
+        <v/>
+      </c>
+      <c r="K26" s="14">
+        <f>$B$4+SUM($D$7:D26)*7-1</f>
+        <v/>
+      </c>
+      <c r="L26" s="14">
+        <f>$B$4+SUM($E$7:E26)*7-1</f>
+        <v/>
+      </c>
+      <c r="M26" s="9">
+        <f>SUMIFS('User Stories'!$H$5:$H$200,'User Stories'!$J$5:$J$200,A26,'User Stories'!$F$5:$F$200,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$200,'User Stories'!$J$5:$J$200,A26,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="N26" s="9" t="inlineStr">
+        <is>
+          <t>The owner opens the procedural region in the Editor, tunes the generator with a live preview, paints terrain, water and mountains, places things, people and camps, and edits each clan's and person's relations, economy, routines and actions; edits are saved on top of the seed and a new game plays them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="25.5" customHeight="1" s="20">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="E27" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="F27" s="9">
+        <f>ROUND((D27+E27)/2,0)</f>
+        <v/>
+      </c>
+      <c r="G27" s="9">
+        <f>H26+1</f>
+        <v/>
+      </c>
+      <c r="H27" s="9">
+        <f>G27+F27-1</f>
+        <v/>
+      </c>
+      <c r="I27" s="14">
+        <f>$B$4+(G27-1)*7</f>
+        <v/>
+      </c>
+      <c r="J27" s="14">
+        <f>$B$4+H27*7-1</f>
+        <v/>
+      </c>
+      <c r="K27" s="14">
+        <f>$B$4+SUM($D$7:D27)*7-1</f>
+        <v/>
+      </c>
+      <c r="L27" s="14">
+        <f>$B$4+SUM($E$7:E27)*7-1</f>
+        <v/>
+      </c>
+      <c r="M27" s="9">
+        <f>SUMIFS('User Stories'!$H$5:$H$200,'User Stories'!$J$5:$J$200,A27,'User Stories'!$F$5:$F$200,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$200,'User Stories'!$J$5:$J$200,A27,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="N27" s="9" t="inlineStr">
+        <is>
+          <t>Clans form alliances and vassal oaths, hold elders' councils, bind themselves by marriage, challenge leaders and use trade and craft knowledge as levers; the player can win the region through Politics; every political rule is editable in the Editor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="25.5" customHeight="1" s="20">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>M14</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D28" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="E28" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="F28" s="9">
+        <f>ROUND((D28+E28)/2,0)</f>
+        <v/>
+      </c>
+      <c r="G28" s="9">
+        <f>H27+1</f>
+        <v/>
+      </c>
+      <c r="H28" s="9">
+        <f>G28+F28-1</f>
+        <v/>
+      </c>
+      <c r="I28" s="14">
+        <f>$B$4+(G28-1)*7</f>
+        <v/>
+      </c>
+      <c r="J28" s="14">
+        <f>$B$4+H28*7-1</f>
+        <v/>
+      </c>
+      <c r="K28" s="14">
+        <f>$B$4+SUM($D$7:D28)*7-1</f>
+        <v/>
+      </c>
+      <c r="L28" s="14">
+        <f>$B$4+SUM($E$7:E28)*7-1</f>
+        <v/>
+      </c>
+      <c r="M28" s="9">
+        <f>SUMIFS('User Stories'!$H$5:$H$200,'User Stories'!$J$5:$J$200,A28,'User Stories'!$F$5:$F$200,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$200,'User Stories'!$J$5:$J$200,A28,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="N28" s="9" t="inlineStr">
+        <is>
+          <t>Clans research by doing in workshops with inventors, pass knowledge by teaching, steal and guard secrets, and unlock recipes, interactions and professions from an editable tech tree; the player can win by forging the Ember Strand while leading in known technologies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="25.5" customHeight="1" s="20">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Playtest and go/no-go (KILL GATE 2)</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E29" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="F29" s="9">
+        <f>ROUND((D29+E29)/2,0)</f>
+        <v/>
+      </c>
+      <c r="G29" s="9">
+        <f>H28+1</f>
+        <v/>
+      </c>
+      <c r="H29" s="9">
+        <f>G29+F29-1</f>
+        <v/>
+      </c>
+      <c r="I29" s="14">
+        <f>$B$4+(G29-1)*7</f>
+        <v/>
+      </c>
+      <c r="J29" s="14">
+        <f>$B$4+H29*7-1</f>
+        <v/>
+      </c>
+      <c r="K29" s="14">
+        <f>$B$4+SUM($D$7:D29)*7-1</f>
+        <v/>
+      </c>
+      <c r="L29" s="14">
+        <f>$B$4+SUM($E$7:E29)*7-1</f>
+        <v/>
+      </c>
+      <c r="M29" s="9">
+        <f>SUMIFS('User Stories'!$H$5:$H$200,'User Stories'!$J$5:$J$200,A29,'User Stories'!$F$5:$F$200,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$200,'User Stories'!$J$5:$J$200,A29,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="N29" s="9" t="inlineStr">
+        <is>
           <t>8 outside playtesters play; success criteria measured; go/no-go decision recorded. Held after M14 (owner, 2026-10-01, D-41).</t>
         </is>
       </c>
     </row>
-    <row r="26" s="20">
-      <c r="A26" s="7" t="n"/>
-      <c r="B26" s="7" t="inlineStr">
+    <row r="30" s="20">
+      <c r="A30" s="7" t="n"/>
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>MVP total</t>
         </is>
       </c>
-      <c r="C26" s="7" t="n"/>
-      <c r="D26" s="7">
-        <f>SUM(D7:D25)</f>
-        <v/>
-      </c>
-      <c r="E26" s="7">
-        <f>SUM(E7:E25)</f>
-        <v/>
-      </c>
-      <c r="F26" s="7">
-        <f>SUM(F7:F25)</f>
-        <v/>
-      </c>
-      <c r="G26" s="7" t="n"/>
-      <c r="H26" s="7">
-        <f>H25</f>
-        <v/>
-      </c>
-      <c r="I26" s="15">
+      <c r="C30" s="7" t="n"/>
+      <c r="D30" s="7">
+        <f>SUM(D7:D29)</f>
+        <v/>
+      </c>
+      <c r="E30" s="7">
+        <f>SUM(E7:E29)</f>
+        <v/>
+      </c>
+      <c r="F30" s="7">
+        <f>SUM(F7:F29)</f>
+        <v/>
+      </c>
+      <c r="G30" s="7" t="n"/>
+      <c r="H30" s="7">
+        <f>H29</f>
+        <v/>
+      </c>
+      <c r="I30" s="15">
         <f>I7</f>
         <v/>
       </c>
-      <c r="J26" s="15">
-        <f>J25</f>
-        <v/>
-      </c>
-      <c r="K26" s="15">
-        <f>K25</f>
-        <v/>
-      </c>
-      <c r="L26" s="15">
-        <f>L25</f>
-        <v/>
-      </c>
-      <c r="M26" s="7" t="n"/>
-      <c r="N26" s="7" t="inlineStr">
+      <c r="J30" s="15">
+        <f>J29</f>
+        <v/>
+      </c>
+      <c r="K30" s="15">
+        <f>K29</f>
+        <v/>
+      </c>
+      <c r="L30" s="15">
+        <f>L29</f>
+        <v/>
+      </c>
+      <c r="M30" s="7" t="n"/>
+      <c r="N30" s="7" t="inlineStr">
         <is>
           <t>Months (likely) = weeks / 4.33</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="27.95" customHeight="1" s="20">
-      <c r="A27" s="7" t="n"/>
-      <c r="B27" s="7" t="inlineStr">
+    <row r="31" ht="27.95" customHeight="1" s="20">
+      <c r="A31" s="7" t="n"/>
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>In months</t>
         </is>
       </c>
-      <c r="C27" s="7" t="n"/>
-      <c r="D27" s="7">
-        <f>ROUND(D26/4.33,1)</f>
-        <v/>
-      </c>
-      <c r="E27" s="7">
-        <f>ROUND(E26/4.33,1)</f>
-        <v/>
-      </c>
-      <c r="F27" s="7">
-        <f>ROUND(F26/4.33,1)</f>
-        <v/>
-      </c>
-      <c r="G27" s="7" t="n"/>
-      <c r="H27" s="7" t="n"/>
-      <c r="I27" s="7" t="n"/>
-      <c r="J27" s="7" t="n"/>
-      <c r="K27" s="7" t="n"/>
-      <c r="L27" s="7" t="n"/>
-      <c r="M27" s="7" t="n"/>
-      <c r="N27" s="7" t="n"/>
-    </row>
-    <row r="28" ht="27.95" customHeight="1" s="20"/>
-    <row r="29" ht="27.95" customHeight="1" s="20">
-      <c r="B29" s="19" t="inlineStr">
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="7">
+        <f>ROUND(D30/4.33,1)</f>
+        <v/>
+      </c>
+      <c r="E31" s="7">
+        <f>ROUND(E30/4.33,1)</f>
+        <v/>
+      </c>
+      <c r="F31" s="7">
+        <f>ROUND(F30/4.33,1)</f>
+        <v/>
+      </c>
+      <c r="G31" s="7" t="n"/>
+      <c r="H31" s="7" t="n"/>
+      <c r="I31" s="7" t="n"/>
+      <c r="J31" s="7" t="n"/>
+      <c r="K31" s="7" t="n"/>
+      <c r="L31" s="7" t="n"/>
+      <c r="M31" s="7" t="n"/>
+      <c r="N31" s="7" t="n"/>
+    </row>
+    <row r="32" ht="27.95" customHeight="1" s="20"/>
+    <row r="33" ht="27.95" customHeight="1" s="20">
+      <c r="B33" s="19" t="inlineStr">
         <is>
           <t>Why the estimate grew: the learning path (requirements, section 8.3) estimated 9-13 months top-down. The bottom-up sum of the MVP stories is higher; this sheet uses the bottom-up figure.</t>
         </is>
       </c>
     </row>
-    <row r="30" s="20">
-      <c r="B30" s="19" t="inlineStr">
+    <row r="34" s="20">
+      <c r="B34" s="19" t="inlineStr">
         <is>
           <t>Buffer: the 'Should' stories are the cut list if time runs short. Cutting all of them saves about 5-11 weeks.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="102" customHeight="1" s="20">
-      <c r="B31" s="19" t="inlineStr">
-        <is>
-          <t>Kill gates: M2 (is the console chronicle interesting? failed 2026-09-30, passed at the M2b retry) and M6 (do playtesters stay?), held after M14 (D-41). Critical path: M0 &gt; M1 &gt; M1b &gt; M2 &gt; M2b &gt; M2c &gt; M2d &gt; M3 &gt; M4 &gt; M5 &gt; M7 &gt; M8 &gt; M9 &gt; M10 &gt; M11 &gt; M12 &gt; M13 &gt; M14 &gt; M6. Dates of M2c onwards are not re-planned yet.</t>
-        </is>
-      </c>
-    </row>
+    <row r="35" ht="102" customHeight="1" s="20">
+      <c r="B35" s="19" t="inlineStr">
+        <is>
+          <t>Kill gates: M2 (failed 2026-09-30, passed at the M2b retry) and M6 (do playtesters stay?), held after M14 (D-41). Critical path: M0 &gt; M1 &gt; M1b &gt; M2 &gt; M2b &gt; M2c &gt; M2d &gt; M3 &gt; M4 &gt; M5 &gt; M7 &gt; M8 &gt; M8b &gt; M8c &gt; M8d &gt; M8e &gt; M9 &gt; M10 &gt; M11 &gt; M12 &gt; M13 &gt; M14 &gt; M6. Dates of M2c onwards are not re-planned yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B31:N31"/>
-    <mergeCell ref="B30:N30"/>
-    <mergeCell ref="B29:N29"/>
+    <mergeCell ref="B35:N35"/>
+    <mergeCell ref="B34:N34"/>
+    <mergeCell ref="B33:N33"/>
   </mergeCells>
-  <conditionalFormatting sqref="P7:IA25">
+  <conditionalFormatting sqref="P7:JO29">
     <cfRule type="expression" priority="1" dxfId="10">
       <formula>AND(P$6&gt;=$G7,P$6&lt;=$H7)</formula>
     </cfRule>
@@ -3649,7 +4077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -3905,7 +4333,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Minimum PC spec (OPEN-19)</t>
+          <t>Minimum PC spec (OPEN-19). Mid-range PC (owner, 2026-10-01): 6-core CPU, 16 GB RAM, RX 6600 / RTX 3060 class GPU (8 GB) with DirectX 12, Windows 10/11; 60 FPS at 1080p on High lighting, Low for weaker PCs. Development PC: RX 7900 XTX, 32 GB RAM, 6-core CPU.</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -3915,12 +4343,12 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M8b</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>US-082</t>
+          <t>US-082, US-234</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
@@ -3930,7 +4358,7 @@
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided</t>
         </is>
       </c>
     </row>
@@ -4238,7 +4666,7 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Technical chain: M0 &gt; M1 &gt; M1b &gt; M2 &gt; M2b &gt; M2c &gt; M2d &gt; M3 &gt; M4 &gt; M5 &gt; M7 &gt; M8 &gt; M9 &gt; M10 &gt; M11 &gt; M12 &gt; M13 &gt; M14 &gt; M6 (each milestone needs the previous one)</t>
+          <t>Technical chain: M0 &gt; M1 &gt; M1b &gt; M2 &gt; M2b &gt; M2c &gt; M2d &gt; M3 &gt; M4 &gt; M5 &gt; M7 &gt; M8 &gt; M8b &gt; M8c &gt; M8d &gt; M8e &gt; M9 &gt; M10 &gt; M11 &gt; M12 &gt; M13 &gt; M14 &gt; M6 (each milestone needs the previous one)</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
@@ -4595,6 +5023,80 @@
         </is>
       </c>
       <c r="G28" s="16" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="25.5" customHeight="1" s="20">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>D-42</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (Round 16): 960x540 with window modes, camera zoom, UI scale; SDL_GPU shaders; sun, moon, fire, torch and effect lights, seasonal day length, weather light; shadows from sun, moon and nearby fires; generated normal maps; buildings from blueprints and pieces, clans build, wear, repair, fire; interiors per building (roof fade or interior map); prefabs in the Editor; M8b, M8c, M8d right after M8</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>Design decision</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>M8b</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>US-230..US-257</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G29" s="16" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="25.5" customHeight="1" s="20">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>D-43</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Assembly of M8b-M8e (Round 17): M8d split into M8d Buildings (US-250, 251, 252, 256) and M8e Building life (US-253, 254, 255, 257); US-256 no longer waits for US-254; M7-M9 assembly rules (D-35) apply; D-06 answered</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Design decision</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>M8b</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>US-230..US-257</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G30" s="16" t="inlineStr">
         <is>
           <t>Decided</t>
         </is>
@@ -4630,7 +5132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -5722,37 +6224,221 @@
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="7" t="n"/>
-      <c r="B27" s="7" t="inlineStr">
+    <row r="27" ht="25.5" customHeight="1" s="20">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>E22</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Resolution and GPU renderer</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>The game renders at 960x540 on Luna's new SDL_GPU renderer, in any window size or full screen, and every screen and editor has room to breathe.</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>M8b</t>
+        </is>
+      </c>
+      <c r="E27" s="9">
+        <f>COUNTIF('User Stories'!$B$5:$B$200,A27)</f>
+        <v/>
+      </c>
+      <c r="F27" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A27,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="G27" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A27,'User Stories'!$H$5:$H$200)</f>
+        <v/>
+      </c>
+      <c r="H27" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A27,'User Stories'!$I$5:$I$200)</f>
+        <v/>
+      </c>
+      <c r="I27" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A27,'User Stories'!$O$5:$O$200,"Done")</f>
+        <v/>
+      </c>
+      <c r="J27" s="17">
+        <f>IFERROR(I27/E27,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="25.5" customHeight="1" s="20">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>E23</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Lighting and shadows</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Days and nights, seasons and weather light the world; fires glow; characters, plants and buildings cast shadows that move with the sun, the moon and nearby fires.</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>M8c</t>
+        </is>
+      </c>
+      <c r="E28" s="9">
+        <f>COUNTIF('User Stories'!$B$5:$B$200,A28)</f>
+        <v/>
+      </c>
+      <c r="F28" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A28,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="G28" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A28,'User Stories'!$H$5:$H$200)</f>
+        <v/>
+      </c>
+      <c r="H28" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A28,'User Stories'!$I$5:$I$200)</f>
+        <v/>
+      </c>
+      <c r="I28" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A28,'User Stories'!$O$5:$O$200,"Done")</f>
+        <v/>
+      </c>
+      <c r="J28" s="17">
+        <f>IFERROR(I28/E28,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="25.5" customHeight="1" s="20">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>E24</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Buildings</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>The hero builds from whole blueprints and piece by piece; the owner composes pre-made buildings in the Editor and places them.</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>M8d</t>
+        </is>
+      </c>
+      <c r="E29" s="9">
+        <f>COUNTIF('User Stories'!$B$5:$B$200,A29)</f>
+        <v/>
+      </c>
+      <c r="F29" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A29,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="G29" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A29,'User Stories'!$H$5:$H$200)</f>
+        <v/>
+      </c>
+      <c r="H29" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A29,'User Stories'!$I$5:$I$200)</f>
+        <v/>
+      </c>
+      <c r="I29" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A29,'User Stories'!$O$5:$O$200,"Done")</f>
+        <v/>
+      </c>
+      <c r="J29" s="17">
+        <f>IFERROR(I29/E29,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="25.5" customHeight="1" s="20">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>E25</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Building life</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Clans build together; interiors by roof fade or interior map; wear, repair, damage and fire; shelter, warmth and storage for the clan.</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>M8e</t>
+        </is>
+      </c>
+      <c r="E30" s="9">
+        <f>COUNTIF('User Stories'!$B$5:$B$200,A30)</f>
+        <v/>
+      </c>
+      <c r="F30" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A30,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="G30" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A30,'User Stories'!$H$5:$H$200)</f>
+        <v/>
+      </c>
+      <c r="H30" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A30,'User Stories'!$I$5:$I$200)</f>
+        <v/>
+      </c>
+      <c r="I30" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A30,'User Stories'!$O$5:$O$200,"Done")</f>
+        <v/>
+      </c>
+      <c r="J30" s="17">
+        <f>IFERROR(I30/E30,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="n"/>
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C27" s="7" t="n"/>
-      <c r="D27" s="7" t="n"/>
-      <c r="E27" s="7">
-        <f>SUM(E5:E26)</f>
-        <v/>
-      </c>
-      <c r="F27" s="7">
-        <f>SUM(F5:F26)</f>
-        <v/>
-      </c>
-      <c r="G27" s="7">
-        <f>SUM(G5:G26)</f>
-        <v/>
-      </c>
-      <c r="H27" s="7">
-        <f>SUM(H5:H26)</f>
-        <v/>
-      </c>
-      <c r="I27" s="7">
-        <f>SUM(I5:I26)</f>
-        <v/>
-      </c>
-      <c r="J27" s="18">
-        <f>IFERROR(I27/E27,0)</f>
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="7" t="n"/>
+      <c r="E31" s="7">
+        <f>SUM(E5:E30)</f>
+        <v/>
+      </c>
+      <c r="F31" s="7">
+        <f>SUM(F5:F30)</f>
+        <v/>
+      </c>
+      <c r="G31" s="7">
+        <f>SUM(G5:G30)</f>
+        <v/>
+      </c>
+      <c r="H31" s="7">
+        <f>SUM(H5:H30)</f>
+        <v/>
+      </c>
+      <c r="I31" s="7">
+        <f>SUM(I5:I30)</f>
+        <v/>
+      </c>
+      <c r="J31" s="18">
+        <f>IFERROR(I31/E31,0)</f>
         <v/>
       </c>
     </row>
@@ -5767,7 +6453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O134"/>
+  <dimension ref="A1:O155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="20" min="1" max="1"/>
@@ -12597,7 +13283,7 @@
       </c>
       <c r="O86" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -12683,7 +13369,7 @@
       </c>
       <c r="O87" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -12769,7 +13455,7 @@
       </c>
       <c r="O88" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -16724,6 +17410,1812 @@
         </is>
       </c>
       <c r="O134" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="124.15" customHeight="1" s="20">
+      <c r="A135" s="7" t="inlineStr">
+        <is>
+          <t>US-230</t>
+        </is>
+      </c>
+      <c r="B135" s="9" t="inlineStr">
+        <is>
+          <t>E22</t>
+        </is>
+      </c>
+      <c r="C135" s="9" t="inlineStr">
+        <is>
+          <t>Luna's SDL_GPU renderer</t>
+        </is>
+      </c>
+      <c r="D135" s="9" t="inlineStr">
+        <is>
+          <t>As the developer, I want Luna to draw through SDL_GPU with shaders, keeping the old renderer as a fallback, so that lighting and shadows become possible without changing game code.</t>
+        </is>
+      </c>
+      <c r="E135" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Same picture
+Given the demo level and the camp
+When they are drawn with the GPU and the old renderer
+Then the screenshots match pixel for pixel at 1x lighting
+Scenario: Fallback
+Given a PC where SDL_GPU cannot start
+When the game starts
+Then it uses the old renderer, says so in the log and plays
+Scenario: Game code
+Given every draw call in src/game/
+When the switch is made
+Then no game file changed its drawing code</t>
+        </is>
+      </c>
+      <c r="F135" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G135" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H135" s="9">
+        <f>VLOOKUP(G135,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I135" s="9">
+        <f>VLOOKUP(G135,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J135" s="9" t="inlineStr">
+        <is>
+          <t>M8b</t>
+        </is>
+      </c>
+      <c r="K135" s="9" t="inlineStr">
+        <is>
+          <t>US-020, D-42</t>
+        </is>
+      </c>
+      <c r="L135" s="9" t="inlineStr">
+        <is>
+          <t>ARC-11, ADR-021, ADR-003</t>
+        </is>
+      </c>
+      <c r="M135" s="9" t="inlineStr">
+        <is>
+          <t>Graphics pipelines, shaders and sprite batching</t>
+        </is>
+      </c>
+      <c r="N135" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O135" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="124.15" customHeight="1" s="20">
+      <c r="A136" s="7" t="inlineStr">
+        <is>
+          <t>US-231</t>
+        </is>
+      </c>
+      <c r="B136" s="9" t="inlineStr">
+        <is>
+          <t>E22</t>
+        </is>
+      </c>
+      <c r="C136" s="9" t="inlineStr">
+        <is>
+          <t>960x540 and window modes</t>
+        </is>
+      </c>
+      <c r="D136" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want the game at 960x540 that fills my screen crisply in a window or full screen, so that it looks sharp on any monitor.</t>
+        </is>
+      </c>
+      <c r="E136" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Scale
+Given a 1920x1080 and a 3840x2160 screen
+When the game runs full screen
+Then it scales by 2 and by 4 with no blur and no border
+Scenario: Modes
+Given the settings screen
+When the player picks windowed (with sizes), borderless or exclusive full screen
+Then the mode changes at once and is saved
+Scenario: Odd sizes
+Given a 2560x1440 screen
+When the game runs
+Then it scales by 2 with a thin border, or fills the screen smoothly if the player chooses Fill</t>
+        </is>
+      </c>
+      <c r="F136" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G136" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H136" s="9">
+        <f>VLOOKUP(G136,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I136" s="9">
+        <f>VLOOKUP(G136,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J136" s="9" t="inlineStr">
+        <is>
+          <t>M8b</t>
+        </is>
+      </c>
+      <c r="K136" s="9" t="inlineStr">
+        <is>
+          <t>US-230, US-081</t>
+        </is>
+      </c>
+      <c r="L136" s="9" t="inlineStr">
+        <is>
+          <t>ENV-18, US-081</t>
+        </is>
+      </c>
+      <c r="M136" s="9" t="inlineStr">
+        <is>
+          <t>Viewports and scaling maths</t>
+        </is>
+      </c>
+      <c r="N136" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O136" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="124.15" customHeight="1" s="20">
+      <c r="A137" s="7" t="inlineStr">
+        <is>
+          <t>US-232</t>
+        </is>
+      </c>
+      <c r="B137" s="9" t="inlineStr">
+        <is>
+          <t>E22</t>
+        </is>
+      </c>
+      <c r="C137" s="9" t="inlineStr">
+        <is>
+          <t>Camera zoom and UI scale</t>
+        </is>
+      </c>
+      <c r="D137" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want to zoom the world and size the interface, so that I can see more of the land or read more easily.</t>
+        </is>
+      </c>
+      <c r="E137" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Zoom
+Given the default camera zoom of 2x
+When the player zooms out
+Then the view shows 1x (30 x 17 tiles) and back, around the hero
+Scenario: UI
+Given UI scale 1x and 2x
+When the player switches
+Then panels, the font and the hotbar resize and stay crisp
+Scenario: Pointer
+Given any zoom
+When the player aims and clicks
+Then the pointer hits the same world spot as before</t>
+        </is>
+      </c>
+      <c r="F137" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G137" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H137" s="9">
+        <f>VLOOKUP(G137,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I137" s="9">
+        <f>VLOOKUP(G137,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J137" s="9" t="inlineStr">
+        <is>
+          <t>M8b</t>
+        </is>
+      </c>
+      <c r="K137" s="9" t="inlineStr">
+        <is>
+          <t>US-231</t>
+        </is>
+      </c>
+      <c r="L137" s="9" t="inlineStr">
+        <is>
+          <t>ENV-18</t>
+        </is>
+      </c>
+      <c r="M137" s="9" t="inlineStr">
+        <is>
+          <t>Two coordinate systems: world and screen</t>
+        </is>
+      </c>
+      <c r="N137" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O137" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="124.15" customHeight="1" s="20">
+      <c r="A138" s="7" t="inlineStr">
+        <is>
+          <t>US-233</t>
+        </is>
+      </c>
+      <c r="B138" s="9" t="inlineStr">
+        <is>
+          <t>E22</t>
+        </is>
+      </c>
+      <c r="C138" s="9" t="inlineStr">
+        <is>
+          <t>Every screen at the new size</t>
+        </is>
+      </c>
+      <c r="D138" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want every screen, panel and editor laid out for 960x540, so that nothing is cramped or out of place.</t>
+        </is>
+      </c>
+      <c r="E138" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Screens
+Given the HUD, hotbar, menus, the run screens, the dialogue panel and the Editor's tool bar, palettes and properties
+When they are opened at 960x540
+Then they use the space, nothing overlaps and the text is legible
+Scenario: Tests
+Given the screenshot tests
+When they run
+Then they pass with the new reference pictures, reviewed by the owner
+Scenario: Old saves
+Given a save and a level from before
+When they load
+Then they play the same</t>
+        </is>
+      </c>
+      <c r="F138" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G138" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H138" s="9">
+        <f>VLOOKUP(G138,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I138" s="9">
+        <f>VLOOKUP(G138,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J138" s="9" t="inlineStr">
+        <is>
+          <t>M8b</t>
+        </is>
+      </c>
+      <c r="K138" s="9" t="inlineStr">
+        <is>
+          <t>US-232</t>
+        </is>
+      </c>
+      <c r="L138" s="9" t="inlineStr">
+        <is>
+          <t>ENV-18, EDT-01</t>
+        </is>
+      </c>
+      <c r="M138" s="9" t="inlineStr">
+        <is>
+          <t>Layout from data instead of fixed numbers</t>
+        </is>
+      </c>
+      <c r="N138" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O138" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="124.15" customHeight="1" s="20">
+      <c r="A139" s="7" t="inlineStr">
+        <is>
+          <t>US-234</t>
+        </is>
+      </c>
+      <c r="B139" s="9" t="inlineStr">
+        <is>
+          <t>E22</t>
+        </is>
+      </c>
+      <c r="C139" s="9" t="inlineStr">
+        <is>
+          <t>Frame budget at the new size</t>
+        </is>
+      </c>
+      <c r="D139" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want the game smooth at 960x540, so that the bigger picture costs nothing in feel.</t>
+        </is>
+      </c>
+      <c r="E139" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Budget
+Given 500 simulated people in the region on the minimum PC (D-06)
+When the game runs for 10 minutes
+Then it holds 60 FPS
+Scenario: Overlay
+Given F3
+When it is pressed
+Then the overlay shows CPU and GPU frame times
+Scenario: Record
+Given the performance run
+When it ends
+Then its numbers are saved in docs/evidence/</t>
+        </is>
+      </c>
+      <c r="F139" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G139" s="9" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H139" s="9">
+        <f>VLOOKUP(G139,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I139" s="9">
+        <f>VLOOKUP(G139,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J139" s="9" t="inlineStr">
+        <is>
+          <t>M8b</t>
+        </is>
+      </c>
+      <c r="K139" s="9" t="inlineStr">
+        <is>
+          <t>US-233, D-06</t>
+        </is>
+      </c>
+      <c r="L139" s="9" t="inlineStr">
+        <is>
+          <t>NFR-03, MVP success criteria</t>
+        </is>
+      </c>
+      <c r="M139" s="9" t="inlineStr">
+        <is>
+          <t>Measuring GPU and CPU time</t>
+        </is>
+      </c>
+      <c r="N139" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O139" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="124.15" customHeight="1" s="20">
+      <c r="A140" s="7" t="inlineStr">
+        <is>
+          <t>US-240</t>
+        </is>
+      </c>
+      <c r="B140" s="9" t="inlineStr">
+        <is>
+          <t>E23</t>
+        </is>
+      </c>
+      <c r="C140" s="9" t="inlineStr">
+        <is>
+          <t>The lighting pipeline</t>
+        </is>
+      </c>
+      <c r="D140" s="9" t="inlineStr">
+        <is>
+          <t>As the developer, I want a lit pass with ambient light, point lights and normal maps in the GPU renderer, so that the world can be lit from data.</t>
+        </is>
+      </c>
+      <c r="E140" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Ambient
+Given an ambient colour in lights.json
+When the scene is drawn
+Then every sprite is tinted by it
+Scenario: Point light
+Given a light with a colour, radius and strength
+When it is placed near a sprite
+Then the sprite's lit side faces the light, using its normal map
+Scenario: Budget
+Given 64 lights on screen
+When the scene is drawn
+Then the frame budget of US-234 still holds</t>
+        </is>
+      </c>
+      <c r="F140" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G140" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H140" s="9">
+        <f>VLOOKUP(G140,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I140" s="9">
+        <f>VLOOKUP(G140,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J140" s="9" t="inlineStr">
+        <is>
+          <t>M8c</t>
+        </is>
+      </c>
+      <c r="K140" s="9" t="inlineStr">
+        <is>
+          <t>US-230</t>
+        </is>
+      </c>
+      <c r="L140" s="9" t="inlineStr">
+        <is>
+          <t>ENV-19, ADR-021</t>
+        </is>
+      </c>
+      <c r="M140" s="9" t="inlineStr">
+        <is>
+          <t>Shader inputs, uniform data and lighting maths</t>
+        </is>
+      </c>
+      <c r="N140" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O140" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="124.15" customHeight="1" s="20">
+      <c r="A141" s="7" t="inlineStr">
+        <is>
+          <t>US-241</t>
+        </is>
+      </c>
+      <c r="B141" s="9" t="inlineStr">
+        <is>
+          <t>E23</t>
+        </is>
+      </c>
+      <c r="C141" s="9" t="inlineStr">
+        <is>
+          <t>Generated normal maps</t>
+        </is>
+      </c>
+      <c r="D141" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want normal maps made from my sprites by a tool, so that lights shade my art without painting a second image.</t>
+        </is>
+      </c>
+      <c r="E141" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Generate
+Given the atlases
+When the atlas tool runs with normal maps on
+Then every atlas gets a matching normal-map atlas
+Scenario: Missing
+Given a sprite without a normal map
+When it is lit
+Then it is lit flat, with no error
+Scenario: Own map
+Given a hand-made normal map named like the sprite
+When the tool runs
+Then the hand-made one is kept</t>
+        </is>
+      </c>
+      <c r="F141" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G141" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H141" s="9">
+        <f>VLOOKUP(G141,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I141" s="9">
+        <f>VLOOKUP(G141,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J141" s="9" t="inlineStr">
+        <is>
+          <t>M8c</t>
+        </is>
+      </c>
+      <c r="K141" s="9" t="inlineStr">
+        <is>
+          <t>US-240, US-120</t>
+        </is>
+      </c>
+      <c r="L141" s="9" t="inlineStr">
+        <is>
+          <t>ENV-19, D-05</t>
+        </is>
+      </c>
+      <c r="M141" s="9" t="inlineStr">
+        <is>
+          <t>Image processing: height and slopes from pixels</t>
+        </is>
+      </c>
+      <c r="N141" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O141" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="124.15" customHeight="1" s="20">
+      <c r="A142" s="7" t="inlineStr">
+        <is>
+          <t>US-242</t>
+        </is>
+      </c>
+      <c r="B142" s="9" t="inlineStr">
+        <is>
+          <t>E23</t>
+        </is>
+      </c>
+      <c r="C142" s="9" t="inlineStr">
+        <is>
+          <t>Day, night and seasons</t>
+        </is>
+      </c>
+      <c r="D142" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want dawn, day, dusk and night to follow the game clock, with longer summer days and short winter days, so that time feels real.</t>
+        </is>
+      </c>
+      <c r="E142" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Cycle
+Given the game clock running
+When a day passes
+Then the light goes through dawn, day, dusk and night colours from sky.json
+Scenario: Seasons
+Given midsummer and midwinter
+When the days are compared
+Then the summer day is longer, as calendar.json says
+Scenario: Moon
+Given night
+When it is drawn
+Then the moon gives a dim, blue light and a direction for shadows</t>
+        </is>
+      </c>
+      <c r="F142" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G142" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H142" s="9">
+        <f>VLOOKUP(G142,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I142" s="9">
+        <f>VLOOKUP(G142,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J142" s="9" t="inlineStr">
+        <is>
+          <t>M8c</t>
+        </is>
+      </c>
+      <c r="K142" s="9" t="inlineStr">
+        <is>
+          <t>US-240, US-010</t>
+        </is>
+      </c>
+      <c r="L142" s="9" t="inlineStr">
+        <is>
+          <t>ENV-19, ENV-20</t>
+        </is>
+      </c>
+      <c r="M142" s="9" t="inlineStr">
+        <is>
+          <t>Interpolating curves over time</t>
+        </is>
+      </c>
+      <c r="N142" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O142" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="124.15" customHeight="1" s="20">
+      <c r="A143" s="7" t="inlineStr">
+        <is>
+          <t>US-243</t>
+        </is>
+      </c>
+      <c r="B143" s="9" t="inlineStr">
+        <is>
+          <t>E23</t>
+        </is>
+      </c>
+      <c r="C143" s="9" t="inlineStr">
+        <is>
+          <t>Fires, torches and glowing effects</t>
+        </is>
+      </c>
+      <c r="D143" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want fires, torches, the sacred fire and elemental effects to light the night with a flicker, so that camps glow in the dark.</t>
+        </is>
+      </c>
+      <c r="E143" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Fire
+Given a lit fire pit at night
+When the scene is drawn
+Then it lights a circle around it with a flicker
+Scenario: Data
+Given a catalog entry with a light field
+When the thing is placed
+Then it emits that light; without the field, none
+Scenario: Torch
+Given a clan member carrying a torch
+When they walk at night
+Then the light moves with them</t>
+        </is>
+      </c>
+      <c r="F143" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G143" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H143" s="9">
+        <f>VLOOKUP(G143,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I143" s="9">
+        <f>VLOOKUP(G143,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J143" s="9" t="inlineStr">
+        <is>
+          <t>M8c</t>
+        </is>
+      </c>
+      <c r="K143" s="9" t="inlineStr">
+        <is>
+          <t>US-240, US-132</t>
+        </is>
+      </c>
+      <c r="L143" s="9" t="inlineStr">
+        <is>
+          <t>ENV-19</t>
+        </is>
+      </c>
+      <c r="M143" s="9" t="inlineStr">
+        <is>
+          <t>Noise for natural flicker</t>
+        </is>
+      </c>
+      <c r="N143" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O143" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="124.15" customHeight="1" s="20">
+      <c r="A144" s="7" t="inlineStr">
+        <is>
+          <t>US-244</t>
+        </is>
+      </c>
+      <c r="B144" s="9" t="inlineStr">
+        <is>
+          <t>E23</t>
+        </is>
+      </c>
+      <c r="C144" s="9" t="inlineStr">
+        <is>
+          <t>Sun and moon shadows</t>
+        </is>
+      </c>
+      <c r="D144" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want characters, plants and buildings to cast shadows that turn and stretch with the sun and the moon, so that the world has depth.</t>
+        </is>
+      </c>
+      <c r="E144" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Day
+Given a tree at 9:00 and at 17:00
+When it is drawn
+Then its shadow points away from the sun and is longer in the morning and evening
+Scenario: Casters
+Given characters, plants and buildings
+When the sun shines
+Then each casts a shadow sized by its height in the catalog
+Scenario: Overcast
+Given fog or heavy cloud
+When it sets in
+Then the shadows fade</t>
+        </is>
+      </c>
+      <c r="F144" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G144" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H144" s="9">
+        <f>VLOOKUP(G144,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I144" s="9">
+        <f>VLOOKUP(G144,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J144" s="9" t="inlineStr">
+        <is>
+          <t>M8c</t>
+        </is>
+      </c>
+      <c r="K144" s="9" t="inlineStr">
+        <is>
+          <t>US-242</t>
+        </is>
+      </c>
+      <c r="L144" s="9" t="inlineStr">
+        <is>
+          <t>ENV-21</t>
+        </is>
+      </c>
+      <c r="M144" s="9" t="inlineStr">
+        <is>
+          <t>Projecting silhouettes with a shear transform</t>
+        </is>
+      </c>
+      <c r="N144" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O144" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="124.15" customHeight="1" s="20">
+      <c r="A145" s="7" t="inlineStr">
+        <is>
+          <t>US-245</t>
+        </is>
+      </c>
+      <c r="B145" s="9" t="inlineStr">
+        <is>
+          <t>E23</t>
+        </is>
+      </c>
+      <c r="C145" s="9" t="inlineStr">
+        <is>
+          <t>Shadows from fires</t>
+        </is>
+      </c>
+      <c r="D145" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want a fire to throw shadows of the people and things near it at night, so that night scenes feel alive.</t>
+        </is>
+      </c>
+      <c r="E145" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Fire shadow
+Given a person standing near a fire at night
+When it is drawn
+Then their shadow points away from the fire
+Scenario: Two fires
+Given a person between two fires
+When it is drawn
+Then they cast two faint shadows
+Scenario: Budget
+Given many fires
+When the scene is drawn
+Then only the nearest fires (from lights.json) cast shadows and the frame budget holds</t>
+        </is>
+      </c>
+      <c r="F145" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G145" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H145" s="9">
+        <f>VLOOKUP(G145,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I145" s="9">
+        <f>VLOOKUP(G145,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J145" s="9" t="inlineStr">
+        <is>
+          <t>M8c</t>
+        </is>
+      </c>
+      <c r="K145" s="9" t="inlineStr">
+        <is>
+          <t>US-244, US-243</t>
+        </is>
+      </c>
+      <c r="L145" s="9" t="inlineStr">
+        <is>
+          <t>ENV-21</t>
+        </is>
+      </c>
+      <c r="M145" s="9" t="inlineStr">
+        <is>
+          <t>Choosing the nearest lights per object within a budget</t>
+        </is>
+      </c>
+      <c r="N145" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O145" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="124.15" customHeight="1" s="20">
+      <c r="A146" s="7" t="inlineStr">
+        <is>
+          <t>US-246</t>
+        </is>
+      </c>
+      <c r="B146" s="9" t="inlineStr">
+        <is>
+          <t>E23</t>
+        </is>
+      </c>
+      <c r="C146" s="9" t="inlineStr">
+        <is>
+          <t>Weather and light</t>
+        </is>
+      </c>
+      <c r="D146" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want clouds, rain, fog and storms to darken and tint the world, with lightning flashes, so that weather changes the mood.</t>
+        </is>
+      </c>
+      <c r="E146" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Dim
+Given rain starting at noon
+When it fades in
+Then the light dims and cools over the same 3 s
+Scenario: Lightning
+Given a storm
+When lightning strikes
+Then the whole scene flashes for a moment
+Scenario: Data
+Given weather.json
+When the owner sets a weather's light
+Then the game uses it</t>
+        </is>
+      </c>
+      <c r="F146" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G146" s="9" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H146" s="9">
+        <f>VLOOKUP(G146,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I146" s="9">
+        <f>VLOOKUP(G146,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J146" s="9" t="inlineStr">
+        <is>
+          <t>M8c</t>
+        </is>
+      </c>
+      <c r="K146" s="9" t="inlineStr">
+        <is>
+          <t>US-242, US-138</t>
+        </is>
+      </c>
+      <c r="L146" s="9" t="inlineStr">
+        <is>
+          <t>ENV-19</t>
+        </is>
+      </c>
+      <c r="M146" s="9" t="inlineStr">
+        <is>
+          <t>Blending light settings</t>
+        </is>
+      </c>
+      <c r="N146" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O146" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="124.15" customHeight="1" s="20">
+      <c r="A147" s="7" t="inlineStr">
+        <is>
+          <t>US-247</t>
+        </is>
+      </c>
+      <c r="B147" s="9" t="inlineStr">
+        <is>
+          <t>E23</t>
+        </is>
+      </c>
+      <c r="C147" s="9" t="inlineStr">
+        <is>
+          <t>Lighting in the Editor and quality settings</t>
+        </is>
+      </c>
+      <c r="D147" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to preview any time of day and place lights in the Editor, and players to choose lighting quality, so that levels look right and run everywhere.</t>
+        </is>
+      </c>
+      <c r="E147" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Preview
+Given the Editor
+When the owner drags the time-of-day slider
+Then the level is lit as at that hour
+Scenario: Place
+Given the light tool
+When the owner places a light and sets it
+Then it is saved in the level and shines in the game
+Scenario: Quality
+Given Low, Medium and High lighting
+When the player picks Low
+Then fire shadows and normal maps switch off and the frame time drops</t>
+        </is>
+      </c>
+      <c r="F147" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G147" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H147" s="9">
+        <f>VLOOKUP(G147,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I147" s="9">
+        <f>VLOOKUP(G147,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J147" s="9" t="inlineStr">
+        <is>
+          <t>M8c</t>
+        </is>
+      </c>
+      <c r="K147" s="9" t="inlineStr">
+        <is>
+          <t>US-243, US-244</t>
+        </is>
+      </c>
+      <c r="L147" s="9" t="inlineStr">
+        <is>
+          <t>ENV-19, EDT-01</t>
+        </is>
+      </c>
+      <c r="M147" s="9" t="inlineStr">
+        <is>
+          <t>Settings that change a pipeline</t>
+        </is>
+      </c>
+      <c r="N147" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O147" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="124.15" customHeight="1" s="20">
+      <c r="A148" s="7" t="inlineStr">
+        <is>
+          <t>US-250</t>
+        </is>
+      </c>
+      <c r="B148" s="9" t="inlineStr">
+        <is>
+          <t>E24</t>
+        </is>
+      </c>
+      <c r="C148" s="9" t="inlineStr">
+        <is>
+          <t>Building pieces and building kinds as data</t>
+        </is>
+      </c>
+      <c r="D148" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want building pieces (walls, floors, roofs, doors, posts) and building kinds (layout, materials, build time, interior mode, uses) in data files, so that I can design buildings without code.</t>
+        </is>
+      </c>
+      <c r="E148" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Load
+Given pieces.json and buildings.json with a hut, a windbreak, a storage pit, a drying rack and a palisade
+When the game starts
+Then every kind and piece is known, with errors naming file, line and field
+Scenario: Own list
+Given buildings in a level
+When it is saved and loaded
+Then they are kept in their own list, not as plants (CI-008)
+Scenario: Uses
+Given a hut with shelter and sleep, a storage pit with storage
+When the data loads
+Then their interactions are offered</t>
+        </is>
+      </c>
+      <c r="F148" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G148" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H148" s="9">
+        <f>VLOOKUP(G148,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I148" s="9">
+        <f>VLOOKUP(G148,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J148" s="9" t="inlineStr">
+        <is>
+          <t>M8d</t>
+        </is>
+      </c>
+      <c r="K148" s="9" t="inlineStr">
+        <is>
+          <t>US-150, US-155</t>
+        </is>
+      </c>
+      <c r="L148" s="9" t="inlineStr">
+        <is>
+          <t>INT-07, EDT-07, ARC-08</t>
+        </is>
+      </c>
+      <c r="M148" s="9" t="inlineStr">
+        <is>
+          <t>Composite data: a whole made of parts</t>
+        </is>
+      </c>
+      <c r="N148" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O148" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="124.15" customHeight="1" s="20">
+      <c r="A149" s="7" t="inlineStr">
+        <is>
+          <t>US-251</t>
+        </is>
+      </c>
+      <c r="B149" s="9" t="inlineStr">
+        <is>
+          <t>E24</t>
+        </is>
+      </c>
+      <c r="C149" s="9" t="inlineStr">
+        <is>
+          <t>Building from blueprints</t>
+        </is>
+      </c>
+      <c r="D149" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want to choose a building, place its blueprint, bring materials and build it over time, so that I can shape my camp.</t>
+        </is>
+      </c>
+      <c r="E149" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Place
+Given known blueprints
+When the player picks a hut and places it
+Then a see-through blueprint shows, red where it cannot stand
+Scenario: Build
+Given a placed blueprint
+When materials are brought and the hero works on it
+Then it rises in stages and is finished after its build time
+Scenario: Cancel
+Given a blueprint under way
+When the player cancels it
+Then the delivered materials are dropped on the site</t>
+        </is>
+      </c>
+      <c r="F149" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G149" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H149" s="9">
+        <f>VLOOKUP(G149,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I149" s="9">
+        <f>VLOOKUP(G149,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J149" s="9" t="inlineStr">
+        <is>
+          <t>M8d</t>
+        </is>
+      </c>
+      <c r="K149" s="9" t="inlineStr">
+        <is>
+          <t>US-250, US-153</t>
+        </is>
+      </c>
+      <c r="L149" s="9" t="inlineStr">
+        <is>
+          <t>INT-07</t>
+        </is>
+      </c>
+      <c r="M149" s="9" t="inlineStr">
+        <is>
+          <t>Placement validity on a grid</t>
+        </is>
+      </c>
+      <c r="N149" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O149" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="124.15" customHeight="1" s="20">
+      <c r="A150" s="7" t="inlineStr">
+        <is>
+          <t>US-252</t>
+        </is>
+      </c>
+      <c r="B150" s="9" t="inlineStr">
+        <is>
+          <t>E24</t>
+        </is>
+      </c>
+      <c r="C150" s="9" t="inlineStr">
+        <is>
+          <t>Building piece by piece</t>
+        </is>
+      </c>
+      <c r="D150" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want to place walls, floors, roofs and doors one by one, so that I can build any shape.</t>
+        </is>
+      </c>
+      <c r="E150" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Pieces
+Given the build menu's pieces
+When the player places walls in a ring, a door and a roof
+Then each piece is built like a small blueprint
+Scenario: Room
+Given an enclosed, roofed space with a door
+When it is finished
+Then it counts as a room: warm, sheltered, with its own light
+Scenario: Paths
+Given a door
+When people walk to the room
+Then they go through the door, never through walls</t>
+        </is>
+      </c>
+      <c r="F150" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G150" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H150" s="9">
+        <f>VLOOKUP(G150,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I150" s="9">
+        <f>VLOOKUP(G150,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J150" s="9" t="inlineStr">
+        <is>
+          <t>M8d</t>
+        </is>
+      </c>
+      <c r="K150" s="9" t="inlineStr">
+        <is>
+          <t>US-251</t>
+        </is>
+      </c>
+      <c r="L150" s="9" t="inlineStr">
+        <is>
+          <t>INT-07</t>
+        </is>
+      </c>
+      <c r="M150" s="9" t="inlineStr">
+        <is>
+          <t>Flood fill to find enclosed rooms</t>
+        </is>
+      </c>
+      <c r="N150" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O150" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="124.15" customHeight="1" s="20">
+      <c r="A151" s="7" t="inlineStr">
+        <is>
+          <t>US-253</t>
+        </is>
+      </c>
+      <c r="B151" s="9" t="inlineStr">
+        <is>
+          <t>E25</t>
+        </is>
+      </c>
+      <c r="C151" s="9" t="inlineStr">
+        <is>
+          <t>Clans build together</t>
+        </is>
+      </c>
+      <c r="D151" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want my clan members to help build and rival clans to grow their own camps, so that building is a shared life.</t>
+        </is>
+      </c>
+      <c r="E151" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Help
+Given a blueprint and idle clan members
+When time passes
+Then they bring materials and build, through the interaction system
+Scenario: Rivals
+Given a rival camp
+When a season passes
+Then it has built at least one building from its own blueprints
+Scenario: Deterministic
+Given the same seed and inputs
+When two runs
+Then the same buildings stand in the same places</t>
+        </is>
+      </c>
+      <c r="F151" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G151" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H151" s="9">
+        <f>VLOOKUP(G151,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I151" s="9">
+        <f>VLOOKUP(G151,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J151" s="9" t="inlineStr">
+        <is>
+          <t>M8e</t>
+        </is>
+      </c>
+      <c r="K151" s="9" t="inlineStr">
+        <is>
+          <t>US-251, US-154</t>
+        </is>
+      </c>
+      <c r="L151" s="9" t="inlineStr">
+        <is>
+          <t>INT-07, INT-05</t>
+        </is>
+      </c>
+      <c r="M151" s="9" t="inlineStr">
+        <is>
+          <t>Job queues for many workers</t>
+        </is>
+      </c>
+      <c r="N151" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O151" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="124.15" customHeight="1" s="20">
+      <c r="A152" s="7" t="inlineStr">
+        <is>
+          <t>US-254</t>
+        </is>
+      </c>
+      <c r="B152" s="9" t="inlineStr">
+        <is>
+          <t>E25</t>
+        </is>
+      </c>
+      <c r="C152" s="9" t="inlineStr">
+        <is>
+          <t>Interiors: roof fade or interior map</t>
+        </is>
+      </c>
+      <c r="D152" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want to see inside buildings, either by the roof fading or by entering an interior, as the building says, so that houses are places to be.</t>
+        </is>
+      </c>
+      <c r="E152" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Fade
+Given a hut set to roof fade
+When the hero walks in
+Then the roof and the front walls fade and the inside shows, lit by its fire and door
+Scenario: Interior
+Given a lodge set to interior map
+When the hero uses its door
+Then the interior level loads and its door leads back outside
+Scenario: Setting
+Given a placed building
+When the owner switches its interior mode in the Editor
+Then the game follows it</t>
+        </is>
+      </c>
+      <c r="F152" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G152" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H152" s="9">
+        <f>VLOOKUP(G152,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I152" s="9">
+        <f>VLOOKUP(G152,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J152" s="9" t="inlineStr">
+        <is>
+          <t>M8e</t>
+        </is>
+      </c>
+      <c r="K152" s="9" t="inlineStr">
+        <is>
+          <t>US-252, US-122</t>
+        </is>
+      </c>
+      <c r="L152" s="9" t="inlineStr">
+        <is>
+          <t>ENV-20, EDT-07</t>
+        </is>
+      </c>
+      <c r="M152" s="9" t="inlineStr">
+        <is>
+          <t>Linking two maps by doors</t>
+        </is>
+      </c>
+      <c r="N152" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O152" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="124.15" customHeight="1" s="20">
+      <c r="A153" s="7" t="inlineStr">
+        <is>
+          <t>US-255</t>
+        </is>
+      </c>
+      <c r="B153" s="9" t="inlineStr">
+        <is>
+          <t>E25</t>
+        </is>
+      </c>
+      <c r="C153" s="9" t="inlineStr">
+        <is>
+          <t>Wear, repair, damage and fire</t>
+        </is>
+      </c>
+      <c r="D153" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want buildings to wear with weather, to be repaired, damaged and to burn, so that they need care.</t>
+        </is>
+      </c>
+      <c r="E153" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Wear
+Given a hut through a winter
+When the season passes
+Then its condition falls as the data says and Repair is offered
+Scenario: Fire
+Given a burning torch dropped by a wooden wall
+When time passes
+Then the wall catches fire, it spreads to wooden neighbours by their materials and ends in rubble
+Scenario: Damage
+Given an attack on a wall
+When it is hit
+Then the wall loses condition and falls at zero</t>
+        </is>
+      </c>
+      <c r="F153" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G153" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H153" s="9">
+        <f>VLOOKUP(G153,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I153" s="9">
+        <f>VLOOKUP(G153,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J153" s="9" t="inlineStr">
+        <is>
+          <t>M8e</t>
+        </is>
+      </c>
+      <c r="K153" s="9" t="inlineStr">
+        <is>
+          <t>US-251, US-029</t>
+        </is>
+      </c>
+      <c r="L153" s="9" t="inlineStr">
+        <is>
+          <t>INT-08, PHY-04</t>
+        </is>
+      </c>
+      <c r="M153" s="9" t="inlineStr">
+        <is>
+          <t>Spreading state across neighbours (cellular rules)</t>
+        </is>
+      </c>
+      <c r="N153" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O153" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="124.15" customHeight="1" s="20">
+      <c r="A154" s="7" t="inlineStr">
+        <is>
+          <t>US-256</t>
+        </is>
+      </c>
+      <c r="B154" s="9" t="inlineStr">
+        <is>
+          <t>E24</t>
+        </is>
+      </c>
+      <c r="C154" s="9" t="inlineStr">
+        <is>
+          <t>Prefab editor and placing buildings</t>
+        </is>
+      </c>
+      <c r="D154" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to compose buildings from pieces in the Editor, save them as prefabs with costs and interior mode, and place them whole, so that levels start with real camps.</t>
+        </is>
+      </c>
+      <c r="E154" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Compose
+Given the Prefab tab
+When the owner places pieces, sets materials, build time and interior mode, and saves
+Then a prefab file is written and appears in the palette
+Scenario: Place
+Given a prefab
+When the owner places it in a level
+Then the finished building stands there in the game
+Scenario: Blueprint
+Given a prefab marked buildable
+When a game starts
+Then the player can build it from the build menu</t>
+        </is>
+      </c>
+      <c r="F154" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G154" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H154" s="9">
+        <f>VLOOKUP(G154,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I154" s="9">
+        <f>VLOOKUP(G154,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J154" s="9" t="inlineStr">
+        <is>
+          <t>M8d</t>
+        </is>
+      </c>
+      <c r="K154" s="9" t="inlineStr">
+        <is>
+          <t>US-252, US-124</t>
+        </is>
+      </c>
+      <c r="L154" s="9" t="inlineStr">
+        <is>
+          <t>EDT-07</t>
+        </is>
+      </c>
+      <c r="M154" s="9" t="inlineStr">
+        <is>
+          <t>Saving a group of parts as one reusable asset</t>
+        </is>
+      </c>
+      <c r="N154" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O154" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="124.15" customHeight="1" s="20">
+      <c r="A155" s="7" t="inlineStr">
+        <is>
+          <t>US-257</t>
+        </is>
+      </c>
+      <c r="B155" s="9" t="inlineStr">
+        <is>
+          <t>E25</t>
+        </is>
+      </c>
+      <c r="C155" s="9" t="inlineStr">
+        <is>
+          <t>Buildings in the clan's life</t>
+        </is>
+      </c>
+      <c r="D155" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want buildings to matter to the clan: shelter and warmth, sleeping, storage and ownership, saved with the world, so that building changes how people live.</t>
+        </is>
+      </c>
+      <c r="E155" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Warmth
+Given a cold night
+When clan members sleep in a hut
+Then their Warmth need falls slower than outside
+Scenario: Storage
+Given a storage pit
+When food is put in
+Then it counts in the clan store and spoils slower
+Scenario: Saved
+Given buildings with owners, condition and contents
+When the game saves and loads
+Then everything is kept</t>
+        </is>
+      </c>
+      <c r="F155" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G155" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H155" s="9">
+        <f>VLOOKUP(G155,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I155" s="9">
+        <f>VLOOKUP(G155,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J155" s="9" t="inlineStr">
+        <is>
+          <t>M8e</t>
+        </is>
+      </c>
+      <c r="K155" s="9" t="inlineStr">
+        <is>
+          <t>US-253, US-011</t>
+        </is>
+      </c>
+      <c r="L155" s="9" t="inlineStr">
+        <is>
+          <t>INT-07, SDC-02</t>
+        </is>
+      </c>
+      <c r="M155" s="9" t="inlineStr">
+        <is>
+          <t>Linking world objects to simulation needs</t>
+        </is>
+      </c>
+      <c r="N155" s="9" t="inlineStr">
+        <is>
+          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+        </is>
+      </c>
+      <c r="O155" s="16" t="inlineStr">
         <is>
           <t>To do</t>
         </is>
@@ -16790,7 +19282,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -16969,7 +19460,7 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>Age 1 needs hit detection, ballistics, basic bodies and material properties only; the rest belongs to later Ages.</t>
+          <t>Age 1 needs hit detection, ballistics, basic bodies and material properties only; the rest belongs to later Ages. Exception (D-42): fire spreading between building pieces is in the MVP.</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">

</xml_diff>

<commit_message>
CI: faster verification (D-46); Codex v2.3 sync; requirements v2.5
Local check builds and tests Debug; CI builds and tests Release on qa and both on main; CI only on qa/main, skips docs-only pushes, cancels superseded runs, caches vcpkg libraries.
</commit_message>
<xml_diff>
--- a/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
+++ b/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
@@ -654,7 +654,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Working tracker for developers. The source of truth is Project Odyssey.docx v2.4, chapter 12; this workbook is generated from the same data. Updated 2026-10-01: M8d split into M8d and M8e (D-43); D-06 decided.</t>
+          <t>Working tracker for developers. The source of truth is Project Odyssey.docx v2.5, chapter 12; this workbook is generated from the same data. Updated 2026-10-01: D-46 (faster verification).</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:JO36"/>
+  <dimension ref="A1:JO35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -4055,7 +4055,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B35:N35"/>
@@ -4077,7 +4076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -5097,6 +5096,43 @@
         </is>
       </c>
       <c r="G30" s="16" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>D-46</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Faster verification: local check = Debug build and tests; CI = Release on qa, Debug and Release on main; CI only on qa and main, skips docs-only pushes, cancels superseded runs, caches vcpkg libraries</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>Process decision</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>M8b</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>all stories from US-230</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G31" s="16" t="inlineStr">
         <is>
           <t>Decided</t>
         </is>

</xml_diff>

<commit_message>
Docs: completeness review; Codex v2.4 sync; requirements v2.6 (D-47)
CI-009 resolved, 3-second check at every exit review, stale decisions closed, MVP scope Decided, Figure 2 redrawn, reading PDFs no longer reported by the workspace sync.
</commit_message>
<xml_diff>
--- a/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
+++ b/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
@@ -654,7 +654,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Working tracker for developers. The source of truth is Project Odyssey.docx v2.5, chapter 12; this workbook is generated from the same data. Updated 2026-10-01: D-46 (faster verification).</t>
+          <t>Working tracker for developers. The source of truth is Project Odyssey.docx v2.6, chapter 12; this workbook is generated from the same data. Updated 2026-10-01: D-47 (housekeeping).</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Product Owner + Solution Architect, 2026-09-29. Status 'Proposed' = awaiting your decision.</t>
+          <t>Product Owner + Solution Architect, 2026-09-29; every scope item Decided by the owner (D-47, 2026-10-01).</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
@@ -911,7 +911,7 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
@@ -938,7 +938,7 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
@@ -965,7 +965,7 @@
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
@@ -992,7 +992,7 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
@@ -4076,7 +4076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -4394,7 +4394,7 @@
       </c>
       <c r="G11" s="16" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided (closed, D-47)</t>
         </is>
       </c>
     </row>
@@ -4468,7 +4468,7 @@
       </c>
       <c r="G13" s="16" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Decided (closed, D-47)</t>
         </is>
       </c>
     </row>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="G14" s="16" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Superseded (D-40, D-41)</t>
         </is>
       </c>
     </row>
@@ -4542,7 +4542,7 @@
       </c>
       <c r="G15" s="16" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided (closed, D-47)</t>
         </is>
       </c>
     </row>
@@ -5133,6 +5133,43 @@
         </is>
       </c>
       <c r="G31" s="16" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>D-47</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Housekeeping: stale decisions closed, MVP scope Decided, STO-01/SDC-01 absorbed, 10 s first-frame limit on CI with the 3 s check on the owner PC at exits, reading PDFs stay on Drive</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>Process decision</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>M8b</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G32" s="16" t="inlineStr">
         <is>
           <t>Decided</t>
         </is>

</xml_diff>

<commit_message>
Docs: sync workspace files from Drive (requirements v2.7, backlog)
</commit_message>
<xml_diff>
--- a/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
+++ b/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
@@ -654,7 +654,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Working tracker for developers. The source of truth is Project Odyssey.docx v2.6, chapter 12; this workbook is generated from the same data. Updated 2026-10-01: D-47 (housekeeping).</t>
+          <t>Working tracker for developers. The source of truth is Project Odyssey.docx v2.7, chapter 12; this workbook is generated from the same data. Updated 2026-10-01: D-48.</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -4653,7 +4653,7 @@
       </c>
       <c r="G18" s="16" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Open: plan ready, recruiting from K-M13 (D-48)</t>
         </is>
       </c>
     </row>
@@ -5170,6 +5170,43 @@
         </is>
       </c>
       <c r="G32" s="16" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>D-48</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>ARC-01..08 confirmed; playtest planned now (docs/plans/M6-playtest-plan.md), recruiting from K-M13; Anima Prompt Catalog as a Google Doc</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>Process decision</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>X-M6</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G33" s="16" t="inlineStr">
         <is>
           <t>Decided</t>
         </is>

</xml_diff>

<commit_message>
Docs: merge parallel versions: Codex v2.6, requirements v2.8
Combines Anima's v2.4/v2.5 and requirements v2.6/v2.7 with the US-231 D-44 alignment made on story/US-231 (CI-010).
</commit_message>
<xml_diff>
--- a/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
+++ b/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
@@ -654,7 +654,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Working tracker for developers. The source of truth is Project Odyssey.docx v2.7, chapter 12; this workbook is generated from the same data. Updated 2026-10-01: D-48.</t>
+          <t>Working tracker for developers. The source of truth is Project Odyssey.docx v2.8, chapter 12; this workbook is generated from the same data. Updated 2026-10-01: merged the M8b assembly edits (D-44) with D-47 and D-48.</t>
         </is>
       </c>
     </row>
@@ -4076,7 +4076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -5207,6 +5207,43 @@
         </is>
       </c>
       <c r="G33" s="16" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>D-44</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>M8b windowed sizes: 1280x720, 1600x900, 1920x1080, 2560x1440; Whole with black bars by default, optional Fill; zoom in Settings and via mouse wheel and keys in play; UI scale in Settings only; first start windowed 1280x720, zoom 2x, UI scale 1x, lighting Medium.</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Design decision</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>M8b</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>US-231..US-233</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G34" s="16" t="inlineStr">
         <is>
           <t>Decided</t>
         </is>
@@ -17640,12 +17677,16 @@
 Then it scales by 2 and by 4 with no blur and no border
 Scenario: Modes
 Given the settings screen
-When the player picks windowed (with sizes), borderless or exclusive full screen
-Then the mode changes at once and is saved
+When the player picks 1280x720, 1600x900, 1920x1080 or 2560x1440 windowed, borderless or exclusive full screen
+Then the mode and size change at once and are saved
 Scenario: Odd sizes
 Given a 2560x1440 screen
 When the game runs
-Then it scales by 2 with a thin border, or fills the screen smoothly if the player chooses Fill</t>
+Then Whole centres the 960x540 image at 2x with black bars; Fill uses the screen area when selected
+Scenario: First start
+Given no settings.json exists
+When the game launches
+Then it opens windowed at 1280x720 with Whole scaling, and defaults to camera zoom 2x, UI scale 1x and lighting Medium</t>
         </is>
       </c>
       <c r="F136" s="9" t="inlineStr">
@@ -17688,7 +17729,7 @@
       </c>
       <c r="N136" s="9" t="inlineStr">
         <is>
-          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+          <t>Resolution and window modes (owner, 2026-10-01, D-42 and D-44)</t>
         </is>
       </c>
       <c r="O136" s="16" t="inlineStr">
@@ -17722,11 +17763,11 @@
         <is>
           <t>Scenario: Zoom
 Given the default camera zoom of 2x
-When the player zooms out
+When the player zooms out in Settings or with the mouse wheel or zoom keys in play
 Then the view shows 1x (30 x 17 tiles) and back, around the hero
 Scenario: UI
 Given UI scale 1x and 2x
-When the player switches
+When the player switches UI scale in Settings
 Then panels, the font and the hotbar resize and stay crisp
 Scenario: Pointer
 Given any zoom
@@ -17774,7 +17815,7 @@
       </c>
       <c r="N137" s="9" t="inlineStr">
         <is>
-          <t>Resolution, lighting and buildings (owner, 2026-10-01, D-42)</t>
+          <t>Camera zoom and UI scale (owner, 2026-10-01, D-44)</t>
         </is>
       </c>
       <c r="O137" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Docs: sync workspace files from Drive (requirements v2.10, backlog: M9a-M9c)
</commit_message>
<xml_diff>
--- a/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
+++ b/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
@@ -654,7 +654,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Working tracker for developers. The source of truth is Project Odyssey.docx v2.8, chapter 12; this workbook is generated from the same data. Updated 2026-10-01: merged the M8b assembly edits (D-44) with D-47 and D-48.</t>
+          <t>Working tracker for developers. The source of truth is Project Odyssey.docx v2.10, chapter 12; this workbook is generated from the same data. Updated 2026-10-01: merged the M8b assembly edits (D-44) with D-47 and D-48.</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" style="20" min="1" max="1"/>
@@ -818,6 +818,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15.75" customHeight="1" s="20">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -832,6 +833,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="15.75" customHeight="1" s="20">
       <c r="A7" s="5" t="inlineStr">
         <is>
@@ -1298,72 +1300,77 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="51" customHeight="1" s="20"/>
-    <row r="26" ht="63.75" customHeight="1" s="20">
-      <c r="A26" s="5" t="inlineStr">
+    <row r="25" ht="38.25" customHeight="1" s="20">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>MVP-17</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>NPCs and trade</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Every placed NPC is a person with owner-defined classes, attitudes and opinions; talk, confront and trade (barter, currency, supply and demand) with any NPC; schedules and NPC-to-NPC interactions; all edited in the Editor; up to 100,000 persons with detail by distance.</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>SDC-08..SDC-12, INT-09..INT-12, EDT-08, NFR-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="63.75" customHeight="1" s="20"/>
+    <row r="27" ht="38.25" customHeight="1" s="20">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Success and kill criteria (decided before building)</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="38.25" customHeight="1" s="20">
-      <c r="A27" s="6" t="inlineStr">
+    <row r="28" ht="63.75" customHeight="1" s="20">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="C28" s="6" t="inlineStr">
         <is>
           <t>How measured</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D28" s="6" t="inlineStr">
         <is>
           <t>Gate</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="63.75" customHeight="1" s="20">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>Voluntary play time</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>5 of 8 playtesters play 30+ minutes without being asked to continue</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
-        <is>
-          <t>Observation + local session log (US-092)</t>
-        </is>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>M6</t>
         </is>
       </c>
     </row>
     <row r="29" ht="51" customHeight="1" s="20">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Emergent story</t>
+          <t>Voluntary play time</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>3 of 8 can retell a story that came from the simulation, not from a script</t>
+          <t>5 of 8 playtesters play 30+ minutes without being asked to continue</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Post-play interview</t>
+          <t>Observation + local session log (US-092)</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
@@ -1375,108 +1382,130 @@
     <row r="30" ht="51" customHeight="1" s="20">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Chronicle interest (early)</t>
+          <t>Emergent story</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>2 of 3 readers find a story in the console chronicle</t>
+          <t>3 of 8 can retell a story that came from the simulation, not from a script</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Show printed chronicle (M2: 3 readers, failed 2026-09-30; M2b retry: the owner reads and judges)</t>
+          <t>Post-play interview</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>M2, retried at M2b</t>
+          <t>M6</t>
         </is>
       </c>
     </row>
     <row r="31" ht="63.75" customHeight="1" s="20">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Frame rate</t>
+          <t>Chronicle interest (early)</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>60 FPS with 500 simulated agents in the region on the minimum PC (OPEN-19)</t>
+          <t>2 of 3 readers find a story in the console chronicle</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>FPS overlay (US-082)</t>
+          <t>Show printed chronicle (M2: 3 readers, failed 2026-09-30; M2b retry: the owner reads and judges)</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>M5</t>
+          <t>M2, retried at M2b</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Determinism</t>
+          <t>Frame rate</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>Same seed + inputs give the same world hash after 10,000 ticks</t>
+          <t>60 FPS with 500 simulated agents in the region on the minimum PC (OPEN-19)</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Automated test in CI</t>
+          <t>FPS overlay (US-082)</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
-          <t>M2 onwards</t>
+          <t>M5</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Stability</t>
+          <t>Determinism</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>No crash in a 2-hour play session or a 100-year soak test</t>
+          <t>Same seed + inputs give the same world hash after 10,000 ticks</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>Soak test + crash log</t>
+          <t>Automated test in CI</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>M5, M6</t>
+          <t>M2 onwards</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
+          <t>Stability</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>No crash in a 2-hour play session or a 100-year soak test</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Soak test + crash log</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>M5, M6</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
           <t>Kill / pivot rule</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>If M2 or M6 fails: stop adding content; redesign the simulation or the loop first</t>
         </is>
       </c>
-      <c r="C34" s="9" t="inlineStr">
+      <c r="C35" s="9" t="inlineStr">
         <is>
           <t>Owner decision, recorded</t>
         </is>
       </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>M2, M6</t>
         </is>
@@ -1504,7 +1533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:JO35"/>
+  <dimension ref="A1:LC38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -1699,6 +1728,46 @@
     <col width="13" customWidth="1" style="20" min="273" max="273"/>
     <col width="13" customWidth="1" style="20" min="274" max="274"/>
     <col width="13" customWidth="1" style="20" min="275" max="275"/>
+    <col width="13" customWidth="1" style="20" min="276" max="276"/>
+    <col width="13" customWidth="1" style="20" min="277" max="277"/>
+    <col width="13" customWidth="1" style="20" min="278" max="278"/>
+    <col width="13" customWidth="1" style="20" min="279" max="279"/>
+    <col width="13" customWidth="1" style="20" min="280" max="280"/>
+    <col width="13" customWidth="1" style="20" min="281" max="281"/>
+    <col width="13" customWidth="1" style="20" min="282" max="282"/>
+    <col width="13" customWidth="1" style="20" min="283" max="283"/>
+    <col width="13" customWidth="1" style="20" min="284" max="284"/>
+    <col width="13" customWidth="1" style="20" min="285" max="285"/>
+    <col width="13" customWidth="1" style="20" min="286" max="286"/>
+    <col width="13" customWidth="1" style="20" min="287" max="287"/>
+    <col width="13" customWidth="1" style="20" min="288" max="288"/>
+    <col width="13" customWidth="1" style="20" min="289" max="289"/>
+    <col width="13" customWidth="1" style="20" min="290" max="290"/>
+    <col width="13" customWidth="1" style="20" min="291" max="291"/>
+    <col width="13" customWidth="1" style="20" min="292" max="292"/>
+    <col width="13" customWidth="1" style="20" min="293" max="293"/>
+    <col width="13" customWidth="1" style="20" min="294" max="294"/>
+    <col width="13" customWidth="1" style="20" min="295" max="295"/>
+    <col width="13" customWidth="1" style="20" min="296" max="296"/>
+    <col width="13" customWidth="1" style="20" min="297" max="297"/>
+    <col width="13" customWidth="1" style="20" min="298" max="298"/>
+    <col width="13" customWidth="1" style="20" min="299" max="299"/>
+    <col width="13" customWidth="1" style="20" min="300" max="300"/>
+    <col width="13" customWidth="1" style="20" min="301" max="301"/>
+    <col width="13" customWidth="1" style="20" min="302" max="302"/>
+    <col width="13" customWidth="1" style="20" min="303" max="303"/>
+    <col width="13" customWidth="1" style="20" min="304" max="304"/>
+    <col width="13" customWidth="1" style="20" min="305" max="305"/>
+    <col width="13" customWidth="1" style="20" min="306" max="306"/>
+    <col width="13" customWidth="1" style="20" min="307" max="307"/>
+    <col width="13" customWidth="1" style="20" min="308" max="308"/>
+    <col width="13" customWidth="1" style="20" min="309" max="309"/>
+    <col width="13" customWidth="1" style="20" min="310" max="310"/>
+    <col width="13" customWidth="1" style="20" min="311" max="311"/>
+    <col width="13" customWidth="1" style="20" min="312" max="312"/>
+    <col width="13" customWidth="1" style="20" min="313" max="313"/>
+    <col width="13" customWidth="1" style="20" min="314" max="314"/>
+    <col width="13" customWidth="1" style="20" min="315" max="315"/>
   </cols>
   <sheetData>
     <row r="1" ht="20.25" customHeight="1" s="20">
@@ -1715,6 +1784,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -1725,6 +1795,7 @@
         <v>46300</v>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="38.25" customHeight="1" s="20">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -2576,6 +2647,126 @@
       <c r="JO6" s="12" t="n">
         <v>260</v>
       </c>
+      <c r="JP6" s="12" t="n">
+        <v>261</v>
+      </c>
+      <c r="JQ6" s="12" t="n">
+        <v>262</v>
+      </c>
+      <c r="JR6" s="12" t="n">
+        <v>263</v>
+      </c>
+      <c r="JS6" s="12" t="n">
+        <v>264</v>
+      </c>
+      <c r="JT6" s="12" t="n">
+        <v>265</v>
+      </c>
+      <c r="JU6" s="12" t="n">
+        <v>266</v>
+      </c>
+      <c r="JV6" s="12" t="n">
+        <v>267</v>
+      </c>
+      <c r="JW6" s="12" t="n">
+        <v>268</v>
+      </c>
+      <c r="JX6" s="12" t="n">
+        <v>269</v>
+      </c>
+      <c r="JY6" s="12" t="n">
+        <v>270</v>
+      </c>
+      <c r="JZ6" s="12" t="n">
+        <v>271</v>
+      </c>
+      <c r="KA6" s="12" t="n">
+        <v>272</v>
+      </c>
+      <c r="KB6" s="12" t="n">
+        <v>273</v>
+      </c>
+      <c r="KC6" s="12" t="n">
+        <v>274</v>
+      </c>
+      <c r="KD6" s="12" t="n">
+        <v>275</v>
+      </c>
+      <c r="KE6" s="12" t="n">
+        <v>276</v>
+      </c>
+      <c r="KF6" s="12" t="n">
+        <v>277</v>
+      </c>
+      <c r="KG6" s="12" t="n">
+        <v>278</v>
+      </c>
+      <c r="KH6" s="12" t="n">
+        <v>279</v>
+      </c>
+      <c r="KI6" s="12" t="n">
+        <v>280</v>
+      </c>
+      <c r="KJ6" s="12" t="n">
+        <v>281</v>
+      </c>
+      <c r="KK6" s="12" t="n">
+        <v>282</v>
+      </c>
+      <c r="KL6" s="12" t="n">
+        <v>283</v>
+      </c>
+      <c r="KM6" s="12" t="n">
+        <v>284</v>
+      </c>
+      <c r="KN6" s="12" t="n">
+        <v>285</v>
+      </c>
+      <c r="KO6" s="12" t="n">
+        <v>286</v>
+      </c>
+      <c r="KP6" s="12" t="n">
+        <v>287</v>
+      </c>
+      <c r="KQ6" s="12" t="n">
+        <v>288</v>
+      </c>
+      <c r="KR6" s="12" t="n">
+        <v>289</v>
+      </c>
+      <c r="KS6" s="12" t="n">
+        <v>290</v>
+      </c>
+      <c r="KT6" s="12" t="n">
+        <v>291</v>
+      </c>
+      <c r="KU6" s="12" t="n">
+        <v>292</v>
+      </c>
+      <c r="KV6" s="12" t="n">
+        <v>293</v>
+      </c>
+      <c r="KW6" s="12" t="n">
+        <v>294</v>
+      </c>
+      <c r="KX6" s="12" t="n">
+        <v>295</v>
+      </c>
+      <c r="KY6" s="12" t="n">
+        <v>296</v>
+      </c>
+      <c r="KZ6" s="12" t="n">
+        <v>297</v>
+      </c>
+      <c r="LA6" s="12" t="n">
+        <v>298</v>
+      </c>
+      <c r="LB6" s="12" t="n">
+        <v>299</v>
+      </c>
+      <c r="LC6" s="12" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="7" ht="42" customHeight="1" s="20">
       <c r="A7" s="7" t="inlineStr">
@@ -3419,12 +3610,12 @@
     <row r="21" ht="25.5" customHeight="1" s="20">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>M8d</t>
+          <t>M9a</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Buildings</t>
+          <t>NPC foundation</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
@@ -3433,10 +3624,10 @@
         </is>
       </c>
       <c r="D21" s="13" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E21" s="13" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F21" s="9">
         <f>ROUND((D21+E21)/2,0)</f>
@@ -3470,21 +3661,17 @@
         <f>SUMIFS('User Stories'!$H$5:$H$200,'User Stories'!$J$5:$J$200,A21,'User Stories'!$F$5:$F$200,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$200,'User Stories'!$J$5:$J$200,A21,'User Stories'!$F$5:$F$200,"Must")</f>
         <v/>
       </c>
-      <c r="N21" s="9" t="inlineStr">
-        <is>
-          <t>The hero builds from blueprints and piece by piece on a building grid, and rooms form; the owner composes prefabs from pieces in the Editor and places them in levels; prefabs marked buildable are offered as blueprints.</t>
-        </is>
-      </c>
+      <c r="N21" s="9" t="n"/>
     </row>
     <row r="22" ht="25.5" customHeight="1" s="20">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>M8e</t>
+          <t>M9b</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Building life</t>
+          <t>Trade economy</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -3496,7 +3683,7 @@
         <v>6</v>
       </c>
       <c r="E22" s="13" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F22" s="9">
         <f>ROUND((D22+E22)/2,0)</f>
@@ -3530,21 +3717,17 @@
         <f>SUMIFS('User Stories'!$H$5:$H$200,'User Stories'!$J$5:$J$200,A22,'User Stories'!$F$5:$F$200,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$200,'User Stories'!$J$5:$J$200,A22,'User Stories'!$F$5:$F$200,"Must")</f>
         <v/>
       </c>
-      <c r="N22" s="9" t="inlineStr">
-        <is>
-          <t>Clan members help build and rival clans build; each building fades its roof or opens an interior map as set in the Editor; buildings wear, are repaired, take damage, burn and fall; they shelter, warm and store for the clan and are saved.</t>
-        </is>
-      </c>
+      <c r="N22" s="9" t="n"/>
     </row>
     <row r="23" ht="25.5" customHeight="1" s="20">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>M9</t>
+          <t>M9c</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Interaction and dialogue editor</t>
+          <t>NPC life</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
@@ -3553,10 +3736,10 @@
         </is>
       </c>
       <c r="D23" s="13" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E23" s="13" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F23" s="9">
         <f>ROUND((D23+E23)/2,0)</f>
@@ -3590,21 +3773,17 @@
         <f>SUMIFS('User Stories'!$H$5:$H$200,'User Stories'!$J$5:$J$200,A23,'User Stories'!$F$5:$F$200,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$200,'User Stories'!$J$5:$J$200,A23,'User Stories'!$F$5:$F$200,"Must")</f>
         <v/>
       </c>
-      <c r="N23" s="9" t="inlineStr">
-        <is>
-          <t>The owner opens any dialogue or interaction in the Editor as a graph, edits it, test-plays it and saves it, and the file still reads well in a text editor.</t>
-        </is>
-      </c>
+      <c r="N23" s="9" t="n"/>
     </row>
     <row r="24" ht="25.5" customHeight="1" s="20">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>M10</t>
+          <t>M8d</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Quests and story authoring</t>
+          <t>Buildings</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
@@ -3613,10 +3792,10 @@
         </is>
       </c>
       <c r="D24" s="13" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E24" s="13" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F24" s="9">
         <f>ROUND((D24+E24)/2,0)</f>
@@ -3652,19 +3831,19 @@
       </c>
       <c r="N24" s="9" t="inlineStr">
         <is>
-          <t>The owner writes a quest in the Editor's graph (or offline in JSON), test-plays it with the debugger and saves it; a player gets it from an NPC, follows it in the journal, tracker and markers, and finishes it; the elder tutorial is a quest and crossroads events are edited as story events.</t>
+          <t>The hero builds from blueprints and piece by piece on a building grid, and rooms form; the owner composes prefabs from pieces in the Editor and places them in levels; prefabs marked buildable are offered as blueprints.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="25.5" customHeight="1" s="20">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>M11</t>
+          <t>M8e</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>Data editors</t>
+          <t>Building life</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
@@ -3673,10 +3852,10 @@
         </is>
       </c>
       <c r="D25" s="13" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E25" s="13" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F25" s="9">
         <f>ROUND((D25+E25)/2,0)</f>
@@ -3712,19 +3891,19 @@
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Every data file has a schema; the owner edits any entity, mechanic, story tuning value, game rule and daily routine in Editor forms with pickers and validation, and the running game reloads it.</t>
+          <t>Clan members help build and rival clans build; each building fades its roof or opens an interior map as set in the Editor; buildings wear, are repaired, take damage, burn and fall; they shelter, warm and store for the clan and are saved.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="25.5" customHeight="1" s="20">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>M12</t>
+          <t>M9</t>
         </is>
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
-          <t>World editing</t>
+          <t>Interaction and dialogue editor</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
@@ -3733,10 +3912,10 @@
         </is>
       </c>
       <c r="D26" s="13" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E26" s="13" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F26" s="9">
         <f>ROUND((D26+E26)/2,0)</f>
@@ -3772,19 +3951,19 @@
       </c>
       <c r="N26" s="9" t="inlineStr">
         <is>
-          <t>The owner opens the procedural region in the Editor, tunes the generator with a live preview, paints terrain, water and mountains, places things, people and camps, and edits each clan's and person's relations, economy, routines and actions; edits are saved on top of the seed and a new game plays them.</t>
+          <t>The owner opens any dialogue or interaction in the Editor as a graph, edits it, test-plays it and saves it, and the file still reads well in a text editor.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="25.5" customHeight="1" s="20">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>M13</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Politics</t>
+          <t>Quests and story authoring</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
@@ -3832,19 +4011,19 @@
       </c>
       <c r="N27" s="9" t="inlineStr">
         <is>
-          <t>Clans form alliances and vassal oaths, hold elders' councils, bind themselves by marriage, challenge leaders and use trade and craft knowledge as levers; the player can win the region through Politics; every political rule is editable in the Editor.</t>
+          <t>The owner writes a quest in the Editor's graph (or offline in JSON), test-plays it with the debugger and saves it; a player gets it from an NPC, follows it in the journal, tracker and markers, and finishes it; the elder tutorial is a quest and crossroads events are edited as story events.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="25.5" customHeight="1" s="20">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>M14</t>
+          <t>M11</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Data editors</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
@@ -3892,19 +4071,19 @@
       </c>
       <c r="N28" s="9" t="inlineStr">
         <is>
-          <t>Clans research by doing in workshops with inventors, pass knowledge by teaching, steal and guard secrets, and unlock recipes, interactions and professions from an editable tech tree; the player can win by forging the Ember Strand while leading in known technologies.</t>
+          <t>Every data file has a schema; the owner edits any entity, mechanic, story tuning value, game rule and daily routine in Editor forms with pickers and validation, and the running game reloads it.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="25.5" customHeight="1" s="20">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>M6</t>
+          <t>M12</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Playtest and go/no-go (KILL GATE 2)</t>
+          <t>World editing</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
@@ -3913,10 +4092,10 @@
         </is>
       </c>
       <c r="D29" s="13" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E29" s="13" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="F29" s="9">
         <f>ROUND((D29+E29)/2,0)</f>
@@ -3952,116 +4131,296 @@
       </c>
       <c r="N29" s="9" t="inlineStr">
         <is>
+          <t>The owner opens the procedural region in the Editor, tunes the generator with a live preview, paints terrain, water and mountains, places things, people and camps, and edits each clan's and person's relations, economy, routines and actions; edits are saved on top of the seed and a new game plays them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="25.5" customHeight="1" s="20">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>M13</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="E30" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="F30" s="9">
+        <f>ROUND((D30+E30)/2,0)</f>
+        <v/>
+      </c>
+      <c r="G30" s="9">
+        <f>H29+1</f>
+        <v/>
+      </c>
+      <c r="H30" s="9">
+        <f>G30+F30-1</f>
+        <v/>
+      </c>
+      <c r="I30" s="14">
+        <f>$B$4+(G30-1)*7</f>
+        <v/>
+      </c>
+      <c r="J30" s="14">
+        <f>$B$4+H30*7-1</f>
+        <v/>
+      </c>
+      <c r="K30" s="14">
+        <f>$B$4+SUM($D$7:D30)*7-1</f>
+        <v/>
+      </c>
+      <c r="L30" s="14">
+        <f>$B$4+SUM($E$7:E30)*7-1</f>
+        <v/>
+      </c>
+      <c r="M30" s="9">
+        <f>SUMIFS('User Stories'!$H$5:$H$200,'User Stories'!$J$5:$J$200,A30,'User Stories'!$F$5:$F$200,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$200,'User Stories'!$J$5:$J$200,A30,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="N30" s="9" t="inlineStr">
+        <is>
+          <t>Clans form alliances and vassal oaths, hold elders' councils, bind themselves by marriage, challenge leaders and use trade and craft knowledge as levers; the player can win the region through Politics; every political rule is editable in the Editor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="25.5" customHeight="1" s="20">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>M14</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="n">
+        <v>9</v>
+      </c>
+      <c r="E31" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="F31" s="9">
+        <f>ROUND((D31+E31)/2,0)</f>
+        <v/>
+      </c>
+      <c r="G31" s="9">
+        <f>H30+1</f>
+        <v/>
+      </c>
+      <c r="H31" s="9">
+        <f>G31+F31-1</f>
+        <v/>
+      </c>
+      <c r="I31" s="14">
+        <f>$B$4+(G31-1)*7</f>
+        <v/>
+      </c>
+      <c r="J31" s="14">
+        <f>$B$4+H31*7-1</f>
+        <v/>
+      </c>
+      <c r="K31" s="14">
+        <f>$B$4+SUM($D$7:D31)*7-1</f>
+        <v/>
+      </c>
+      <c r="L31" s="14">
+        <f>$B$4+SUM($E$7:E31)*7-1</f>
+        <v/>
+      </c>
+      <c r="M31" s="9">
+        <f>SUMIFS('User Stories'!$H$5:$H$200,'User Stories'!$J$5:$J$200,A31,'User Stories'!$F$5:$F$200,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$200,'User Stories'!$J$5:$J$200,A31,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="N31" s="9" t="inlineStr">
+        <is>
+          <t>Clans research by doing in workshops with inventors, pass knowledge by teaching, steal and guard secrets, and unlock recipes, interactions and professions from an editable tech tree; the player can win by forging the Ember Strand while leading in known technologies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="25.5" customHeight="1" s="20">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>M6</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Playtest and go/no-go (KILL GATE 2)</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D32" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="F32" s="9">
+        <f>ROUND((D32+E32)/2,0)</f>
+        <v/>
+      </c>
+      <c r="G32" s="9">
+        <f>H31+1</f>
+        <v/>
+      </c>
+      <c r="H32" s="9">
+        <f>G32+F32-1</f>
+        <v/>
+      </c>
+      <c r="I32" s="14">
+        <f>$B$4+(G32-1)*7</f>
+        <v/>
+      </c>
+      <c r="J32" s="14">
+        <f>$B$4+H32*7-1</f>
+        <v/>
+      </c>
+      <c r="K32" s="14">
+        <f>$B$4+SUM($D$7:D32)*7-1</f>
+        <v/>
+      </c>
+      <c r="L32" s="14">
+        <f>$B$4+SUM($E$7:E32)*7-1</f>
+        <v/>
+      </c>
+      <c r="M32" s="9">
+        <f>SUMIFS('User Stories'!$H$5:$H$200,'User Stories'!$J$5:$J$200,A32,'User Stories'!$F$5:$F$200,"Must")&amp;" - "&amp;SUMIFS('User Stories'!$I$5:$I$200,'User Stories'!$J$5:$J$200,A32,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="N32" s="9" t="inlineStr">
+        <is>
           <t>8 outside playtesters play; success criteria measured; go/no-go decision recorded. Held after M14 (owner, 2026-10-01, D-41).</t>
         </is>
       </c>
     </row>
-    <row r="30" s="20">
-      <c r="A30" s="7" t="n"/>
-      <c r="B30" s="7" t="inlineStr">
+    <row r="33" s="20">
+      <c r="A33" s="7" t="n"/>
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>MVP total</t>
         </is>
       </c>
-      <c r="C30" s="7" t="n"/>
-      <c r="D30" s="7">
-        <f>SUM(D7:D29)</f>
-        <v/>
-      </c>
-      <c r="E30" s="7">
-        <f>SUM(E7:E29)</f>
-        <v/>
-      </c>
-      <c r="F30" s="7">
-        <f>SUM(F7:F29)</f>
-        <v/>
-      </c>
-      <c r="G30" s="7" t="n"/>
-      <c r="H30" s="7">
-        <f>H29</f>
-        <v/>
-      </c>
-      <c r="I30" s="15">
+      <c r="C33" s="7" t="n"/>
+      <c r="D33" s="7">
+        <f>SUM(D7:D32)</f>
+        <v/>
+      </c>
+      <c r="E33" s="7">
+        <f>SUM(E7:E32)</f>
+        <v/>
+      </c>
+      <c r="F33" s="7">
+        <f>SUM(F7:F32)</f>
+        <v/>
+      </c>
+      <c r="G33" s="7" t="n"/>
+      <c r="H33" s="7">
+        <f>H32</f>
+        <v/>
+      </c>
+      <c r="I33" s="15">
         <f>I7</f>
         <v/>
       </c>
-      <c r="J30" s="15">
-        <f>J29</f>
-        <v/>
-      </c>
-      <c r="K30" s="15">
-        <f>K29</f>
-        <v/>
-      </c>
-      <c r="L30" s="15">
-        <f>L29</f>
-        <v/>
-      </c>
-      <c r="M30" s="7" t="n"/>
-      <c r="N30" s="7" t="inlineStr">
+      <c r="J33" s="15">
+        <f>J32</f>
+        <v/>
+      </c>
+      <c r="K33" s="15">
+        <f>K32</f>
+        <v/>
+      </c>
+      <c r="L33" s="15">
+        <f>L32</f>
+        <v/>
+      </c>
+      <c r="M33" s="7" t="n"/>
+      <c r="N33" s="7" t="inlineStr">
         <is>
           <t>Months (likely) = weeks / 4.33</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="27.95" customHeight="1" s="20">
-      <c r="A31" s="7" t="n"/>
-      <c r="B31" s="7" t="inlineStr">
+    <row r="34" ht="27.95" customHeight="1" s="20">
+      <c r="A34" s="7" t="n"/>
+      <c r="B34" s="7" t="inlineStr">
         <is>
           <t>In months</t>
         </is>
       </c>
-      <c r="C31" s="7" t="n"/>
-      <c r="D31" s="7">
-        <f>ROUND(D30/4.33,1)</f>
-        <v/>
-      </c>
-      <c r="E31" s="7">
-        <f>ROUND(E30/4.33,1)</f>
-        <v/>
-      </c>
-      <c r="F31" s="7">
-        <f>ROUND(F30/4.33,1)</f>
-        <v/>
-      </c>
-      <c r="G31" s="7" t="n"/>
-      <c r="H31" s="7" t="n"/>
-      <c r="I31" s="7" t="n"/>
-      <c r="J31" s="7" t="n"/>
-      <c r="K31" s="7" t="n"/>
-      <c r="L31" s="7" t="n"/>
-      <c r="M31" s="7" t="n"/>
-      <c r="N31" s="7" t="n"/>
-    </row>
-    <row r="32" ht="27.95" customHeight="1" s="20"/>
-    <row r="33" ht="27.95" customHeight="1" s="20">
-      <c r="B33" s="19" t="inlineStr">
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="7">
+        <f>ROUND(D33/4.33,1)</f>
+        <v/>
+      </c>
+      <c r="E34" s="7">
+        <f>ROUND(E33/4.33,1)</f>
+        <v/>
+      </c>
+      <c r="F34" s="7">
+        <f>ROUND(F33/4.33,1)</f>
+        <v/>
+      </c>
+      <c r="G34" s="7" t="n"/>
+      <c r="H34" s="7" t="n"/>
+      <c r="I34" s="7" t="n"/>
+      <c r="J34" s="7" t="n"/>
+      <c r="K34" s="7" t="n"/>
+      <c r="L34" s="7" t="n"/>
+      <c r="M34" s="7" t="n"/>
+      <c r="N34" s="7" t="n"/>
+    </row>
+    <row r="35" ht="27.95" customHeight="1" s="20"/>
+    <row r="36" ht="27.95" customHeight="1" s="20">
+      <c r="B36" s="19" t="inlineStr">
         <is>
           <t>Why the estimate grew: the learning path (requirements, section 8.3) estimated 9-13 months top-down. The bottom-up sum of the MVP stories is higher; this sheet uses the bottom-up figure.</t>
         </is>
       </c>
     </row>
-    <row r="34" s="20">
-      <c r="B34" s="19" t="inlineStr">
+    <row r="37" s="20">
+      <c r="B37" s="19" t="inlineStr">
         <is>
           <t>Buffer: the 'Should' stories are the cut list if time runs short. Cutting all of them saves about 5-11 weeks.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="102" customHeight="1" s="20">
-      <c r="B35" s="19" t="inlineStr">
-        <is>
-          <t>Kill gates: M2 (failed 2026-09-30, passed at the M2b retry) and M6 (do playtesters stay?), held after M14 (D-41). Critical path: M0 &gt; M1 &gt; M1b &gt; M2 &gt; M2b &gt; M2c &gt; M2d &gt; M3 &gt; M4 &gt; M5 &gt; M7 &gt; M8 &gt; M8b &gt; M8c &gt; M8d &gt; M8e &gt; M9 &gt; M10 &gt; M11 &gt; M12 &gt; M13 &gt; M14 &gt; M6. Dates of M2c onwards are not re-planned yet.</t>
+    <row r="38" ht="102" customHeight="1" s="20">
+      <c r="B38" s="19" t="inlineStr">
+        <is>
+          <t>Kill gates: M2 (failed 2026-09-30, passed at the M2b retry) and M6 (do playtesters stay?), held after M14 (D-41). Critical path: M0 &gt; M1 &gt; M1b &gt; M2 &gt; M2b &gt; M2c &gt; M2d &gt; M3 &gt; M4 &gt; M5 &gt; M7 &gt; M8 &gt; M8b &gt; M8c &gt; M9a &gt; M9b &gt; M9c &gt; M8d &gt; M8e &gt; M9 &gt; M10 &gt; M11 &gt; M12 &gt; M13 &gt; M14 &gt; M6. Dates of M2c onwards are not re-planned yet.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B35:N35"/>
-    <mergeCell ref="B34:N34"/>
-    <mergeCell ref="B33:N33"/>
+    <mergeCell ref="B38:N38"/>
+    <mergeCell ref="B37:N37"/>
+    <mergeCell ref="B36:N36"/>
   </mergeCells>
-  <conditionalFormatting sqref="P7:JO29">
+  <conditionalFormatting sqref="P7:LC32">
     <cfRule type="expression" priority="1" dxfId="10">
       <formula>AND(P$6&gt;=$G7,P$6&lt;=$H7)</formula>
     </cfRule>
@@ -4076,7 +4435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -5212,7 +5571,7 @@
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" s="20">
       <c r="A34" s="7" t="inlineStr">
         <is>
           <t>D-44</t>
@@ -5244,6 +5603,43 @@
         </is>
       </c>
       <c r="G34" s="16" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" s="20">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>D-52</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade economy and NPC life: 24 answers and 4 follow-ups (docs/decision-requests/D-52.md); three milestones right after M8c</t>
+        </is>
+      </c>
+      <c r="C35" s="9" t="inlineStr">
+        <is>
+          <t>Design decision</t>
+        </is>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
+        <is>
+          <t>M9a</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>US-260..US-270, US-280..US-284, US-290..US-294</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G35" s="16" t="inlineStr">
         <is>
           <t>Decided</t>
         </is>
@@ -5279,7 +5675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -6555,37 +6951,175 @@
         <v/>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="7" t="n"/>
-      <c r="B31" s="7" t="inlineStr">
+    <row r="31" ht="25.5" customHeight="1" s="20">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>E26</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>Every placed NPC is a person with one or more classes, an attitude and opinions; the player talks to, confronts and acts on any NPC; the owner sets every NPC in the Editor; 100,000 persons run with detail by distance.</t>
+        </is>
+      </c>
+      <c r="D31" s="9" t="inlineStr">
+        <is>
+          <t>M9a</t>
+        </is>
+      </c>
+      <c r="E31" s="9">
+        <f>COUNTIF('User Stories'!$B$5:$B$200,A31)</f>
+        <v/>
+      </c>
+      <c r="F31" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A31,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="G31" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A31,'User Stories'!$H$5:$H$200)</f>
+        <v/>
+      </c>
+      <c r="H31" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A31,'User Stories'!$I$5:$I$200)</f>
+        <v/>
+      </c>
+      <c r="I31" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A31,'User Stories'!$O$5:$O$200,"Done")</f>
+        <v/>
+      </c>
+      <c r="J31" s="17">
+        <f>IFERROR(I31/E31,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="25.5" customHeight="1" s="20">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>E27</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Trade economy</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>The player trades with any trader by barter or the region's currency; prices follow supply and demand and opinion; limited stock restocks daily; currencies and stock are set in the Editor.</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>M9b</t>
+        </is>
+      </c>
+      <c r="E32" s="9">
+        <f>COUNTIF('User Stories'!$B$5:$B$200,A32)</f>
+        <v/>
+      </c>
+      <c r="F32" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A32,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="G32" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A32,'User Stories'!$H$5:$H$200)</f>
+        <v/>
+      </c>
+      <c r="H32" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A32,'User Stories'!$I$5:$I$200)</f>
+        <v/>
+      </c>
+      <c r="I32" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A32,'User Stories'!$O$5:$O$200,"Done")</f>
+        <v/>
+      </c>
+      <c r="J32" s="17">
+        <f>IFERROR(I32/E32,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="25.5" customHeight="1" s="20">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>E28</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>NPC life</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>NPCs follow day and night schedules, act from their classes, custom actions and events, and do everything to each other with the same files, all edited in the Editor.</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>M9c</t>
+        </is>
+      </c>
+      <c r="E33" s="9">
+        <f>COUNTIF('User Stories'!$B$5:$B$200,A33)</f>
+        <v/>
+      </c>
+      <c r="F33" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A33,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="G33" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A33,'User Stories'!$H$5:$H$200)</f>
+        <v/>
+      </c>
+      <c r="H33" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A33,'User Stories'!$I$5:$I$200)</f>
+        <v/>
+      </c>
+      <c r="I33" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A33,'User Stories'!$O$5:$O$200,"Done")</f>
+        <v/>
+      </c>
+      <c r="J33" s="17">
+        <f>IFERROR(I33/E33,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" s="20">
+      <c r="A34" s="7" t="n"/>
+      <c r="B34" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C31" s="7" t="n"/>
-      <c r="D31" s="7" t="n"/>
-      <c r="E31" s="7">
-        <f>SUM(E5:E30)</f>
-        <v/>
-      </c>
-      <c r="F31" s="7">
-        <f>SUM(F5:F30)</f>
-        <v/>
-      </c>
-      <c r="G31" s="7">
-        <f>SUM(G5:G30)</f>
-        <v/>
-      </c>
-      <c r="H31" s="7">
-        <f>SUM(H5:H30)</f>
-        <v/>
-      </c>
-      <c r="I31" s="7">
-        <f>SUM(I5:I30)</f>
-        <v/>
-      </c>
-      <c r="J31" s="18">
-        <f>IFERROR(I31/E31,0)</f>
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="7" t="n"/>
+      <c r="E34" s="7">
+        <f>SUM(E5:E33)</f>
+        <v/>
+      </c>
+      <c r="F34" s="7">
+        <f>SUM(F5:F33)</f>
+        <v/>
+      </c>
+      <c r="G34" s="7">
+        <f>SUM(G5:G33)</f>
+        <v/>
+      </c>
+      <c r="H34" s="7">
+        <f>SUM(H5:H33)</f>
+        <v/>
+      </c>
+      <c r="I34" s="7">
+        <f>SUM(I5:I33)</f>
+        <v/>
+      </c>
+      <c r="J34" s="18">
+        <f>IFERROR(I34/E34,0)</f>
         <v/>
       </c>
     </row>
@@ -6600,7 +7134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O155"/>
+  <dimension ref="A1:O176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="20" min="1" max="1"/>
@@ -19367,6 +19901,1780 @@
         </is>
       </c>
       <c r="O155" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="124.15" customHeight="1" s="20">
+      <c r="A156" s="7" t="inlineStr">
+        <is>
+          <t>US-260</t>
+        </is>
+      </c>
+      <c r="B156" s="9" t="inlineStr">
+        <is>
+          <t>E26</t>
+        </is>
+      </c>
+      <c r="C156" s="9" t="inlineStr">
+        <is>
+          <t>NPC Classes</t>
+        </is>
+      </c>
+      <c r="D156" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to create, edit, delete and assign NPC Classes in the Editor, each with a colour, an icon, tags, default dialogues and default actions, so that I can say what kinds of people my world has.</t>
+        </is>
+      </c>
+      <c r="E156" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Create
+Given the NPC Classes tab
+When the owner creates the class healer with a green colour and the tag healer and saves
+Then assets/data/npc-classes/healer.json exists and the class is offered in every class picker
+Scenario: Delete in use
+Given a class used by two placed NPCs
+When the owner deletes it
+Then the Editor refuses and names both NPCs
+Scenario: Mistake
+Given a class file with an unknown icon
+When the game starts
+Then the error names the file, the line and the field, and the other classes load</t>
+        </is>
+      </c>
+      <c r="F156" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G156" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H156" s="9">
+        <f>VLOOKUP(G156,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I156" s="9">
+        <f>VLOOKUP(G156,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J156" s="9" t="inlineStr">
+        <is>
+          <t>M9a</t>
+        </is>
+      </c>
+      <c r="K156" s="9" t="inlineStr">
+        <is>
+          <t>US-150, US-126</t>
+        </is>
+      </c>
+      <c r="L156" s="9" t="inlineStr">
+        <is>
+          <t>SDC-08, EDT-08</t>
+        </is>
+      </c>
+      <c r="M156" s="9" t="inlineStr">
+        <is>
+          <t>Catalogs keyed by id; refusing a delete that would leave dangling references.</t>
+        </is>
+      </c>
+      <c r="N156" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O156" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="124.15" customHeight="1" s="20">
+      <c r="A157" s="7" t="inlineStr">
+        <is>
+          <t>US-261</t>
+        </is>
+      </c>
+      <c r="B157" s="9" t="inlineStr">
+        <is>
+          <t>E26</t>
+        </is>
+      </c>
+      <c r="C157" s="9" t="inlineStr">
+        <is>
+          <t>Kind defaults and placed-NPC overrides</t>
+        </is>
+      </c>
+      <c r="D157" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want defaults per NPC kind and per-NPC changes in the level, so that a new wanderer starts sensible and each placed one can differ.</t>
+        </is>
+      </c>
+      <c r="E157" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Precedence
+Given the class trader allows trade and a placed NPC of that class denies it
+When the game resolves the NPC's actions
+Then trade is denied for that NPC only
+Scenario: Old level
+Given a level saved before this story
+When it is loaded and saved
+Then the file is unchanged
+Scenario: Reload
+Given a kind file changed on disk while playing
+When the owner presses F5
+Then the change applies to every NPC of that kind without an override</t>
+        </is>
+      </c>
+      <c r="F157" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G157" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H157" s="9">
+        <f>VLOOKUP(G157,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I157" s="9">
+        <f>VLOOKUP(G157,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J157" s="9" t="inlineStr">
+        <is>
+          <t>M9a</t>
+        </is>
+      </c>
+      <c r="K157" s="9" t="inlineStr">
+        <is>
+          <t>US-260, US-122</t>
+        </is>
+      </c>
+      <c r="L157" s="9" t="inlineStr">
+        <is>
+          <t>SDC-09, EDT-08</t>
+        </is>
+      </c>
+      <c r="M157" s="9" t="inlineStr">
+        <is>
+          <t>Layered defaults; std::optional for 'not set'; merging lists with a precedence rule.</t>
+        </is>
+      </c>
+      <c r="N157" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O157" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="124.15" customHeight="1" s="20">
+      <c r="A158" s="7" t="inlineStr">
+        <is>
+          <t>US-262</t>
+        </is>
+      </c>
+      <c r="B158" s="9" t="inlineStr">
+        <is>
+          <t>E26</t>
+        </is>
+      </c>
+      <c r="C158" s="9" t="inlineStr">
+        <is>
+          <t>Placed NPCs are full persons</t>
+        </is>
+      </c>
+      <c r="D158" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want the people placed in a level to be real members of the world, with needs, memories, ageing and families, so that they feel alive like my clan.</t>
+        </is>
+      </c>
+      <c r="E158" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Person
+Given a placed wanderer
+When a day passes
+Then its needs change and a memory of the day exists, as for a clan member
+Scenario: Saved
+Given a placed person who aged one day and met the hero
+When the game is saved and loaded
+Then age, needs and memories are the same
+Scenario: Creatures
+Given a placed goblin of class monster
+When the level loads
+Then it is a creature, not a person, and fights as before</t>
+        </is>
+      </c>
+      <c r="F158" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G158" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H158" s="9">
+        <f>VLOOKUP(G158,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I158" s="9">
+        <f>VLOOKUP(G158,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J158" s="9" t="inlineStr">
+        <is>
+          <t>M9a</t>
+        </is>
+      </c>
+      <c r="K158" s="9" t="inlineStr">
+        <is>
+          <t>US-261, US-154</t>
+        </is>
+      </c>
+      <c r="L158" s="9" t="inlineStr">
+        <is>
+          <t>SDC-09</t>
+        </is>
+      </c>
+      <c r="M158" s="9" t="inlineStr">
+        <is>
+          <t>Identity and lifetime: one id from the level file to the save.</t>
+        </is>
+      </c>
+      <c r="N158" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O158" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="124.15" customHeight="1" s="20">
+      <c r="A159" s="7" t="inlineStr">
+        <is>
+          <t>US-263</t>
+        </is>
+      </c>
+      <c r="B159" s="9" t="inlineStr">
+        <is>
+          <t>E26</t>
+        </is>
+      </c>
+      <c r="C159" s="9" t="inlineStr">
+        <is>
+          <t>The NPC store and detail by distance</t>
+        </is>
+      </c>
+      <c r="D159" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want the world to hold up to 100,000 region-loaded NPCs while the game stays smooth, so that the end game can be crowded.</t>
+        </is>
+      </c>
+      <c r="E159" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Load
+Given 100,000 generated persons in a headless run
+When one in-game day is simulated
+Then it finishes within the budget of ADR-022 on the D-06 PC and the determinism hash is stable over two runs
+Scenario: Near and far
+Given a person who walks out of the near radius and back
+When the days pass
+Then its needs and memories continue without a jump or a loss
+Scenario: Frame
+Given the test level with 100,000 far persons loaded
+When the game runs for one minute
+Then the frame time stays within the D-06 target</t>
+        </is>
+      </c>
+      <c r="F159" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G159" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H159" s="9">
+        <f>VLOOKUP(G159,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I159" s="9">
+        <f>VLOOKUP(G159,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J159" s="9" t="inlineStr">
+        <is>
+          <t>M9a</t>
+        </is>
+      </c>
+      <c r="K159" s="9" t="inlineStr">
+        <is>
+          <t>US-262</t>
+        </is>
+      </c>
+      <c r="L159" s="9" t="inlineStr">
+        <is>
+          <t>NFR-08, SDC-09</t>
+        </is>
+      </c>
+      <c r="M159" s="9" t="inlineStr">
+        <is>
+          <t>Struct of arrays and cache lines; spatial hashing; why O(n^2) breaks at 100,000.</t>
+        </is>
+      </c>
+      <c r="N159" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O159" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="124.15" customHeight="1" s="20">
+      <c r="A160" s="7" t="inlineStr">
+        <is>
+          <t>US-264</t>
+        </is>
+      </c>
+      <c r="B160" s="9" t="inlineStr">
+        <is>
+          <t>E26</t>
+        </is>
+      </c>
+      <c r="C160" s="9" t="inlineStr">
+        <is>
+          <t>Attitudes and opinions</t>
+        </is>
+      </c>
+      <c r="D160" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want every NPC to have its own attitude to me and to others, changed by what we do, so that my choices matter person by person.</t>
+        </is>
+      </c>
+      <c r="E160" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Gift
+Given a neutral NPC
+When the hero gives it a gift worth the 'gift' amount
+Then its opinion of the hero rises by that amount and its word changes when a threshold is crossed
+Scenario: Family
+Given two NPCs of the same family
+When the level loads
+Then each starts with the 'same family' opinion of the other
+Scenario: Sparse
+Given 100,000 persons where 10 pairs have met
+When the store is inspected
+Then exactly 10 opinion entries exist</t>
+        </is>
+      </c>
+      <c r="F160" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G160" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H160" s="9">
+        <f>VLOOKUP(G160,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I160" s="9">
+        <f>VLOOKUP(G160,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J160" s="9" t="inlineStr">
+        <is>
+          <t>M9a</t>
+        </is>
+      </c>
+      <c r="K160" s="9" t="inlineStr">
+        <is>
+          <t>US-263</t>
+        </is>
+      </c>
+      <c r="L160" s="9" t="inlineStr">
+        <is>
+          <t>SDC-10</t>
+        </is>
+      </c>
+      <c r="M160" s="9" t="inlineStr">
+        <is>
+          <t>Sparse maps keyed by pairs; deriving words from numbers with thresholds.</t>
+        </is>
+      </c>
+      <c r="N160" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O160" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="124.15" customHeight="1" s="20">
+      <c r="A161" s="7" t="inlineStr">
+        <is>
+          <t>US-265</t>
+        </is>
+      </c>
+      <c r="B161" s="9" t="inlineStr">
+        <is>
+          <t>E26</t>
+        </is>
+      </c>
+      <c r="C161" s="9" t="inlineStr">
+        <is>
+          <t>Talk with placed NPCs</t>
+        </is>
+      </c>
+      <c r="D161" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want to talk to any NPC that has something to say, so that every person in a level can speak.</t>
+        </is>
+      </c>
+      <c r="E161" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Talk
+Given a placed NPC with a player dialogue, 2 m from the hero
+When the player right-clicks it and chooses Talk
+Then its dialogue opens and the game pauses
+Scenario: No script
+Given a placed NPC with no player dialogue
+When the player right-clicks it
+Then Talk is not offered
+Scenario: Clan unchanged
+Given a clan member
+When the player chooses Talk
+Then the conversation is the same as before this story</t>
+        </is>
+      </c>
+      <c r="F161" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G161" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H161" s="9">
+        <f>VLOOKUP(G161,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I161" s="9">
+        <f>VLOOKUP(G161,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J161" s="9" t="inlineStr">
+        <is>
+          <t>M9a</t>
+        </is>
+      </c>
+      <c r="K161" s="9" t="inlineStr">
+        <is>
+          <t>US-264, US-161</t>
+        </is>
+      </c>
+      <c r="L161" s="9" t="inlineStr">
+        <is>
+          <t>SDC-11, SDC-03</t>
+        </is>
+      </c>
+      <c r="M161" s="9" t="inlineStr">
+        <is>
+          <t>One interface for many kinds of things; data-driven dispatch by tags.</t>
+        </is>
+      </c>
+      <c r="N161" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O161" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="124.15" customHeight="1" s="20">
+      <c r="A162" s="7" t="inlineStr">
+        <is>
+          <t>US-266</t>
+        </is>
+      </c>
+      <c r="B162" s="9" t="inlineStr">
+        <is>
+          <t>E26</t>
+        </is>
+      </c>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>Confront</t>
+        </is>
+      </c>
+      <c r="D162" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want a separate Confront button with taunt, insult, ask for peace, antagonise and de-escalate, so that I can deal with hostile NPCs by words and live with the consequences.</t>
+        </is>
+      </c>
+      <c r="E162" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Calm down
+Given a hostile NPC about to attack
+When the player chooses De-escalate and the check succeeds
+Then it stops attacking and its opinion of the hero rises
+Scenario: Insult
+Given an NPC with two friends within hearing range
+When the player insults it
+Then its opinion and its friends' opinions of the hero fall by the data amounts
+Scenario: Separate
+Given a friendly NPC
+When the player presses the Confront key
+Then the five confront actions are offered and Talk is not among them</t>
+        </is>
+      </c>
+      <c r="F162" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G162" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H162" s="9">
+        <f>VLOOKUP(G162,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I162" s="9">
+        <f>VLOOKUP(G162,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J162" s="9" t="inlineStr">
+        <is>
+          <t>M9a</t>
+        </is>
+      </c>
+      <c r="K162" s="9" t="inlineStr">
+        <is>
+          <t>US-265</t>
+        </is>
+      </c>
+      <c r="L162" s="9" t="inlineStr">
+        <is>
+          <t>SDC-11</t>
+        </is>
+      </c>
+      <c r="M162" s="9" t="inlineStr">
+        <is>
+          <t>Intents mapped from keys; effects that spread to bystanders.</t>
+        </is>
+      </c>
+      <c r="N162" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O162" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="124.15" customHeight="1" s="20">
+      <c r="A163" s="7" t="inlineStr">
+        <is>
+          <t>US-267</t>
+        </is>
+      </c>
+      <c r="B163" s="9" t="inlineStr">
+        <is>
+          <t>E26</t>
+        </is>
+      </c>
+      <c r="C163" s="9" t="inlineStr">
+        <is>
+          <t>Actions and the Actions pop-up</t>
+        </is>
+      </c>
+      <c r="D163" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want to see every action an NPC could offer and what each needs, while the menu shows only what I can do now, so that I know how to unlock the rest.</t>
+        </is>
+      </c>
+      <c r="E163" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Hidden
+Given a trader whose trade needs the attitude friendly and who is wary of the hero
+When the player right-clicks it
+Then Trade is not in the menu
+Scenario: Pop-up
+Given the same trader
+When the player opens the Actions pop-up
+Then Trade is listed with 'needs: friendly or better'</t>
+        </is>
+      </c>
+      <c r="F163" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G163" s="9" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H163" s="9">
+        <f>VLOOKUP(G163,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I163" s="9">
+        <f>VLOOKUP(G163,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J163" s="9" t="inlineStr">
+        <is>
+          <t>M9a</t>
+        </is>
+      </c>
+      <c r="K163" s="9" t="inlineStr">
+        <is>
+          <t>US-265</t>
+        </is>
+      </c>
+      <c r="L163" s="9" t="inlineStr">
+        <is>
+          <t>INT-09</t>
+        </is>
+      </c>
+      <c r="M163" s="9" t="inlineStr">
+        <is>
+          <t>Filtering with std::ranges; turning conditions into readable text.</t>
+        </is>
+      </c>
+      <c r="N163" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O163" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="124.15" customHeight="1" s="20">
+      <c r="A164" s="7" t="inlineStr">
+        <is>
+          <t>US-268</t>
+        </is>
+      </c>
+      <c r="B164" s="9" t="inlineStr">
+        <is>
+          <t>E26</t>
+        </is>
+      </c>
+      <c r="C164" s="9" t="inlineStr">
+        <is>
+          <t>Editor NPC panel</t>
+        </is>
+      </c>
+      <c r="D164" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to select a placed NPC in the Editor and set its name, classes, attitude, family, dialogues by partner type and actions, so that I set every NPC by hand.</t>
+        </is>
+      </c>
+      <c r="E164" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Edit
+Given a placed wanderer selected
+When the owner gives it the classes trader and elder, the attitude friendly and its own player dialogue, and saves
+Then the level holds only those differences and F1 plays with them
+Scenario: Actions
+Given the actions list of a placed NPC
+When the owner unticks Give gift and plays
+Then that NPC's menu does not offer Give gift
+Scenario: Undo
+Given five panel changes
+When the owner presses Ctrl+Z five times
+Then the NPC is as it was</t>
+        </is>
+      </c>
+      <c r="F164" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G164" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H164" s="9">
+        <f>VLOOKUP(G164,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I164" s="9">
+        <f>VLOOKUP(G164,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J164" s="9" t="inlineStr">
+        <is>
+          <t>M9a</t>
+        </is>
+      </c>
+      <c r="K164" s="9" t="inlineStr">
+        <is>
+          <t>US-267, US-125</t>
+        </is>
+      </c>
+      <c r="L164" s="9" t="inlineStr">
+        <is>
+          <t>EDT-08, SDC-08</t>
+        </is>
+      </c>
+      <c r="M164" s="9" t="inlineStr">
+        <is>
+          <t>Forms bound to data; saving only the differences.</t>
+        </is>
+      </c>
+      <c r="N164" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O164" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="124.15" customHeight="1" s="20">
+      <c r="A165" s="7" t="inlineStr">
+        <is>
+          <t>US-269</t>
+        </is>
+      </c>
+      <c r="B165" s="9" t="inlineStr">
+        <is>
+          <t>E26</t>
+        </is>
+      </c>
+      <c r="C165" s="9" t="inlineStr">
+        <is>
+          <t>Editor kinds tab and map markers</t>
+        </is>
+      </c>
+      <c r="D165" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want a tab for each NPC kind's defaults and a colour ring with an icon under each placed NPC, so that I can change a whole kind at once and read a level at a glance.</t>
+        </is>
+      </c>
+      <c r="E165" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Kind
+Given the kinds tab
+When the owner sets goblin to neutral and saves
+Then every placed goblin without an override is neutral in play
+Scenario: Markers
+Given a level with a trader, a guard and a goblin
+When the owner opens it in the Editor
+Then each shows its ring and icon, and none shows in Game mode</t>
+        </is>
+      </c>
+      <c r="F165" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G165" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H165" s="9">
+        <f>VLOOKUP(G165,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I165" s="9">
+        <f>VLOOKUP(G165,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J165" s="9" t="inlineStr">
+        <is>
+          <t>M9a</t>
+        </is>
+      </c>
+      <c r="K165" s="9" t="inlineStr">
+        <is>
+          <t>US-268</t>
+        </is>
+      </c>
+      <c r="L165" s="9" t="inlineStr">
+        <is>
+          <t>EDT-08</t>
+        </is>
+      </c>
+      <c r="M165" s="9" t="inlineStr">
+        <is>
+          <t>Reusing a widget for two data sources; stable JSON field order.</t>
+        </is>
+      </c>
+      <c r="N165" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O165" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="124.15" customHeight="1" s="20">
+      <c r="A166" s="7" t="inlineStr">
+        <is>
+          <t>US-270</t>
+        </is>
+      </c>
+      <c r="B166" s="9" t="inlineStr">
+        <is>
+          <t>E26</t>
+        </is>
+      </c>
+      <c r="C166" s="9" t="inlineStr">
+        <is>
+          <t>NPC test level</t>
+        </is>
+      </c>
+      <c r="D166" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want a test level with seven NPCs that shows every M9a feature, so that I can try it all in one walk.</t>
+        </is>
+      </c>
+      <c r="E166" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Walk-through
+Given `odysseus.exe --level assets/levels/npc-test.json`
+When the owner follows the checklist
+Then every NPC offers exactly the actions its classes and overrides allow, the Actions pop-up explains the rest, confront changes opinions, the goblin attacks
+Scenario: Loads clean
+Given the test level
+When the game loads it
+Then the log has no class, kind, interaction or dialogue error</t>
+        </is>
+      </c>
+      <c r="F166" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G166" s="9" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H166" s="9">
+        <f>VLOOKUP(G166,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I166" s="9">
+        <f>VLOOKUP(G166,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J166" s="9" t="inlineStr">
+        <is>
+          <t>M9a</t>
+        </is>
+      </c>
+      <c r="K166" s="9" t="inlineStr">
+        <is>
+          <t>US-269</t>
+        </is>
+      </c>
+      <c r="L166" s="9" t="inlineStr">
+        <is>
+          <t>SDC-08..SDC-11, INT-09</t>
+        </is>
+      </c>
+      <c r="M166" s="9" t="inlineStr">
+        <is>
+          <t>Smoke tests that load every shipped file.</t>
+        </is>
+      </c>
+      <c r="N166" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O166" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="124.15" customHeight="1" s="20">
+      <c r="A167" s="7" t="inlineStr">
+        <is>
+          <t>US-280</t>
+        </is>
+      </c>
+      <c r="B167" s="9" t="inlineStr">
+        <is>
+          <t>E27</t>
+        </is>
+      </c>
+      <c r="C167" s="9" t="inlineStr">
+        <is>
+          <t>Currencies per region</t>
+        </is>
+      </c>
+      <c r="D167" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to choose in the Editor which items are currency in a region, so that trade can use money where I want it.</t>
+        </is>
+      </c>
+      <c r="E167" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Set
+Given the test level's settings
+When the owner marks shells as currency with value 1 and saves
+Then trades in that level accept shells
+Scenario: None
+Given a level with no currency
+When the player trades
+Then only barter is offered</t>
+        </is>
+      </c>
+      <c r="F167" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G167" s="9" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H167" s="9">
+        <f>VLOOKUP(G167,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I167" s="9">
+        <f>VLOOKUP(G167,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J167" s="9" t="inlineStr">
+        <is>
+          <t>M9b</t>
+        </is>
+      </c>
+      <c r="K167" s="9" t="inlineStr">
+        <is>
+          <t>US-270</t>
+        </is>
+      </c>
+      <c r="L167" s="9" t="inlineStr">
+        <is>
+          <t>INT-11, EDT-08</t>
+        </is>
+      </c>
+      <c r="M167" s="9" t="inlineStr">
+        <is>
+          <t>Value types; why money is an integer.</t>
+        </is>
+      </c>
+      <c r="N167" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O167" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="124.15" customHeight="1" s="20">
+      <c r="A168" s="7" t="inlineStr">
+        <is>
+          <t>US-281</t>
+        </is>
+      </c>
+      <c r="B168" s="9" t="inlineStr">
+        <is>
+          <t>E27</t>
+        </is>
+      </c>
+      <c r="C168" s="9" t="inlineStr">
+        <is>
+          <t>Trader stock</t>
+        </is>
+      </c>
+      <c r="D168" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want traders to have limited goods that come back each day and to pay more for what they want, so that trade is a choice.</t>
+        </is>
+      </c>
+      <c r="E168" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Restock
+Given a trader with 0 flint and a restock of 2 per day
+When a day passes
+Then it has 2 flint
+Scenario: Wants
+Given a trader who wants berries
+When the hero sells berries and then furs
+Then berries count at full value and furs at half
+Scenario: Saved
+Given stock after a trade
+When save and load
+Then the stock is the same</t>
+        </is>
+      </c>
+      <c r="F168" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G168" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H168" s="9">
+        <f>VLOOKUP(G168,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I168" s="9">
+        <f>VLOOKUP(G168,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J168" s="9" t="inlineStr">
+        <is>
+          <t>M9b</t>
+        </is>
+      </c>
+      <c r="K168" s="9" t="inlineStr">
+        <is>
+          <t>US-280</t>
+        </is>
+      </c>
+      <c r="L168" s="9" t="inlineStr">
+        <is>
+          <t>INT-11</t>
+        </is>
+      </c>
+      <c r="M168" s="9" t="inlineStr">
+        <is>
+          <t>Integer arithmetic and rounding rules written down.</t>
+        </is>
+      </c>
+      <c r="N168" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O168" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="124.15" customHeight="1" s="20">
+      <c r="A169" s="7" t="inlineStr">
+        <is>
+          <t>US-282</t>
+        </is>
+      </c>
+      <c r="B169" s="9" t="inlineStr">
+        <is>
+          <t>E27</t>
+        </is>
+      </c>
+      <c r="C169" s="9" t="inlineStr">
+        <is>
+          <t>Supply and demand, and reputation</t>
+        </is>
+      </c>
+      <c r="D169" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want prices to rise when goods are scarce and fall when they are plentiful, and better deals from people who like me, so that the economy feels real.</t>
+        </is>
+      </c>
+      <c r="E169" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Scarce
+Given flint scarce in the region
+When the hero asks its price twice a day apart while it gets scarcer
+Then the second price is higher
+Scenario: Reputation
+Given two traders with equal stock, one friendly and one suspicious
+When the hero asks the same item's price
+Then the friendly one is cheaper
+Scenario: Gate
+Given a trader whose rare goods need friendly
+When the wary hero opens trade
+Then the rare goods are not offered and the Actions pop-up says why</t>
+        </is>
+      </c>
+      <c r="F169" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G169" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H169" s="9">
+        <f>VLOOKUP(G169,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I169" s="9">
+        <f>VLOOKUP(G169,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J169" s="9" t="inlineStr">
+        <is>
+          <t>M9b</t>
+        </is>
+      </c>
+      <c r="K169" s="9" t="inlineStr">
+        <is>
+          <t>US-281, US-264</t>
+        </is>
+      </c>
+      <c r="L169" s="9" t="inlineStr">
+        <is>
+          <t>INT-12, SDC-10</t>
+        </is>
+      </c>
+      <c r="M169" s="9" t="inlineStr">
+        <is>
+          <t>Fixed-point formulas; clamping; tuning through data.</t>
+        </is>
+      </c>
+      <c r="N169" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O169" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="124.15" customHeight="1" s="20">
+      <c r="A170" s="7" t="inlineStr">
+        <is>
+          <t>US-283</t>
+        </is>
+      </c>
+      <c r="B170" s="9" t="inlineStr">
+        <is>
+          <t>E27</t>
+        </is>
+      </c>
+      <c r="C170" s="9" t="inlineStr">
+        <is>
+          <t>Trade screen for any trader</t>
+        </is>
+      </c>
+      <c r="D170" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want one trade screen for every trader, with barter and currency, so that I can trade with a passing NPC as with a rival camp.</t>
+        </is>
+      </c>
+      <c r="E170" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Trade
+Given a friendly trader with 6 flint and the hero with 10 berries
+When the player gives berries worth 2 flint
+Then the hero has 2 more flint and the trader 2 fewer, the berries moved
+Scenario: Currency
+Given a region with shells as currency
+When the player buys 1 fur for shells
+Then the shells move at the shown price
+Scenario: Rivals unchanged
+Given a rival camp
+When the player chooses Barter
+Then it works as before this story</t>
+        </is>
+      </c>
+      <c r="F170" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G170" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H170" s="9">
+        <f>VLOOKUP(G170,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I170" s="9">
+        <f>VLOOKUP(G170,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J170" s="9" t="inlineStr">
+        <is>
+          <t>M9b</t>
+        </is>
+      </c>
+      <c r="K170" s="9" t="inlineStr">
+        <is>
+          <t>US-282</t>
+        </is>
+      </c>
+      <c r="L170" s="9" t="inlineStr">
+        <is>
+          <t>INT-11</t>
+        </is>
+      </c>
+      <c r="M170" s="9" t="inlineStr">
+        <is>
+          <t>std::variant for 'one of several kinds'.</t>
+        </is>
+      </c>
+      <c r="N170" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O170" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="124.15" customHeight="1" s="20">
+      <c r="A171" s="7" t="inlineStr">
+        <is>
+          <t>US-284</t>
+        </is>
+      </c>
+      <c r="B171" s="9" t="inlineStr">
+        <is>
+          <t>E27</t>
+        </is>
+      </c>
+      <c r="C171" s="9" t="inlineStr">
+        <is>
+          <t>Editor trade panel</t>
+        </is>
+      </c>
+      <c r="D171" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to set a trader's stock, restock, wants and price settings in the Editor, so that each trader is my own.</t>
+        </is>
+      </c>
+      <c r="E171" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Edit
+Given the test level's trader selected
+When the owner adds 3 furs, a restock of 1 per day and the want berries, and saves
+Then play shows the furs and restocks one a day
+Scenario: Walk-through
+Given the extended checklist
+When the owner follows the trade steps
+Then each step behaves as written</t>
+        </is>
+      </c>
+      <c r="F171" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G171" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H171" s="9">
+        <f>VLOOKUP(G171,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I171" s="9">
+        <f>VLOOKUP(G171,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J171" s="9" t="inlineStr">
+        <is>
+          <t>M9b</t>
+        </is>
+      </c>
+      <c r="K171" s="9" t="inlineStr">
+        <is>
+          <t>US-283</t>
+        </is>
+      </c>
+      <c r="L171" s="9" t="inlineStr">
+        <is>
+          <t>EDT-08, INT-11</t>
+        </is>
+      </c>
+      <c r="M171" s="9" t="inlineStr">
+        <is>
+          <t>Table widgets bound to maps.</t>
+        </is>
+      </c>
+      <c r="N171" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O171" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="124.15" customHeight="1" s="20">
+      <c r="A172" s="7" t="inlineStr">
+        <is>
+          <t>US-290</t>
+        </is>
+      </c>
+      <c r="B172" s="9" t="inlineStr">
+        <is>
+          <t>E28</t>
+        </is>
+      </c>
+      <c r="C172" s="9" t="inlineStr">
+        <is>
+          <t>Day and night schedules</t>
+        </is>
+      </c>
+      <c r="D172" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want to give every NPC a daily schedule in the Editor, so that people work, eat, meet and sleep at their own hours.</t>
+        </is>
+      </c>
+      <c r="E172" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Follow
+Given an NPC scheduled to work at the market from 06:00 and sleep at home from 21:00
+When the day passes
+Then it is at the market at 10:00 and at home at 22:00
+Scenario: Interrupt
+Given the same NPC very hungry at 10:00
+When it eats
+Then it returns to the market afterwards</t>
+        </is>
+      </c>
+      <c r="F172" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G172" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H172" s="9">
+        <f>VLOOKUP(G172,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I172" s="9">
+        <f>VLOOKUP(G172,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J172" s="9" t="inlineStr">
+        <is>
+          <t>M9c</t>
+        </is>
+      </c>
+      <c r="K172" s="9" t="inlineStr">
+        <is>
+          <t>US-284</t>
+        </is>
+      </c>
+      <c r="L172" s="9" t="inlineStr">
+        <is>
+          <t>SDC-12, SDC-07, EDT-08</t>
+        </is>
+      </c>
+      <c r="M172" s="9" t="inlineStr">
+        <is>
+          <t>Time-based state machines; interruptions and resumption.</t>
+        </is>
+      </c>
+      <c r="N172" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O172" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" ht="124.15" customHeight="1" s="20">
+      <c r="A173" s="7" t="inlineStr">
+        <is>
+          <t>US-291</t>
+        </is>
+      </c>
+      <c r="B173" s="9" t="inlineStr">
+        <is>
+          <t>E28</t>
+        </is>
+      </c>
+      <c r="C173" s="9" t="inlineStr">
+        <is>
+          <t>Action sources</t>
+        </is>
+      </c>
+      <c r="D173" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want NPCs to act from their classes, from my custom actions and from world events, and later from quests, all set in the Editor, so that I control what people do.</t>
+        </is>
+      </c>
+      <c r="E173" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Class
+Given an NPC of class guard whose class action is patrol
+When it is idle on duty
+Then it patrols
+Scenario: Event
+Given an event action 'help put out fire' for class villager
+When a fire starts within 12 m of a villager
+Then the villager goes to help
+Scenario: Hook
+Given the quest-action source
+When the game runs
+Then it offers nothing and costs nothing until M10</t>
+        </is>
+      </c>
+      <c r="F173" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G173" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H173" s="9">
+        <f>VLOOKUP(G173,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I173" s="9">
+        <f>VLOOKUP(G173,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J173" s="9" t="inlineStr">
+        <is>
+          <t>M9c</t>
+        </is>
+      </c>
+      <c r="K173" s="9" t="inlineStr">
+        <is>
+          <t>US-290</t>
+        </is>
+      </c>
+      <c r="L173" s="9" t="inlineStr">
+        <is>
+          <t>SDC-12, EDT-08</t>
+        </is>
+      </c>
+      <c r="M173" s="9" t="inlineStr">
+        <is>
+          <t>Strategy objects as sources; extension points.</t>
+        </is>
+      </c>
+      <c r="N173" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O173" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="124.15" customHeight="1" s="20">
+      <c r="A174" s="7" t="inlineStr">
+        <is>
+          <t>US-292</t>
+        </is>
+      </c>
+      <c r="B174" s="9" t="inlineStr">
+        <is>
+          <t>E28</t>
+        </is>
+      </c>
+      <c r="C174" s="9" t="inlineStr">
+        <is>
+          <t>NPCs act on each other</t>
+        </is>
+      </c>
+      <c r="D174" s="9" t="inlineStr">
+        <is>
+          <t>As the player, I want NPCs to talk, fight, trade, give gifts and confront each other with the same rules as me, so that the world lives without me.</t>
+        </is>
+      </c>
+      <c r="E174" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Trade
+Given two traders near each other where one wants what the other has
+When they are idle
+Then they trade and both stocks change
+Scenario: Fight
+Given two NPCs who are hostile to each other
+When they meet
+Then they fight and the bystanders' opinions change
+Scenario: Budget
+Given the 100,000-person load test
+When a day is simulated
+Then it still meets ADR-022</t>
+        </is>
+      </c>
+      <c r="F174" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G174" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H174" s="9">
+        <f>VLOOKUP(G174,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I174" s="9">
+        <f>VLOOKUP(G174,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J174" s="9" t="inlineStr">
+        <is>
+          <t>M9c</t>
+        </is>
+      </c>
+      <c r="K174" s="9" t="inlineStr">
+        <is>
+          <t>US-291</t>
+        </is>
+      </c>
+      <c r="L174" s="9" t="inlineStr">
+        <is>
+          <t>INT-10</t>
+        </is>
+      </c>
+      <c r="M174" s="9" t="inlineStr">
+        <is>
+          <t>Symmetric actor and target; budgets per tick.</t>
+        </is>
+      </c>
+      <c r="N174" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O174" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="124.15" customHeight="1" s="20">
+      <c r="A175" s="7" t="inlineStr">
+        <is>
+          <t>US-293</t>
+        </is>
+      </c>
+      <c r="B175" s="9" t="inlineStr">
+        <is>
+          <t>E28</t>
+        </is>
+      </c>
+      <c r="C175" s="9" t="inlineStr">
+        <is>
+          <t>Default interactions by partner type</t>
+        </is>
+      </c>
+      <c r="D175" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want each class and NPC to have default dialogues and actions for meeting the player, other classes, animals and the environment, with a list I can extend, so that every meeting has a sensible reaction.</t>
+        </is>
+      </c>
+      <c r="E175" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Animals
+Given a hunter class whose Animals default is hunt
+When a deer is near an idle hunter
+Then the hunter hunts it
+Scenario: Extend
+Given a new partner type 'buildings' added to the data file
+When the Editor opens
+Then the NPC panel offers defaults for buildings</t>
+        </is>
+      </c>
+      <c r="F175" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G175" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H175" s="9">
+        <f>VLOOKUP(G175,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I175" s="9">
+        <f>VLOOKUP(G175,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J175" s="9" t="inlineStr">
+        <is>
+          <t>M9c</t>
+        </is>
+      </c>
+      <c r="K175" s="9" t="inlineStr">
+        <is>
+          <t>US-292</t>
+        </is>
+      </c>
+      <c r="L175" s="9" t="inlineStr">
+        <is>
+          <t>INT-10</t>
+        </is>
+      </c>
+      <c r="M175" s="9" t="inlineStr">
+        <is>
+          <t>Data-driven enumerations.</t>
+        </is>
+      </c>
+      <c r="N175" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O175" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="124.15" customHeight="1" s="20">
+      <c r="A176" s="7" t="inlineStr">
+        <is>
+          <t>US-294</t>
+        </is>
+      </c>
+      <c r="B176" s="9" t="inlineStr">
+        <is>
+          <t>E28</t>
+        </is>
+      </c>
+      <c r="C176" s="9" t="inlineStr">
+        <is>
+          <t>Living test level</t>
+        </is>
+      </c>
+      <c r="D176" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want the test level to show a day of NPC life, and the 100,000-person soak to pass, so that I can judge M9c in one sitting.</t>
+        </is>
+      </c>
+      <c r="E176" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Day
+Given the test level
+When the owner watches one in-game day
+Then every NPC follows its schedule and at least one NPC-to-NPC trade and one conversation happen
+Scenario: Soak
+Given 100,000 persons
+When 10 in-game days run headless
+Then the budget of ADR-022 holds and the determinism hash is stable</t>
+        </is>
+      </c>
+      <c r="F176" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G176" s="9" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H176" s="9">
+        <f>VLOOKUP(G176,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I176" s="9">
+        <f>VLOOKUP(G176,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J176" s="9" t="inlineStr">
+        <is>
+          <t>M9c</t>
+        </is>
+      </c>
+      <c r="K176" s="9" t="inlineStr">
+        <is>
+          <t>US-293</t>
+        </is>
+      </c>
+      <c r="L176" s="9" t="inlineStr">
+        <is>
+          <t>SDC-12, INT-10, NFR-08</t>
+        </is>
+      </c>
+      <c r="M176" s="9" t="inlineStr">
+        <is>
+          <t>Soak tests and what they catch.</t>
+        </is>
+      </c>
+      <c r="N176" s="9" t="inlineStr">
+        <is>
+          <t>NPC foundation, trade and life (owner, 2026-10-04, D-52)</t>
+        </is>
+      </c>
+      <c r="O176" s="16" t="inlineStr">
         <is>
           <t>To do</t>
         </is>

</xml_diff>

<commit_message>
US-182: getting and handing in quests
</commit_message>
<xml_diff>
--- a/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
+++ b/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
@@ -654,10 +654,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Working tracker for developers. The source of truth is Project Odyssey.docx v2.10, chapter 12; this workbook is generated from the same data. Updated 2026-10-01: merged the M8b assembly edits (D-44) with D-47 and D-48.</t>
-        </is>
-      </c>
-    </row>
+          <t>Working tracker for developers. The source of truth is Project Odyssey.docx v2.11, chapter 12; this workbook is generated from the same data. Updated 2026-10-01: merged the M8b assembly edits (D-44) with D-47 and D-48.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="15.75" customHeight="1" s="20">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -700,6 +701,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="15.75" customHeight="1" s="20">
       <c r="A11" s="5" t="inlineStr">
         <is>
@@ -818,7 +820,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15.75" customHeight="1" s="20">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -833,7 +834,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="15.75" customHeight="1" s="20">
       <c r="A7" s="5" t="inlineStr">
         <is>
@@ -1784,7 +1784,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -1795,7 +1794,6 @@
         <v>46300</v>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="38.25" customHeight="1" s="20">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -14222,7 +14220,7 @@
       </c>
       <c r="O89" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -14308,7 +14306,7 @@
       </c>
       <c r="O90" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -14394,7 +14392,7 @@
       </c>
       <c r="O91" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -14480,7 +14478,7 @@
       </c>
       <c r="O92" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -14566,7 +14564,7 @@
       </c>
       <c r="O93" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -14652,7 +14650,7 @@
       </c>
       <c r="O94" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -14738,7 +14736,7 @@
       </c>
       <c r="O95" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -14824,7 +14822,7 @@
       </c>
       <c r="O96" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -14910,7 +14908,7 @@
       </c>
       <c r="O97" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -14996,7 +14994,7 @@
       </c>
       <c r="O98" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -15082,7 +15080,7 @@
       </c>
       <c r="O99" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18178,7 +18176,7 @@
       </c>
       <c r="O135" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18268,7 +18266,7 @@
       </c>
       <c r="O136" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18354,7 +18352,7 @@
       </c>
       <c r="O137" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18440,7 +18438,7 @@
       </c>
       <c r="O138" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18526,7 +18524,7 @@
       </c>
       <c r="O139" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18612,7 +18610,7 @@
       </c>
       <c r="O140" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18698,7 +18696,7 @@
       </c>
       <c r="O141" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18784,7 +18782,7 @@
       </c>
       <c r="O142" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18870,7 +18868,7 @@
       </c>
       <c r="O143" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -18956,7 +18954,7 @@
       </c>
       <c r="O144" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19042,7 +19040,7 @@
       </c>
       <c r="O145" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19128,7 +19126,7 @@
       </c>
       <c r="O146" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19214,7 +19212,7 @@
       </c>
       <c r="O147" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19300,7 +19298,7 @@
       </c>
       <c r="O148" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19386,7 +19384,7 @@
       </c>
       <c r="O149" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19472,7 +19470,7 @@
       </c>
       <c r="O150" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19558,7 +19556,7 @@
       </c>
       <c r="O151" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19644,7 +19642,7 @@
       </c>
       <c r="O152" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19730,7 +19728,7 @@
       </c>
       <c r="O153" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19816,7 +19814,7 @@
       </c>
       <c r="O154" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19902,7 +19900,7 @@
       </c>
       <c r="O155" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -19988,7 +19986,7 @@
       </c>
       <c r="O156" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20074,7 +20072,7 @@
       </c>
       <c r="O157" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20160,7 +20158,7 @@
       </c>
       <c r="O158" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20246,7 +20244,7 @@
       </c>
       <c r="O159" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20332,7 +20330,7 @@
       </c>
       <c r="O160" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20418,7 +20416,7 @@
       </c>
       <c r="O161" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20504,7 +20502,7 @@
       </c>
       <c r="O162" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20586,7 +20584,7 @@
       </c>
       <c r="O163" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20672,7 +20670,7 @@
       </c>
       <c r="O164" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20754,7 +20752,7 @@
       </c>
       <c r="O165" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20836,7 +20834,7 @@
       </c>
       <c r="O166" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -20918,7 +20916,7 @@
       </c>
       <c r="O167" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -21004,7 +21002,7 @@
       </c>
       <c r="O168" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -21090,7 +21088,7 @@
       </c>
       <c r="O169" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -21176,7 +21174,7 @@
       </c>
       <c r="O170" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -21258,7 +21256,7 @@
       </c>
       <c r="O171" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -21340,7 +21338,7 @@
       </c>
       <c r="O172" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -21426,7 +21424,7 @@
       </c>
       <c r="O173" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -21512,7 +21510,7 @@
       </c>
       <c r="O174" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -21594,7 +21592,7 @@
       </c>
       <c r="O175" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -21676,7 +21674,7 @@
       </c>
       <c r="O176" s="16" t="inlineStr">
         <is>
-          <t>To do</t>
+          <t>Done</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Codex v2.13: sync from Anima (M10b Editor help and live data, D-58; adopts v2.12, CI-013)
Brief docs/plans/M10b-editor-help-live-data-brief.md, decision D-58 (owner, 11 answers),
requirements v2.11 and backlog (epic E29, US-300..US-305, EDT-09..11, NFR-09, MVP-18)
mirrored from Drive. New milestone M10b after X-M10; P-013 adopts.
</commit_message>
<xml_diff>
--- a/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
+++ b/docs/project/requirements/Project Odyssey - MVP Backlog.xlsx
@@ -818,7 +818,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15.75" customHeight="1" s="20">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -833,7 +832,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="15.75" customHeight="1" s="20">
       <c r="A7" s="5" t="inlineStr">
         <is>
@@ -1784,7 +1782,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -1795,7 +1792,6 @@
         <v>46300</v>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="38.25" customHeight="1" s="20">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -4435,7 +4431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -5640,6 +5636,43 @@
         </is>
       </c>
       <c r="G35" s="16" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" s="20">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>D-58</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Editor help and live data: 11 answers (docs/decision-requests/D-58.md); new milestone M10b after X-M10</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Design decision</t>
+        </is>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>M10b</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>US-300..US-305</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G36" s="16" t="inlineStr">
         <is>
           <t>Decided</t>
         </is>
@@ -5675,7 +5708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="20" min="1" max="1"/>
@@ -7089,37 +7122,83 @@
         <v/>
       </c>
     </row>
-    <row r="34" s="20">
-      <c r="A34" s="7" t="n"/>
-      <c r="B34" s="7" t="inlineStr">
+    <row r="34" ht="25.5" customHeight="1" s="20">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>E29</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Editor help and live data</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Every Editor field explains itself and suggests its values; whatever the owner saves shows in the running game at once, and level edits win over an older run save.</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>M10b</t>
+        </is>
+      </c>
+      <c r="E34" s="9">
+        <f>COUNTIF('User Stories'!$B$5:$B$200,A34)</f>
+        <v/>
+      </c>
+      <c r="F34" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A34,'User Stories'!$F$5:$F$200,"Must")</f>
+        <v/>
+      </c>
+      <c r="G34" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A34,'User Stories'!$H$5:$H$200)</f>
+        <v/>
+      </c>
+      <c r="H34" s="9">
+        <f>SUMIF('User Stories'!$B$5:$B$200,A34,'User Stories'!$I$5:$I$200)</f>
+        <v/>
+      </c>
+      <c r="I34" s="9">
+        <f>COUNTIFS('User Stories'!$B$5:$B$200,A34,'User Stories'!$O$5:$O$200,"Done")</f>
+        <v/>
+      </c>
+      <c r="J34" s="17">
+        <f>IFERROR(I34/E34,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="n"/>
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C34" s="7" t="n"/>
-      <c r="D34" s="7" t="n"/>
-      <c r="E34" s="7">
-        <f>SUM(E5:E33)</f>
-        <v/>
-      </c>
-      <c r="F34" s="7">
-        <f>SUM(F5:F33)</f>
-        <v/>
-      </c>
-      <c r="G34" s="7">
-        <f>SUM(G5:G33)</f>
-        <v/>
-      </c>
-      <c r="H34" s="7">
-        <f>SUM(H5:H33)</f>
-        <v/>
-      </c>
-      <c r="I34" s="7">
-        <f>SUM(I5:I33)</f>
-        <v/>
-      </c>
-      <c r="J34" s="18">
-        <f>IFERROR(I34/E34,0)</f>
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="7" t="n"/>
+      <c r="E35" s="7">
+        <f>SUM(E5:E34)</f>
+        <v/>
+      </c>
+      <c r="F35" s="7">
+        <f>SUM(F5:F34)</f>
+        <v/>
+      </c>
+      <c r="G35" s="7">
+        <f>SUM(G5:G34)</f>
+        <v/>
+      </c>
+      <c r="H35" s="7">
+        <f>SUM(H5:H34)</f>
+        <v/>
+      </c>
+      <c r="I35" s="7">
+        <f>SUM(I5:I34)</f>
+        <v/>
+      </c>
+      <c r="J35" s="18">
+        <f>IFERROR(I35/E35,0)</f>
         <v/>
       </c>
     </row>
@@ -7134,7 +7213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O176"/>
+  <dimension ref="A1:O182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" style="20" min="1" max="1"/>
@@ -21675,6 +21754,534 @@
         </is>
       </c>
       <c r="O176" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="124.15" customHeight="1" s="20">
+      <c r="A177" s="7" t="inlineStr">
+        <is>
+          <t>US-300</t>
+        </is>
+      </c>
+      <c r="B177" s="9" t="inlineStr">
+        <is>
+          <t>E29</t>
+        </is>
+      </c>
+      <c r="C177" s="9" t="inlineStr">
+        <is>
+          <t>Field tooltips from help.json</t>
+        </is>
+      </c>
+      <c r="D177" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want every Editor field to say what it does, its range and an example, so that I never need the guide to fill a form.</t>
+        </is>
+      </c>
+      <c r="E177" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Hover
+Given the NPC panel
+When the pointer rests on Sword
+Then a tooltip shows purpose, range and example from help.json
+Scenario: Coverage
+Given all panels of the Level, Building and Graph editors
+When the coverage test builds them
+Then every field has a help entry; a missing one fails the test by name
+Scenario: Broken file
+Given a help.json with a syntax error
+When the Editor opens
+Then fields show no tooltip, the status line names the line, nothing crashes</t>
+        </is>
+      </c>
+      <c r="F177" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G177" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H177" s="9">
+        <f>VLOOKUP(G177,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I177" s="9">
+        <f>VLOOKUP(G177,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J177" s="9" t="inlineStr">
+        <is>
+          <t>M10b</t>
+        </is>
+      </c>
+      <c r="K177" s="9" t="inlineStr">
+        <is>
+          <t>US-123, US-173</t>
+        </is>
+      </c>
+      <c r="L177" s="9" t="inlineStr">
+        <is>
+          <t>EDT-09</t>
+        </is>
+      </c>
+      <c r="M177" s="9" t="inlineStr">
+        <is>
+          <t>Loading text data once and looking it up by key; tests that walk every widget.</t>
+        </is>
+      </c>
+      <c r="N177" s="9" t="inlineStr">
+        <is>
+          <t>Editor help and live data (owner, 2026-10-05, D-58)</t>
+        </is>
+      </c>
+      <c r="O177" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="124.15" customHeight="1" s="20">
+      <c r="A178" s="7" t="inlineStr">
+        <is>
+          <t>US-301</t>
+        </is>
+      </c>
+      <c r="B178" s="9" t="inlineStr">
+        <is>
+          <t>E29</t>
+        </is>
+      </c>
+      <c r="C178" s="9" t="inlineStr">
+        <is>
+          <t>Suggestion list widget</t>
+        </is>
+      </c>
+      <c r="D178" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want a list of matching values under the field I type in, so that I pick instead of remembering names.</t>
+        </is>
+      </c>
+      <c r="E178" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Filter
+Given a field suggesting trader, trapper, elder
+When I type 'tr'
+Then the list shows trader and trapper
+Scenario: Keys
+Given the list open
+When I press Down then Tab
+Then the second row is the field's text; Esc closes and keeps what I typed
+Scenario: Quiet
+Given the list closed
+When I press Tab, Enter or the arrows
+Then they do what they did before M10b</t>
+        </is>
+      </c>
+      <c r="F178" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G178" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H178" s="9">
+        <f>VLOOKUP(G178,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I178" s="9">
+        <f>VLOOKUP(G178,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J178" s="9" t="inlineStr">
+        <is>
+          <t>M10b</t>
+        </is>
+      </c>
+      <c r="K178" s="9" t="inlineStr">
+        <is>
+          <t>US-300</t>
+        </is>
+      </c>
+      <c r="L178" s="9" t="inlineStr">
+        <is>
+          <t>EDT-10</t>
+        </is>
+      </c>
+      <c r="M178" s="9" t="inlineStr">
+        <is>
+          <t>A reusable overlay widget; keyboard focus and who gets a key.</t>
+        </is>
+      </c>
+      <c r="N178" s="9" t="inlineStr">
+        <is>
+          <t>Editor help and live data (owner, 2026-10-05, D-58)</t>
+        </is>
+      </c>
+      <c r="O178" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="124.15" customHeight="1" s="20">
+      <c r="A179" s="7" t="inlineStr">
+        <is>
+          <t>US-302</t>
+        </is>
+      </c>
+      <c r="B179" s="9" t="inlineStr">
+        <is>
+          <t>E29</t>
+        </is>
+      </c>
+      <c r="C179" s="9" t="inlineStr">
+        <is>
+          <t>Suggestions on every field</t>
+        </is>
+      </c>
+      <c r="D179" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want every field to suggest the values it accepts, so that I never type an id that does not exist.</t>
+        </is>
+      </c>
+      <c r="E179" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Text
+Given the NPC Script field
+When I type 'el'
+Then the .dlg files starting with 'el' are listed
+Scenario: Lists
+Given the Classes field holding 'trader, '
+When I type 'e'
+Then the classes starting with 'e' are listed and accepting one keeps 'trader, '
+Scenario: Numbers
+Given the HP field of a wolf
+When it gets focus
+Then the list shows the kind default, the min, the max and the last 5 values typed there
+Scenario: Fresh
+Given a new NPC Class saved
+When I open the Classes field
+Then the new class is listed without a restart</t>
+        </is>
+      </c>
+      <c r="F179" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G179" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H179" s="9">
+        <f>VLOOKUP(G179,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I179" s="9">
+        <f>VLOOKUP(G179,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J179" s="9" t="inlineStr">
+        <is>
+          <t>M10b</t>
+        </is>
+      </c>
+      <c r="K179" s="9" t="inlineStr">
+        <is>
+          <t>US-301, US-260, US-170</t>
+        </is>
+      </c>
+      <c r="L179" s="9" t="inlineStr">
+        <is>
+          <t>EDT-10</t>
+        </is>
+      </c>
+      <c r="M179" s="9" t="inlineStr">
+        <is>
+          <t>Strategy functions as data sources; completing one item of a comma list.</t>
+        </is>
+      </c>
+      <c r="N179" s="9" t="inlineStr">
+        <is>
+          <t>Editor help and live data (owner, 2026-10-05, D-58)</t>
+        </is>
+      </c>
+      <c r="O179" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="124.15" customHeight="1" s="20">
+      <c r="A180" s="7" t="inlineStr">
+        <is>
+          <t>US-303</t>
+        </is>
+      </c>
+      <c r="B180" s="9" t="inlineStr">
+        <is>
+          <t>E29</t>
+        </is>
+      </c>
+      <c r="C180" s="9" t="inlineStr">
+        <is>
+          <t>Live reload of every data file</t>
+        </is>
+      </c>
+      <c r="D180" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want everything I save to show in the running game at once, so that I test changes without a restart.</t>
+        </is>
+      </c>
+      <c r="E180" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Catalog
+Given a running game
+When I change a light kind's colour in lights.json and save
+Then placed lights of that kind shine in the new colour within 1 s
+Scenario: Object
+Given objects.json
+When I add an object and save
+Then it is on the object page of the palette without a restart
+Scenario: All or nothing
+Given a broken interaction file saved
+When the reload runs
+Then the last good data stays and the mistakes panel names file and line
+Scenario: Missing kind
+Given a placed thing whose kind I deleted
+When the data reloads
+Then it shows a red marker and a warning naming the level entry; the game runs on</t>
+        </is>
+      </c>
+      <c r="F180" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G180" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H180" s="9">
+        <f>VLOOKUP(G180,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I180" s="9">
+        <f>VLOOKUP(G180,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J180" s="9" t="inlineStr">
+        <is>
+          <t>M10b</t>
+        </is>
+      </c>
+      <c r="K180" s="9" t="inlineStr">
+        <is>
+          <t>US-156, US-260</t>
+        </is>
+      </c>
+      <c r="L180" s="9" t="inlineStr">
+        <is>
+          <t>EDT-11, NFR-09</t>
+        </is>
+      </c>
+      <c r="M180" s="9" t="inlineStr">
+        <is>
+          <t>A registry of reloadable data sets; swapping data only when the new copy is clean.</t>
+        </is>
+      </c>
+      <c r="N180" s="9" t="inlineStr">
+        <is>
+          <t>Editor help and live data (owner, 2026-10-05, D-58)</t>
+        </is>
+      </c>
+      <c r="O180" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="124.15" customHeight="1" s="20">
+      <c r="A181" s="7" t="inlineStr">
+        <is>
+          <t>US-304</t>
+        </is>
+      </c>
+      <c r="B181" s="9" t="inlineStr">
+        <is>
+          <t>E29</t>
+        </is>
+      </c>
+      <c r="C181" s="9" t="inlineStr">
+        <is>
+          <t>File watch for outside edits</t>
+        </is>
+      </c>
+      <c r="D181" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want files I edit in a text editor to reload by themselves, so that I can work outside the Editor too.</t>
+        </is>
+      </c>
+      <c r="E181" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Outside
+Given the game running
+When I save an interaction file in a text editor
+Then the change is live within 1 s without F5
+Scenario: Own writes
+Given the Editor saves a file
+When the watcher sees it
+Then it is not reloaded a second time
+Scenario: Open level
+Given the Editor open with unsaved changes
+When the level file changes on disk
+Then nothing is overwritten and the status line says the file changed</t>
+        </is>
+      </c>
+      <c r="F181" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G181" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H181" s="9">
+        <f>VLOOKUP(G181,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I181" s="9">
+        <f>VLOOKUP(G181,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J181" s="9" t="inlineStr">
+        <is>
+          <t>M10b</t>
+        </is>
+      </c>
+      <c r="K181" s="9" t="inlineStr">
+        <is>
+          <t>US-303</t>
+        </is>
+      </c>
+      <c r="L181" s="9" t="inlineStr">
+        <is>
+          <t>EDT-11, NFR-09</t>
+        </is>
+      </c>
+      <c r="M181" s="9" t="inlineStr">
+        <is>
+          <t>Polling file times; debouncing; ignoring your own writes.</t>
+        </is>
+      </c>
+      <c r="N181" s="9" t="inlineStr">
+        <is>
+          <t>Editor help and live data (owner, 2026-10-05, D-58)</t>
+        </is>
+      </c>
+      <c r="O181" s="16" t="inlineStr">
+        <is>
+          <t>To do</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="124.15" customHeight="1" s="20">
+      <c r="A182" s="7" t="inlineStr">
+        <is>
+          <t>US-305</t>
+        </is>
+      </c>
+      <c r="B182" s="9" t="inlineStr">
+        <is>
+          <t>E29</t>
+        </is>
+      </c>
+      <c r="C182" s="9" t="inlineStr">
+        <is>
+          <t>Level edits win over the run save</t>
+        </is>
+      </c>
+      <c r="D182" s="9" t="inlineStr">
+        <is>
+          <t>As the owner, I want my level edits to win over an older run save, so that what I saved is what I play.</t>
+        </is>
+      </c>
+      <c r="E182" s="9" t="inlineStr">
+        <is>
+          <t>Scenario: Edited
+Given a run saved
+When I move a berry bush in the Editor and save
+Then the next start (and F1) shows it in its new place, fresh
+Scenario: Untouched
+Given the same run
+When I start again
+Then berries I picked on another bush still ripen; the clan and hero are as saved
+Scenario: Removed
+Given an NPC deleted from the level
+When the run loads
+Then it is not in the run and the status line counts the update
+Scenario: Old save
+Given a save from before M10b
+When it loads
+Then it behaves as before once and is written with a baseline</t>
+        </is>
+      </c>
+      <c r="F182" s="9" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="G182" s="9" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H182" s="9">
+        <f>VLOOKUP(G182,'Read Me'!$A$13:$C$15,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="I182" s="9">
+        <f>VLOOKUP(G182,'Read Me'!$A$13:$C$15,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="J182" s="9" t="inlineStr">
+        <is>
+          <t>M10b</t>
+        </is>
+      </c>
+      <c r="K182" s="9" t="inlineStr">
+        <is>
+          <t>US-303, US-153</t>
+        </is>
+      </c>
+      <c r="L182" s="9" t="inlineStr">
+        <is>
+          <t>EDT-11, ADR-010</t>
+        </is>
+      </c>
+      <c r="M182" s="9" t="inlineStr">
+        <is>
+          <t>Content hashes as a baseline; merging by id; save versions and migrations.</t>
+        </is>
+      </c>
+      <c r="N182" s="9" t="inlineStr">
+        <is>
+          <t>Editor help and live data (owner, 2026-10-05, D-58)</t>
+        </is>
+      </c>
+      <c r="O182" s="16" t="inlineStr">
         <is>
           <t>To do</t>
         </is>

</xml_diff>